<commit_message>
Add easy Excel calendar input panel
</commit_message>
<xml_diff>
--- a/app/template/캘린더(자동).xlsx
+++ b/app/template/캘린더(자동).xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="Ra8fa69654b904b79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26.8" sheetId="1" r:id="R5562feb40d6648fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="일정데이터" sheetId="3" r:id="R5de38ba42f9b4404"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="R2c594194fa964a28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26.8" sheetId="1" r:id="R85b6f1c98ace4766"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -158,7 +157,7 @@
     <x:numFmt numFmtId="201" formatCode="hh:mm"/>
     <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </x:numFmts>
-  <x:fonts count="16">
+  <x:fonts count="18">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -248,8 +247,19 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="맑은 고딕"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF667085"/>
+      <x:name val="맑은 고딕"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF667085"/>
+      <x:name val="맑은 고딕"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -286,6 +296,11 @@
         <x:fgColor rgb="FF315D8A"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F4F7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="18">
     <x:border/>
@@ -494,7 +509,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="43">
+  <x:cellXfs count="49">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -586,6 +601,24 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="17" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -639,14 +672,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CalendarEvents" displayName="CalendarEvents" ref="A4:H5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CalendarEvents" displayName="CalendarEvents" ref="J4:Q5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
-    <x:tableColumn id="1" name="ID"/>
-    <x:tableColumn id="2" name="날짜"/>
-    <x:tableColumn id="3" name="제목"/>
-    <x:tableColumn id="4" name="메모"/>
-    <x:tableColumn id="5" name="색상"/>
-    <x:tableColumn id="6" name="알림시각"/>
+    <x:tableColumn id="1" name="날짜"/>
+    <x:tableColumn id="2" name="제목"/>
+    <x:tableColumn id="3" name="메모"/>
+    <x:tableColumn id="4" name="색상"/>
+    <x:tableColumn id="5" name="알림시각"/>
+    <x:tableColumn id="6" name="ID"/>
     <x:tableColumn id="7" name="수정시간"/>
     <x:tableColumn id="8" name="삭제시간"/>
   </x:tableColumns>
@@ -3312,9 +3345,17 @@
   <x:cols>
     <x:col min="2" max="8" width="26.625" style="8" customWidth="1"/>
     <x:col min="9" max="9" width="54" style="8" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="34" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="13" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="13" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="34" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="23" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="23" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
+    <x:row r="1" ht="32" customHeight="1">
       <x:c r="G1" s="9">
         <x:v>2026</x:v>
       </x:c>
@@ -3324,8 +3365,18 @@
       <x:c r="I1" s="7" t="s">
         <x:v>35</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" ht="17.25" customHeight="1">
+      <x:c r="J1" s="25" t="str">
+        <x:v>Cellendar 간편 일정 입력</x:v>
+      </x:c>
+      <x:c r="K1" s="25"/>
+      <x:c r="L1" s="25"/>
+      <x:c r="M1" s="25"/>
+      <x:c r="N1" s="25"/>
+      <x:c r="O1" s="25"/>
+      <x:c r="P1" s="25"/>
+      <x:c r="Q1" s="25"/>
+    </x:row>
+    <x:row r="2" ht="26" customHeight="1">
       <x:c r="B2" s="4" t="s">
         <x:v>36</x:v>
       </x:c>
@@ -3350,6 +3401,16 @@
       <x:c r="I2" s="3" t="s">
         <x:v>43</x:v>
       </x:c>
+      <x:c r="J2" s="27" t="str">
+        <x:v>날짜·제목·메모를 입력하세요. ID·수정시간·삭제시간은 앱이 관리합니다.</x:v>
+      </x:c>
+      <x:c r="K2" s="27"/>
+      <x:c r="L2" s="27"/>
+      <x:c r="M2" s="27"/>
+      <x:c r="N2" s="27"/>
+      <x:c r="O2" s="27"/>
+      <x:c r="P2" s="27"/>
+      <x:c r="Q2" s="27"/>
     </x:row>
     <x:row r="3" ht="17.25" customHeight="1">
       <x:c r="B3" s="11" t="n">
@@ -3382,399 +3443,352 @@
       </x:c>
       <x:c r="I3" s="1"/>
     </x:row>
-    <x:row r="4" ht="80.0999984741211" customHeight="1">
-      <x:c r="B4" s="33" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=B3)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="C4" s="34" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=C3)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="D4" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=D3)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="E4" s="34" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=E3)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="F4" s="34" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=F3)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="G4" s="34" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=G3)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="H4" s="36" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=H3)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="B4" s="39" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=B3)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="C4" s="40" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=C3)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="D4" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=D3)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="E4" s="40" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=E3)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="F4" s="40" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=F3)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="G4" s="40" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=G3)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="H4" s="42" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=H3)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
       </x:c>
       <x:c r="I4" s="1"/>
+      <x:c r="J4" s="29" t="str">
+        <x:v>날짜</x:v>
+      </x:c>
+      <x:c r="K4" s="29" t="str">
+        <x:v>제목</x:v>
+      </x:c>
+      <x:c r="L4" s="29" t="str">
+        <x:v>메모</x:v>
+      </x:c>
+      <x:c r="M4" s="29" t="str">
+        <x:v>색상</x:v>
+      </x:c>
+      <x:c r="N4" s="29" t="str">
+        <x:v>알림시각</x:v>
+      </x:c>
+      <x:c r="O4" s="36" t="str">
+        <x:v>ID</x:v>
+      </x:c>
+      <x:c r="P4" s="36" t="str">
+        <x:v>수정시간</x:v>
+      </x:c>
+      <x:c r="Q4" s="36" t="str">
+        <x:v>삭제시간</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="17.25" customHeight="1">
-      <x:c r="B5" s="37" t="n">
+      <x:c r="B5" s="43" t="n">
         <x:f>H3+1</x:f>
         <x:v>46236</x:v>
       </x:c>
-      <x:c r="C5" s="38" t="n">
+      <x:c r="C5" s="44" t="n">
         <x:f t="shared" ref="C5:H5" si="1">B5+1</x:f>
         <x:v>46237</x:v>
       </x:c>
-      <x:c r="D5" s="38">
+      <x:c r="D5" s="44">
         <x:f t="shared" si="1"/>
         <x:v>46238</x:v>
       </x:c>
-      <x:c r="E5" s="38">
+      <x:c r="E5" s="44">
         <x:f t="shared" si="1"/>
         <x:v>46239</x:v>
       </x:c>
-      <x:c r="F5" s="38">
+      <x:c r="F5" s="44">
         <x:f t="shared" si="1"/>
         <x:v>46240</x:v>
       </x:c>
-      <x:c r="G5" s="38">
+      <x:c r="G5" s="44">
         <x:f t="shared" si="1"/>
         <x:v>46241</x:v>
       </x:c>
-      <x:c r="H5" s="39">
+      <x:c r="H5" s="45">
         <x:f t="shared" si="1"/>
         <x:v>46242</x:v>
       </x:c>
       <x:c r="I5" s="1"/>
+      <x:c r="J5" s="30"/>
+      <x:c r="K5" t="str"/>
+      <x:c r="L5" t="str"/>
+      <x:c r="M5" t="str">
+        <x:v>#4f8ef7</x:v>
+      </x:c>
+      <x:c r="N5" s="31" t="str"/>
+      <x:c r="O5" s="37" t="str"/>
+      <x:c r="P5" s="38" t="str"/>
+      <x:c r="Q5" s="38" t="str"/>
     </x:row>
     <x:row r="6" ht="80.0999984741211" customHeight="1">
-      <x:c r="B6" s="33" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=B5)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="C6" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=C5)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="D6" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=D5)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="E6" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=E5)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="F6" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=F5)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="G6" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=G5)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="H6" s="36" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=H5)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
+      <x:c r="B6" s="39" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=B5)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="C6" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=C5)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="D6" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=D5)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="E6" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=E5)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="F6" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=F5)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="G6" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=G5)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="H6" s="42" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=H5)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
       </x:c>
       <x:c r="I6" s="1"/>
     </x:row>
     <x:row r="7" ht="17.25" customHeight="1">
-      <x:c r="B7" s="37" t="n">
+      <x:c r="B7" s="43" t="n">
         <x:f>H5+1</x:f>
         <x:v>46243</x:v>
       </x:c>
-      <x:c r="C7" s="38" t="n">
+      <x:c r="C7" s="44" t="n">
         <x:f t="shared" ref="C7:H7" si="2">B7+1</x:f>
         <x:v>46244</x:v>
       </x:c>
-      <x:c r="D7" s="38">
+      <x:c r="D7" s="44">
         <x:f t="shared" si="2"/>
         <x:v>46245</x:v>
       </x:c>
-      <x:c r="E7" s="38">
+      <x:c r="E7" s="44">
         <x:f t="shared" si="2"/>
         <x:v>46246</x:v>
       </x:c>
-      <x:c r="F7" s="38">
+      <x:c r="F7" s="44">
         <x:f t="shared" si="2"/>
         <x:v>46247</x:v>
       </x:c>
-      <x:c r="G7" s="38">
+      <x:c r="G7" s="44">
         <x:f t="shared" si="2"/>
         <x:v>46248</x:v>
       </x:c>
-      <x:c r="H7" s="39">
+      <x:c r="H7" s="45">
         <x:f t="shared" si="2"/>
         <x:v>46249</x:v>
       </x:c>
       <x:c r="I7" s="1"/>
     </x:row>
     <x:row r="8" ht="80.0999984741211" customHeight="1">
-      <x:c r="B8" s="33" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=B7)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="C8" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=C7)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="D8" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=D7)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="E8" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=E7)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="F8" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=F7)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="G8" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=G7)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="H8" s="36" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=H7)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
+      <x:c r="B8" s="39" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=B7)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="C8" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=C7)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="D8" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=D7)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="E8" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=E7)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="F8" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=F7)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="G8" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=G7)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="H8" s="42" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=H7)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
       </x:c>
       <x:c r="I8" s="1"/>
     </x:row>
     <x:row r="9" ht="17.25" customHeight="1">
-      <x:c r="B9" s="37" t="n">
+      <x:c r="B9" s="43" t="n">
         <x:f>H7+1</x:f>
         <x:v>46250</x:v>
       </x:c>
-      <x:c r="C9" s="38" t="n">
+      <x:c r="C9" s="44" t="n">
         <x:f t="shared" ref="C9:H9" si="3">B9+1</x:f>
         <x:v>46251</x:v>
       </x:c>
-      <x:c r="D9" s="38">
+      <x:c r="D9" s="44">
         <x:f t="shared" si="3"/>
         <x:v>46252</x:v>
       </x:c>
-      <x:c r="E9" s="38">
+      <x:c r="E9" s="44">
         <x:f t="shared" si="3"/>
         <x:v>46253</x:v>
       </x:c>
-      <x:c r="F9" s="38">
+      <x:c r="F9" s="44">
         <x:f t="shared" si="3"/>
         <x:v>46254</x:v>
       </x:c>
-      <x:c r="G9" s="38">
+      <x:c r="G9" s="44">
         <x:f t="shared" si="3"/>
         <x:v>46255</x:v>
       </x:c>
-      <x:c r="H9" s="39">
+      <x:c r="H9" s="45">
         <x:f t="shared" si="3"/>
         <x:v>46256</x:v>
       </x:c>
       <x:c r="I9" s="1"/>
     </x:row>
     <x:row r="10" ht="80.0999984741211" customHeight="1">
-      <x:c r="B10" s="33" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=B9)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="C10" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=C9)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="D10" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=D9)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="E10" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=E9)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="F10" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=F9)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="G10" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=G9)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="H10" s="36" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=H9)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
+      <x:c r="B10" s="39" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=B9)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="C10" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=C9)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="D10" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=D9)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="E10" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=E9)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="F10" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=F9)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="G10" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=G9)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="H10" s="42" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=H9)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
       </x:c>
       <x:c r="I10" s="1"/>
     </x:row>
     <x:row r="11" ht="17.25" customHeight="1">
-      <x:c r="B11" s="37" t="n">
+      <x:c r="B11" s="43" t="n">
         <x:f>H9+1</x:f>
         <x:v>46257</x:v>
       </x:c>
-      <x:c r="C11" s="38" t="n">
+      <x:c r="C11" s="44" t="n">
         <x:f t="shared" ref="C11:H11" si="4">B11+1</x:f>
         <x:v>46258</x:v>
       </x:c>
-      <x:c r="D11" s="38">
+      <x:c r="D11" s="44">
         <x:f t="shared" si="4"/>
         <x:v>46259</x:v>
       </x:c>
-      <x:c r="E11" s="38">
+      <x:c r="E11" s="44">
         <x:f t="shared" si="4"/>
         <x:v>46260</x:v>
       </x:c>
-      <x:c r="F11" s="38">
+      <x:c r="F11" s="44">
         <x:f t="shared" si="4"/>
         <x:v>46261</x:v>
       </x:c>
-      <x:c r="G11" s="38">
+      <x:c r="G11" s="44">
         <x:f t="shared" si="4"/>
         <x:v>46262</x:v>
       </x:c>
-      <x:c r="H11" s="39">
+      <x:c r="H11" s="45">
         <x:f t="shared" si="4"/>
         <x:v>46263</x:v>
       </x:c>
       <x:c r="I11" s="1"/>
     </x:row>
     <x:row r="12" ht="80.0999984741211" customHeight="1">
-      <x:c r="B12" s="33" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=B11)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="C12" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=C11)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="D12" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=D11)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="E12" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=E11)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="F12" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=F11)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="G12" s="35" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=G11)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="H12" s="36" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=H11)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
+      <x:c r="B12" s="39" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=B11)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="C12" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=C11)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="D12" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=D11)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="E12" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=E11)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="F12" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=F11)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="G12" s="41" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=G11)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="H12" s="42" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=H11)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
       </x:c>
       <x:c r="I12" s="1"/>
     </x:row>
     <x:row r="13">
-      <x:c r="B13" s="37" t="n">
+      <x:c r="B13" s="43" t="n">
         <x:f>H11+1</x:f>
         <x:v>46264</x:v>
       </x:c>
-      <x:c r="C13" s="38" t="n">
+      <x:c r="C13" s="44" t="n">
         <x:f t="shared" ref="C13:H13" si="5">B13+1</x:f>
         <x:v>46265</x:v>
       </x:c>
-      <x:c r="D13" s="38">
+      <x:c r="D13" s="44">
         <x:f t="shared" si="5"/>
         <x:v>46266</x:v>
       </x:c>
-      <x:c r="E13" s="38">
+      <x:c r="E13" s="44">
         <x:f t="shared" si="5"/>
         <x:v>46267</x:v>
       </x:c>
-      <x:c r="F13" s="38">
+      <x:c r="F13" s="44">
         <x:f t="shared" si="5"/>
         <x:v>46268</x:v>
       </x:c>
-      <x:c r="G13" s="38">
+      <x:c r="G13" s="44">
         <x:f t="shared" si="5"/>
         <x:v>46269</x:v>
       </x:c>
-      <x:c r="H13" s="39">
+      <x:c r="H13" s="45">
         <x:f t="shared" si="5"/>
         <x:v>46270</x:v>
       </x:c>
       <x:c r="I13" s="1"/>
     </x:row>
     <x:row r="14" ht="80.0999984741211" customHeight="1">
-      <x:c r="B14" s="40" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=B13)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="C14" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=C13)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="D14" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=D13)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="E14" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=E13)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="F14" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=F13)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="G14" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=G13)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
-      </x:c>
-      <x:c r="H14" s="42" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(('일정데이터'!$B$5:$B$504=H13)*('일정데이터'!$H$5:$H$504=""),'일정데이터'!$C$5:$C$504,"")),"")</x:f>
+      <x:c r="B14" s="46" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=B13)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="C14" s="47" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=C13)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="D14" s="47" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=D13)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="E14" s="47" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=E13)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="F14" s="47" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=F13)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="G14" s="47" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=G13)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+      </x:c>
+      <x:c r="H14" s="48" t="str">
+        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=H13)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
       </x:c>
       <x:c r="I14" s="2"/>
     </x:row>
   </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="J1:Q1"/>
+    <x:mergeCell ref="J2:Q2"/>
+  </x:mergeCells>
   <x:conditionalFormatting sqref="B3:H3 B5:H5 B7:H7 B9:H9 B11:H11 B13:H13">
     <x:cfRule type="expression" dxfId="1" priority="3" stopIfTrue="1">
       <x:formula>MONTH(B3)&lt;&gt;$H$1</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="36" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="23" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="25" t="str">
-        <x:v>Cellendar 일정 동기화 데이터</x:v>
-      </x:c>
-      <x:c r="B1" s="25"/>
-      <x:c r="C1" s="25"/>
-      <x:c r="D1" s="25"/>
-      <x:c r="E1" s="25"/>
-      <x:c r="F1" s="25"/>
-      <x:c r="G1" s="25"/>
-      <x:c r="H1" s="25"/>
-    </x:row>
-    <x:row r="2" ht="26" customHeight="1">
-      <x:c r="A2" s="27" t="str">
-        <x:v>날짜와 제목을 입력하세요. ID·수정시간·삭제시간은 앱이 관리하므로 수정하지 마세요.</x:v>
-      </x:c>
-      <x:c r="B2" s="27"/>
-      <x:c r="C2" s="27"/>
-      <x:c r="D2" s="27"/>
-      <x:c r="E2" s="27"/>
-      <x:c r="F2" s="27"/>
-      <x:c r="G2" s="27"/>
-      <x:c r="H2" s="27"/>
-    </x:row>
-    <x:row r="4" ht="24" customHeight="1">
-      <x:c r="A4" s="29" t="str">
-        <x:v>ID</x:v>
-      </x:c>
-      <x:c r="B4" s="29" t="str">
-        <x:v>날짜</x:v>
-      </x:c>
-      <x:c r="C4" s="29" t="str">
-        <x:v>제목</x:v>
-      </x:c>
-      <x:c r="D4" s="29" t="str">
-        <x:v>메모</x:v>
-      </x:c>
-      <x:c r="E4" s="29" t="str">
-        <x:v>색상</x:v>
-      </x:c>
-      <x:c r="F4" s="29" t="str">
-        <x:v>알림시각</x:v>
-      </x:c>
-      <x:c r="G4" s="29" t="str">
-        <x:v>수정시간</x:v>
-      </x:c>
-      <x:c r="H4" s="29" t="str">
-        <x:v>삭제시간</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" t="str"/>
-      <x:c r="B5" s="30"/>
-      <x:c r="C5" t="str"/>
-      <x:c r="D5" t="str"/>
-      <x:c r="E5" t="str">
-        <x:v>#4f8ef7</x:v>
-      </x:c>
-      <x:c r="F5" s="31" t="str"/>
-      <x:c r="G5" s="32" t="str"/>
-      <x:c r="H5" s="32" t="str"/>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R198044018efe4887"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc9658e8ecab4408"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Excel calendar event display
</commit_message>
<xml_diff>
--- a/app/template/캘린더(자동).xlsx
+++ b/app/template/캘린더(자동).xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="R2c594194fa964a28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26.8" sheetId="1" r:id="R85b6f1c98ace4766"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="Rd5f1e1b4306d4543"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26.8" sheetId="1" r:id="R52b05809fe034df7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3445,25 +3445,25 @@
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="B4" s="39" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=B3)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="C4" s="40" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=C3)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="D4" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=D3)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="E4" s="40" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=E3)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="F4" s="40" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=F3)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="G4" s="40" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=G3)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="H4" s="42" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=H3)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="I4" s="1"/>
       <x:c r="J4" s="29" t="str">
@@ -3534,25 +3534,25 @@
     </x:row>
     <x:row r="6" ht="80.0999984741211" customHeight="1">
       <x:c r="B6" s="39" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=B5)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="C6" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=C5)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="D6" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=D5)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="E6" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=E5)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="F6" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=F5)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="G6" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=G5)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="H6" s="42" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=H5)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="I6" s="1"/>
     </x:row>
@@ -3589,25 +3589,25 @@
     </x:row>
     <x:row r="8" ht="80.0999984741211" customHeight="1">
       <x:c r="B8" s="39" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=B7)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="C8" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=C7)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="D8" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=D7)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="E8" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=E7)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="F8" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=F7)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="G8" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=G7)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="H8" s="42" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=H7)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="I8" s="1"/>
     </x:row>
@@ -3644,25 +3644,25 @@
     </x:row>
     <x:row r="10" ht="80.0999984741211" customHeight="1">
       <x:c r="B10" s="39" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=B9)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="C10" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=C9)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="D10" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=D9)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="E10" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=E9)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="F10" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=F9)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="G10" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=G9)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="H10" s="42" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=H9)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="I10" s="1"/>
     </x:row>
@@ -3699,25 +3699,25 @@
     </x:row>
     <x:row r="12" ht="80.0999984741211" customHeight="1">
       <x:c r="B12" s="39" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=B11)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="C12" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=C11)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="D12" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=D11)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="E12" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=E11)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="F12" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=F11)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="G12" s="41" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=G11)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="H12" s="42" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=H11)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="I12" s="1"/>
     </x:row>
@@ -3754,25 +3754,25 @@
     </x:row>
     <x:row r="14" ht="80.0999984741211" customHeight="1">
       <x:c r="B14" s="46" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=B13)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="C14" s="47" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=C13)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="D14" s="47" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=D13)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="E14" s="47" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=E13)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="F14" s="47" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=F13)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="G14" s="47" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=G13)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="H14" s="48" t="str">
-        <x:f>IFERROR(TEXTJOIN(CHAR(10),TRUE,IF(($J$5:$J$504=H13)*($Q$5:$Q$504=""),$K$5:$K$504,"")),"")</x:f>
+        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="I14" s="2"/>
     </x:row>
@@ -3788,7 +3788,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc9658e8ecab4408"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc90ee55832d947b0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Make Excel event entry user friendly
</commit_message>
<xml_diff>
--- a/app/template/캘린더(자동).xlsx
+++ b/app/template/캘린더(자동).xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="Rd5f1e1b4306d4543"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26.8" sheetId="1" r:id="R52b05809fe034df7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="R09f9af01ded440b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26.8" sheetId="1" r:id="R9078901e1f4b44c5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,7 +157,7 @@
     <x:numFmt numFmtId="201" formatCode="hh:mm"/>
     <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </x:numFmts>
-  <x:fonts count="18">
+  <x:fonts count="19">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -248,18 +248,22 @@
       <x:name val="맑은 고딕"/>
     </x:font>
     <x:font>
-      <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FF667085"/>
+      <x:color rgb="FF243447"/>
       <x:name val="맑은 고딕"/>
     </x:font>
     <x:font>
-      <x:sz val="11"/>
-      <x:color rgb="FF667085"/>
+      <x:sz val="9"/>
+      <x:color rgb="FF7A8492"/>
+      <x:name val="맑은 고딕"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF98A2B3"/>
       <x:name val="맑은 고딕"/>
     </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -298,11 +302,21 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF2F4F7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF7F9FC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="18">
+  <x:borders count="20">
     <x:border/>
     <x:border>
       <x:left style="medium">
@@ -503,13 +517,41 @@
         <x:color theme="0" tint="-0.15"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFE7DCA8"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFE7DCA8"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFE7DCA8"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFE7DCA8"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9DEE5"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9DEE5"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9DEE5"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9DEE5"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="49">
+  <x:cellXfs count="55">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -594,31 +636,49 @@
     <x:xf numFmtId="0" fontId="15" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="9" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="16" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="16" fillId="8" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="17" fillId="9" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="18" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="17" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="202" fontId="17" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="18" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -672,18 +732,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CalendarEvents" displayName="CalendarEvents" ref="J4:Q5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CalendarEvents" displayName="CalendarEvents" ref="J4:Q34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="날짜"/>
     <x:tableColumn id="2" name="제목"/>
     <x:tableColumn id="3" name="메모"/>
-    <x:tableColumn id="4" name="색상"/>
-    <x:tableColumn id="5" name="알림시각"/>
+    <x:tableColumn id="4" name="알림시각"/>
+    <x:tableColumn id="5" name="색상"/>
     <x:tableColumn id="6" name="ID"/>
     <x:tableColumn id="7" name="수정시간"/>
     <x:tableColumn id="8" name="삭제시간"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -3346,13 +3406,15 @@
     <x:col min="2" max="8" width="26.625" style="8" customWidth="1"/>
     <x:col min="9" max="9" width="54" style="8" customWidth="1"/>
     <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="34" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="32" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="13" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="13" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="34" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="23" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="23" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="12" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="18" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="14" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="11" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -3375,6 +3437,12 @@
       <x:c r="O1" s="25"/>
       <x:c r="P1" s="25"/>
       <x:c r="Q1" s="25"/>
+      <x:c r="S1" s="43" t="str">
+        <x:v>자동 날짜 목록</x:v>
+      </x:c>
+      <x:c r="T1" s="43" t="str">
+        <x:v>색상 목록</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="B2" s="4" t="s">
@@ -3402,7 +3470,7 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="J2" s="27" t="str">
-        <x:v>날짜·제목·메모를 입력하세요. ID·수정시간·삭제시간은 앱이 관리합니다.</x:v>
+        <x:v>노란 칸만 입력하세요. 날짜와 색상은 목록에서 선택할 수 있습니다.</x:v>
       </x:c>
       <x:c r="K2" s="27"/>
       <x:c r="L2" s="27"/>
@@ -3411,6 +3479,13 @@
       <x:c r="O2" s="27"/>
       <x:c r="P2" s="27"/>
       <x:c r="Q2" s="27"/>
+      <x:c r="S2" s="44" t="n">
+        <x:f>IF(1&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,1),"")</x:f>
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="T2" s="43" t="str">
+        <x:v>파랑</x:v>
+      </x:c>
     </x:row>
     <x:row r="3" ht="17.25" customHeight="1">
       <x:c r="B3" s="11" t="n">
@@ -3442,339 +3517,771 @@
         <x:v>46235</x:v>
       </x:c>
       <x:c r="I3" s="1"/>
+      <x:c r="S3" s="44" t="n">
+        <x:f>IF(2&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,2),"")</x:f>
+        <x:v>46236</x:v>
+      </x:c>
+      <x:c r="T3" s="43" t="str">
+        <x:v>빨강</x:v>
+      </x:c>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
-      <x:c r="B4" s="39" t="str">
+      <x:c r="B4" s="45" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="C4" s="40" t="str">
+      <x:c r="C4" s="46" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="D4" s="41" t="str">
+      <x:c r="D4" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="E4" s="40" t="str">
+      <x:c r="E4" s="46" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="F4" s="40" t="str">
+      <x:c r="F4" s="46" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="G4" s="40" t="str">
+      <x:c r="G4" s="46" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="H4" s="42" t="str">
+      <x:c r="H4" s="48" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="I4" s="1"/>
-      <x:c r="J4" s="29" t="str">
+      <x:c r="J4" s="30" t="str">
         <x:v>날짜</x:v>
       </x:c>
-      <x:c r="K4" s="29" t="str">
+      <x:c r="K4" s="30" t="str">
         <x:v>제목</x:v>
       </x:c>
-      <x:c r="L4" s="29" t="str">
+      <x:c r="L4" s="30" t="str">
         <x:v>메모</x:v>
       </x:c>
-      <x:c r="M4" s="29" t="str">
+      <x:c r="M4" s="30" t="str">
+        <x:v>알림시각</x:v>
+      </x:c>
+      <x:c r="N4" s="30" t="str">
         <x:v>색상</x:v>
       </x:c>
-      <x:c r="N4" s="29" t="str">
-        <x:v>알림시각</x:v>
-      </x:c>
-      <x:c r="O4" s="36" t="str">
+      <x:c r="O4" s="30" t="str">
         <x:v>ID</x:v>
       </x:c>
-      <x:c r="P4" s="36" t="str">
+      <x:c r="P4" s="30" t="str">
         <x:v>수정시간</x:v>
       </x:c>
-      <x:c r="Q4" s="36" t="str">
+      <x:c r="Q4" s="30" t="str">
         <x:v>삭제시간</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" ht="17.25" customHeight="1">
-      <x:c r="B5" s="43" t="n">
+      <x:c r="S4" s="44" t="n">
+        <x:f>IF(3&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,3),"")</x:f>
+        <x:v>46237</x:v>
+      </x:c>
+      <x:c r="T4" s="43" t="str">
+        <x:v>초록</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="B5" s="49" t="n">
         <x:f>H3+1</x:f>
         <x:v>46236</x:v>
       </x:c>
-      <x:c r="C5" s="44" t="n">
+      <x:c r="C5" s="50" t="n">
         <x:f t="shared" ref="C5:H5" si="1">B5+1</x:f>
         <x:v>46237</x:v>
       </x:c>
-      <x:c r="D5" s="44">
+      <x:c r="D5" s="50">
         <x:f t="shared" si="1"/>
         <x:v>46238</x:v>
       </x:c>
-      <x:c r="E5" s="44">
+      <x:c r="E5" s="50">
         <x:f t="shared" si="1"/>
         <x:v>46239</x:v>
       </x:c>
-      <x:c r="F5" s="44">
+      <x:c r="F5" s="50">
         <x:f t="shared" si="1"/>
         <x:v>46240</x:v>
       </x:c>
-      <x:c r="G5" s="44">
+      <x:c r="G5" s="50">
         <x:f t="shared" si="1"/>
         <x:v>46241</x:v>
       </x:c>
-      <x:c r="H5" s="45">
+      <x:c r="H5" s="51">
         <x:f t="shared" si="1"/>
         <x:v>46242</x:v>
       </x:c>
       <x:c r="I5" s="1"/>
-      <x:c r="J5" s="30"/>
-      <x:c r="K5" t="str"/>
-      <x:c r="L5" t="str"/>
-      <x:c r="M5" t="str">
-        <x:v>#4f8ef7</x:v>
-      </x:c>
-      <x:c r="N5" s="31" t="str"/>
-      <x:c r="O5" s="37" t="str"/>
-      <x:c r="P5" s="38" t="str"/>
-      <x:c r="Q5" s="38" t="str"/>
-    </x:row>
-    <x:row r="6" ht="80.0999984741211" customHeight="1">
-      <x:c r="B6" s="39" t="str">
+      <x:c r="J5" s="37" t="str"/>
+      <x:c r="K5" s="33" t="str"/>
+      <x:c r="L5" s="33" t="str"/>
+      <x:c r="M5" s="38" t="str"/>
+      <x:c r="N5" s="33" t="str"/>
+      <x:c r="O5" s="36" t="str"/>
+      <x:c r="P5" s="39" t="str"/>
+      <x:c r="Q5" s="39" t="str"/>
+      <x:c r="S5" s="44" t="n">
+        <x:f>IF(4&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,4),"")</x:f>
+        <x:v>46238</x:v>
+      </x:c>
+      <x:c r="T5" s="43" t="str">
+        <x:v>주황</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="B6" s="45" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="C6" s="41" t="str">
+      <x:c r="C6" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="D6" s="41" t="str">
+      <x:c r="D6" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="E6" s="41" t="str">
+      <x:c r="E6" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="F6" s="41" t="str">
+      <x:c r="F6" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="G6" s="41" t="str">
+      <x:c r="G6" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="H6" s="42" t="str">
+      <x:c r="H6" s="48" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="I6" s="1"/>
-    </x:row>
-    <x:row r="7" ht="17.25" customHeight="1">
-      <x:c r="B7" s="43" t="n">
+      <x:c r="J6" s="37" t="str"/>
+      <x:c r="K6" s="33" t="str"/>
+      <x:c r="L6" s="33" t="str"/>
+      <x:c r="M6" s="38" t="str"/>
+      <x:c r="N6" s="33" t="str"/>
+      <x:c r="O6" s="36" t="str"/>
+      <x:c r="P6" s="39" t="str"/>
+      <x:c r="Q6" s="39" t="str"/>
+      <x:c r="S6" s="44" t="n">
+        <x:f>IF(5&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,5),"")</x:f>
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="T6" s="43" t="str">
+        <x:v>보라</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="B7" s="49" t="n">
         <x:f>H5+1</x:f>
         <x:v>46243</x:v>
       </x:c>
-      <x:c r="C7" s="44" t="n">
+      <x:c r="C7" s="50" t="n">
         <x:f t="shared" ref="C7:H7" si="2">B7+1</x:f>
         <x:v>46244</x:v>
       </x:c>
-      <x:c r="D7" s="44">
+      <x:c r="D7" s="50">
         <x:f t="shared" si="2"/>
         <x:v>46245</x:v>
       </x:c>
-      <x:c r="E7" s="44">
+      <x:c r="E7" s="50">
         <x:f t="shared" si="2"/>
         <x:v>46246</x:v>
       </x:c>
-      <x:c r="F7" s="44">
+      <x:c r="F7" s="50">
         <x:f t="shared" si="2"/>
         <x:v>46247</x:v>
       </x:c>
-      <x:c r="G7" s="44">
+      <x:c r="G7" s="50">
         <x:f t="shared" si="2"/>
         <x:v>46248</x:v>
       </x:c>
-      <x:c r="H7" s="45">
+      <x:c r="H7" s="51">
         <x:f t="shared" si="2"/>
         <x:v>46249</x:v>
       </x:c>
       <x:c r="I7" s="1"/>
-    </x:row>
-    <x:row r="8" ht="80.0999984741211" customHeight="1">
-      <x:c r="B8" s="39" t="str">
+      <x:c r="J7" s="37" t="str"/>
+      <x:c r="K7" s="33" t="str"/>
+      <x:c r="L7" s="33" t="str"/>
+      <x:c r="M7" s="38" t="str"/>
+      <x:c r="N7" s="33" t="str"/>
+      <x:c r="O7" s="36" t="str"/>
+      <x:c r="P7" s="39" t="str"/>
+      <x:c r="Q7" s="39" t="str"/>
+      <x:c r="S7" s="44" t="n">
+        <x:f>IF(6&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,6),"")</x:f>
+        <x:v>46240</x:v>
+      </x:c>
+      <x:c r="T7" s="43" t="str">
+        <x:v>분홍</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="22" customHeight="1">
+      <x:c r="B8" s="45" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="C8" s="41" t="str">
+      <x:c r="C8" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="D8" s="41" t="str">
+      <x:c r="D8" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="E8" s="41" t="str">
+      <x:c r="E8" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="F8" s="41" t="str">
+      <x:c r="F8" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="G8" s="41" t="str">
+      <x:c r="G8" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="H8" s="42" t="str">
+      <x:c r="H8" s="48" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="I8" s="1"/>
-    </x:row>
-    <x:row r="9" ht="17.25" customHeight="1">
-      <x:c r="B9" s="43" t="n">
+      <x:c r="J8" s="37" t="str"/>
+      <x:c r="K8" s="33" t="str"/>
+      <x:c r="L8" s="33" t="str"/>
+      <x:c r="M8" s="38" t="str"/>
+      <x:c r="N8" s="33" t="str"/>
+      <x:c r="O8" s="36" t="str"/>
+      <x:c r="P8" s="39" t="str"/>
+      <x:c r="Q8" s="39" t="str"/>
+      <x:c r="S8" s="44" t="n">
+        <x:f>IF(7&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,7),"")</x:f>
+        <x:v>46241</x:v>
+      </x:c>
+      <x:c r="T8" s="43" t="str">
+        <x:v>회색</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="22" customHeight="1">
+      <x:c r="B9" s="49" t="n">
         <x:f>H7+1</x:f>
         <x:v>46250</x:v>
       </x:c>
-      <x:c r="C9" s="44" t="n">
+      <x:c r="C9" s="50" t="n">
         <x:f t="shared" ref="C9:H9" si="3">B9+1</x:f>
         <x:v>46251</x:v>
       </x:c>
-      <x:c r="D9" s="44">
+      <x:c r="D9" s="50">
         <x:f t="shared" si="3"/>
         <x:v>46252</x:v>
       </x:c>
-      <x:c r="E9" s="44">
+      <x:c r="E9" s="50">
         <x:f t="shared" si="3"/>
         <x:v>46253</x:v>
       </x:c>
-      <x:c r="F9" s="44">
+      <x:c r="F9" s="50">
         <x:f t="shared" si="3"/>
         <x:v>46254</x:v>
       </x:c>
-      <x:c r="G9" s="44">
+      <x:c r="G9" s="50">
         <x:f t="shared" si="3"/>
         <x:v>46255</x:v>
       </x:c>
-      <x:c r="H9" s="45">
+      <x:c r="H9" s="51">
         <x:f t="shared" si="3"/>
         <x:v>46256</x:v>
       </x:c>
       <x:c r="I9" s="1"/>
-    </x:row>
-    <x:row r="10" ht="80.0999984741211" customHeight="1">
-      <x:c r="B10" s="39" t="str">
+      <x:c r="J9" s="37" t="str"/>
+      <x:c r="K9" s="33" t="str"/>
+      <x:c r="L9" s="33" t="str"/>
+      <x:c r="M9" s="38" t="str"/>
+      <x:c r="N9" s="33" t="str"/>
+      <x:c r="O9" s="36" t="str"/>
+      <x:c r="P9" s="39" t="str"/>
+      <x:c r="Q9" s="39" t="str"/>
+      <x:c r="S9" s="44" t="n">
+        <x:f>IF(8&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,8),"")</x:f>
+        <x:v>46242</x:v>
+      </x:c>
+      <x:c r="T9" s="43"/>
+    </x:row>
+    <x:row r="10" ht="22" customHeight="1">
+      <x:c r="B10" s="45" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="C10" s="41" t="str">
+      <x:c r="C10" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="D10" s="41" t="str">
+      <x:c r="D10" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="E10" s="41" t="str">
+      <x:c r="E10" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="F10" s="41" t="str">
+      <x:c r="F10" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="G10" s="41" t="str">
+      <x:c r="G10" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="H10" s="42" t="str">
+      <x:c r="H10" s="48" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="I10" s="1"/>
-    </x:row>
-    <x:row r="11" ht="17.25" customHeight="1">
-      <x:c r="B11" s="43" t="n">
+      <x:c r="J10" s="37" t="str"/>
+      <x:c r="K10" s="33" t="str"/>
+      <x:c r="L10" s="33" t="str"/>
+      <x:c r="M10" s="38" t="str"/>
+      <x:c r="N10" s="33" t="str"/>
+      <x:c r="O10" s="36" t="str"/>
+      <x:c r="P10" s="39" t="str"/>
+      <x:c r="Q10" s="39" t="str"/>
+      <x:c r="S10" s="44" t="n">
+        <x:f>IF(9&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,9),"")</x:f>
+        <x:v>46243</x:v>
+      </x:c>
+      <x:c r="T10" s="43"/>
+    </x:row>
+    <x:row r="11" ht="22" customHeight="1">
+      <x:c r="B11" s="49" t="n">
         <x:f>H9+1</x:f>
         <x:v>46257</x:v>
       </x:c>
-      <x:c r="C11" s="44" t="n">
+      <x:c r="C11" s="50" t="n">
         <x:f t="shared" ref="C11:H11" si="4">B11+1</x:f>
         <x:v>46258</x:v>
       </x:c>
-      <x:c r="D11" s="44">
+      <x:c r="D11" s="50">
         <x:f t="shared" si="4"/>
         <x:v>46259</x:v>
       </x:c>
-      <x:c r="E11" s="44">
+      <x:c r="E11" s="50">
         <x:f t="shared" si="4"/>
         <x:v>46260</x:v>
       </x:c>
-      <x:c r="F11" s="44">
+      <x:c r="F11" s="50">
         <x:f t="shared" si="4"/>
         <x:v>46261</x:v>
       </x:c>
-      <x:c r="G11" s="44">
+      <x:c r="G11" s="50">
         <x:f t="shared" si="4"/>
         <x:v>46262</x:v>
       </x:c>
-      <x:c r="H11" s="45">
+      <x:c r="H11" s="51">
         <x:f t="shared" si="4"/>
         <x:v>46263</x:v>
       </x:c>
       <x:c r="I11" s="1"/>
-    </x:row>
-    <x:row r="12" ht="80.0999984741211" customHeight="1">
-      <x:c r="B12" s="39" t="str">
+      <x:c r="J11" s="37" t="str"/>
+      <x:c r="K11" s="33" t="str"/>
+      <x:c r="L11" s="33" t="str"/>
+      <x:c r="M11" s="38" t="str"/>
+      <x:c r="N11" s="33" t="str"/>
+      <x:c r="O11" s="36" t="str"/>
+      <x:c r="P11" s="39" t="str"/>
+      <x:c r="Q11" s="39" t="str"/>
+      <x:c r="S11" s="44" t="n">
+        <x:f>IF(10&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,10),"")</x:f>
+        <x:v>46244</x:v>
+      </x:c>
+      <x:c r="T11" s="43"/>
+    </x:row>
+    <x:row r="12" ht="22" customHeight="1">
+      <x:c r="B12" s="45" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="C12" s="41" t="str">
+      <x:c r="C12" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="D12" s="41" t="str">
+      <x:c r="D12" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="E12" s="41" t="str">
+      <x:c r="E12" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="F12" s="41" t="str">
+      <x:c r="F12" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="G12" s="41" t="str">
+      <x:c r="G12" s="47" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="H12" s="42" t="str">
+      <x:c r="H12" s="48" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="I12" s="1"/>
-    </x:row>
-    <x:row r="13">
-      <x:c r="B13" s="43" t="n">
+      <x:c r="J12" s="37" t="str"/>
+      <x:c r="K12" s="33" t="str"/>
+      <x:c r="L12" s="33" t="str"/>
+      <x:c r="M12" s="38" t="str"/>
+      <x:c r="N12" s="33" t="str"/>
+      <x:c r="O12" s="36" t="str"/>
+      <x:c r="P12" s="39" t="str"/>
+      <x:c r="Q12" s="39" t="str"/>
+      <x:c r="S12" s="44" t="n">
+        <x:f>IF(11&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,11),"")</x:f>
+        <x:v>46245</x:v>
+      </x:c>
+      <x:c r="T12" s="43"/>
+    </x:row>
+    <x:row r="13" ht="22" customHeight="1">
+      <x:c r="B13" s="49" t="n">
         <x:f>H11+1</x:f>
         <x:v>46264</x:v>
       </x:c>
-      <x:c r="C13" s="44" t="n">
+      <x:c r="C13" s="50" t="n">
         <x:f t="shared" ref="C13:H13" si="5">B13+1</x:f>
         <x:v>46265</x:v>
       </x:c>
-      <x:c r="D13" s="44">
+      <x:c r="D13" s="50">
         <x:f t="shared" si="5"/>
         <x:v>46266</x:v>
       </x:c>
-      <x:c r="E13" s="44">
+      <x:c r="E13" s="50">
         <x:f t="shared" si="5"/>
         <x:v>46267</x:v>
       </x:c>
-      <x:c r="F13" s="44">
+      <x:c r="F13" s="50">
         <x:f t="shared" si="5"/>
         <x:v>46268</x:v>
       </x:c>
-      <x:c r="G13" s="44">
+      <x:c r="G13" s="50">
         <x:f t="shared" si="5"/>
         <x:v>46269</x:v>
       </x:c>
-      <x:c r="H13" s="45">
+      <x:c r="H13" s="51">
         <x:f t="shared" si="5"/>
         <x:v>46270</x:v>
       </x:c>
       <x:c r="I13" s="1"/>
-    </x:row>
-    <x:row r="14" ht="80.0999984741211" customHeight="1">
-      <x:c r="B14" s="46" t="str">
+      <x:c r="J13" s="37" t="str"/>
+      <x:c r="K13" s="33" t="str"/>
+      <x:c r="L13" s="33" t="str"/>
+      <x:c r="M13" s="38" t="str"/>
+      <x:c r="N13" s="33" t="str"/>
+      <x:c r="O13" s="36" t="str"/>
+      <x:c r="P13" s="39" t="str"/>
+      <x:c r="Q13" s="39" t="str"/>
+      <x:c r="S13" s="44" t="n">
+        <x:f>IF(12&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,12),"")</x:f>
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="T13" s="43"/>
+    </x:row>
+    <x:row r="14" ht="22" customHeight="1">
+      <x:c r="B14" s="52" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="C14" s="47" t="str">
+      <x:c r="C14" s="53" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="D14" s="47" t="str">
+      <x:c r="D14" s="53" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="E14" s="47" t="str">
+      <x:c r="E14" s="53" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="F14" s="47" t="str">
+      <x:c r="F14" s="53" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="G14" s="47" t="str">
+      <x:c r="G14" s="53" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
-      <x:c r="H14" s="48" t="str">
+      <x:c r="H14" s="54" t="str">
         <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
       </x:c>
       <x:c r="I14" s="2"/>
+      <x:c r="J14" s="37" t="str"/>
+      <x:c r="K14" s="33" t="str"/>
+      <x:c r="L14" s="33" t="str"/>
+      <x:c r="M14" s="38" t="str"/>
+      <x:c r="N14" s="33" t="str"/>
+      <x:c r="O14" s="36" t="str"/>
+      <x:c r="P14" s="39" t="str"/>
+      <x:c r="Q14" s="39" t="str"/>
+      <x:c r="S14" s="44" t="n">
+        <x:f>IF(13&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,13),"")</x:f>
+        <x:v>46247</x:v>
+      </x:c>
+      <x:c r="T14" s="43"/>
+    </x:row>
+    <x:row r="15" ht="22" customHeight="1">
+      <x:c r="J15" s="37" t="str"/>
+      <x:c r="K15" s="33" t="str"/>
+      <x:c r="L15" s="33" t="str"/>
+      <x:c r="M15" s="38" t="str"/>
+      <x:c r="N15" s="33" t="str"/>
+      <x:c r="O15" s="36" t="str"/>
+      <x:c r="P15" s="39" t="str"/>
+      <x:c r="Q15" s="39" t="str"/>
+      <x:c r="S15" s="44" t="n">
+        <x:f>IF(14&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,14),"")</x:f>
+        <x:v>46248</x:v>
+      </x:c>
+      <x:c r="T15" s="43"/>
+    </x:row>
+    <x:row r="16" ht="22" customHeight="1">
+      <x:c r="J16" s="37" t="str"/>
+      <x:c r="K16" s="33" t="str"/>
+      <x:c r="L16" s="33" t="str"/>
+      <x:c r="M16" s="38" t="str"/>
+      <x:c r="N16" s="33" t="str"/>
+      <x:c r="O16" s="36" t="str"/>
+      <x:c r="P16" s="39" t="str"/>
+      <x:c r="Q16" s="39" t="str"/>
+      <x:c r="S16" s="44" t="n">
+        <x:f>IF(15&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,15),"")</x:f>
+        <x:v>46249</x:v>
+      </x:c>
+      <x:c r="T16" s="43"/>
+    </x:row>
+    <x:row r="17" ht="22" customHeight="1">
+      <x:c r="J17" s="37" t="str"/>
+      <x:c r="K17" s="33" t="str"/>
+      <x:c r="L17" s="33" t="str"/>
+      <x:c r="M17" s="38" t="str"/>
+      <x:c r="N17" s="33" t="str"/>
+      <x:c r="O17" s="36" t="str"/>
+      <x:c r="P17" s="39" t="str"/>
+      <x:c r="Q17" s="39" t="str"/>
+      <x:c r="S17" s="44" t="n">
+        <x:f>IF(16&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,16),"")</x:f>
+        <x:v>46250</x:v>
+      </x:c>
+      <x:c r="T17" s="43"/>
+    </x:row>
+    <x:row r="18" ht="22" customHeight="1">
+      <x:c r="J18" s="37" t="str"/>
+      <x:c r="K18" s="33" t="str"/>
+      <x:c r="L18" s="33" t="str"/>
+      <x:c r="M18" s="38" t="str"/>
+      <x:c r="N18" s="33" t="str"/>
+      <x:c r="O18" s="36" t="str"/>
+      <x:c r="P18" s="39" t="str"/>
+      <x:c r="Q18" s="39" t="str"/>
+      <x:c r="S18" s="44" t="n">
+        <x:f>IF(17&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,17),"")</x:f>
+        <x:v>46251</x:v>
+      </x:c>
+      <x:c r="T18" s="43"/>
+    </x:row>
+    <x:row r="19" ht="22" customHeight="1">
+      <x:c r="J19" s="37" t="str"/>
+      <x:c r="K19" s="33" t="str"/>
+      <x:c r="L19" s="33" t="str"/>
+      <x:c r="M19" s="38" t="str"/>
+      <x:c r="N19" s="33" t="str"/>
+      <x:c r="O19" s="36" t="str"/>
+      <x:c r="P19" s="39" t="str"/>
+      <x:c r="Q19" s="39" t="str"/>
+      <x:c r="S19" s="44" t="n">
+        <x:f>IF(18&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,18),"")</x:f>
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="T19" s="43"/>
+    </x:row>
+    <x:row r="20" ht="22" customHeight="1">
+      <x:c r="J20" s="37" t="str"/>
+      <x:c r="K20" s="33" t="str"/>
+      <x:c r="L20" s="33" t="str"/>
+      <x:c r="M20" s="38" t="str"/>
+      <x:c r="N20" s="33" t="str"/>
+      <x:c r="O20" s="36" t="str"/>
+      <x:c r="P20" s="39" t="str"/>
+      <x:c r="Q20" s="39" t="str"/>
+      <x:c r="S20" s="44" t="n">
+        <x:f>IF(19&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,19),"")</x:f>
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="T20" s="43"/>
+    </x:row>
+    <x:row r="21" ht="22" customHeight="1">
+      <x:c r="J21" s="37" t="str"/>
+      <x:c r="K21" s="33" t="str"/>
+      <x:c r="L21" s="33" t="str"/>
+      <x:c r="M21" s="38" t="str"/>
+      <x:c r="N21" s="33" t="str"/>
+      <x:c r="O21" s="36" t="str"/>
+      <x:c r="P21" s="39" t="str"/>
+      <x:c r="Q21" s="39" t="str"/>
+      <x:c r="S21" s="44" t="n">
+        <x:f>IF(20&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,20),"")</x:f>
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="T21" s="43"/>
+    </x:row>
+    <x:row r="22" ht="22" customHeight="1">
+      <x:c r="J22" s="37" t="str"/>
+      <x:c r="K22" s="33" t="str"/>
+      <x:c r="L22" s="33" t="str"/>
+      <x:c r="M22" s="38" t="str"/>
+      <x:c r="N22" s="33" t="str"/>
+      <x:c r="O22" s="36" t="str"/>
+      <x:c r="P22" s="39" t="str"/>
+      <x:c r="Q22" s="39" t="str"/>
+      <x:c r="S22" s="44" t="n">
+        <x:f>IF(21&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,21),"")</x:f>
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="T22" s="43"/>
+    </x:row>
+    <x:row r="23" ht="22" customHeight="1">
+      <x:c r="J23" s="37" t="str"/>
+      <x:c r="K23" s="33" t="str"/>
+      <x:c r="L23" s="33" t="str"/>
+      <x:c r="M23" s="38" t="str"/>
+      <x:c r="N23" s="33" t="str"/>
+      <x:c r="O23" s="36" t="str"/>
+      <x:c r="P23" s="39" t="str"/>
+      <x:c r="Q23" s="39" t="str"/>
+      <x:c r="S23" s="44" t="n">
+        <x:f>IF(22&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,22),"")</x:f>
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="T23" s="43"/>
+    </x:row>
+    <x:row r="24" ht="22" customHeight="1">
+      <x:c r="J24" s="37" t="str"/>
+      <x:c r="K24" s="33" t="str"/>
+      <x:c r="L24" s="33" t="str"/>
+      <x:c r="M24" s="38" t="str"/>
+      <x:c r="N24" s="33" t="str"/>
+      <x:c r="O24" s="36" t="str"/>
+      <x:c r="P24" s="39" t="str"/>
+      <x:c r="Q24" s="39" t="str"/>
+      <x:c r="S24" s="44" t="n">
+        <x:f>IF(23&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,23),"")</x:f>
+        <x:v>46257</x:v>
+      </x:c>
+      <x:c r="T24" s="43"/>
+    </x:row>
+    <x:row r="25" ht="22" customHeight="1">
+      <x:c r="J25" s="37" t="str"/>
+      <x:c r="K25" s="33" t="str"/>
+      <x:c r="L25" s="33" t="str"/>
+      <x:c r="M25" s="38" t="str"/>
+      <x:c r="N25" s="33" t="str"/>
+      <x:c r="O25" s="36" t="str"/>
+      <x:c r="P25" s="39" t="str"/>
+      <x:c r="Q25" s="39" t="str"/>
+      <x:c r="S25" s="44" t="n">
+        <x:f>IF(24&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,24),"")</x:f>
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="T25" s="43"/>
+    </x:row>
+    <x:row r="26" ht="22" customHeight="1">
+      <x:c r="J26" s="37" t="str"/>
+      <x:c r="K26" s="33" t="str"/>
+      <x:c r="L26" s="33" t="str"/>
+      <x:c r="M26" s="38" t="str"/>
+      <x:c r="N26" s="33" t="str"/>
+      <x:c r="O26" s="36" t="str"/>
+      <x:c r="P26" s="39" t="str"/>
+      <x:c r="Q26" s="39" t="str"/>
+      <x:c r="S26" s="44" t="n">
+        <x:f>IF(25&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,25),"")</x:f>
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="T26" s="43"/>
+    </x:row>
+    <x:row r="27" ht="22" customHeight="1">
+      <x:c r="J27" s="37" t="str"/>
+      <x:c r="K27" s="33" t="str"/>
+      <x:c r="L27" s="33" t="str"/>
+      <x:c r="M27" s="38" t="str"/>
+      <x:c r="N27" s="33" t="str"/>
+      <x:c r="O27" s="36" t="str"/>
+      <x:c r="P27" s="39" t="str"/>
+      <x:c r="Q27" s="39" t="str"/>
+      <x:c r="S27" s="44" t="n">
+        <x:f>IF(26&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,26),"")</x:f>
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="T27" s="43"/>
+    </x:row>
+    <x:row r="28" ht="22" customHeight="1">
+      <x:c r="J28" s="37" t="str"/>
+      <x:c r="K28" s="33" t="str"/>
+      <x:c r="L28" s="33" t="str"/>
+      <x:c r="M28" s="38" t="str"/>
+      <x:c r="N28" s="33" t="str"/>
+      <x:c r="O28" s="36" t="str"/>
+      <x:c r="P28" s="39" t="str"/>
+      <x:c r="Q28" s="39" t="str"/>
+      <x:c r="S28" s="44" t="n">
+        <x:f>IF(27&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,27),"")</x:f>
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="T28" s="43"/>
+    </x:row>
+    <x:row r="29" ht="22" customHeight="1">
+      <x:c r="J29" s="37" t="str"/>
+      <x:c r="K29" s="33" t="str"/>
+      <x:c r="L29" s="33" t="str"/>
+      <x:c r="M29" s="38" t="str"/>
+      <x:c r="N29" s="33" t="str"/>
+      <x:c r="O29" s="36" t="str"/>
+      <x:c r="P29" s="39" t="str"/>
+      <x:c r="Q29" s="39" t="str"/>
+      <x:c r="S29" s="44" t="n">
+        <x:f>IF(28&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,28),"")</x:f>
+        <x:v>46262</x:v>
+      </x:c>
+      <x:c r="T29" s="43"/>
+    </x:row>
+    <x:row r="30" ht="22" customHeight="1">
+      <x:c r="J30" s="37" t="str"/>
+      <x:c r="K30" s="33" t="str"/>
+      <x:c r="L30" s="33" t="str"/>
+      <x:c r="M30" s="38" t="str"/>
+      <x:c r="N30" s="33" t="str"/>
+      <x:c r="O30" s="36" t="str"/>
+      <x:c r="P30" s="39" t="str"/>
+      <x:c r="Q30" s="39" t="str"/>
+      <x:c r="S30" s="44" t="n">
+        <x:f>IF(29&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,29),"")</x:f>
+        <x:v>46263</x:v>
+      </x:c>
+      <x:c r="T30" s="43"/>
+    </x:row>
+    <x:row r="31" ht="22" customHeight="1">
+      <x:c r="J31" s="37" t="str"/>
+      <x:c r="K31" s="33" t="str"/>
+      <x:c r="L31" s="33" t="str"/>
+      <x:c r="M31" s="38" t="str"/>
+      <x:c r="N31" s="33" t="str"/>
+      <x:c r="O31" s="36" t="str"/>
+      <x:c r="P31" s="39" t="str"/>
+      <x:c r="Q31" s="39" t="str"/>
+      <x:c r="S31" s="44" t="n">
+        <x:f>IF(30&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,30),"")</x:f>
+        <x:v>46264</x:v>
+      </x:c>
+      <x:c r="T31" s="43"/>
+    </x:row>
+    <x:row r="32" ht="22" customHeight="1">
+      <x:c r="J32" s="37" t="str"/>
+      <x:c r="K32" s="33" t="str"/>
+      <x:c r="L32" s="33" t="str"/>
+      <x:c r="M32" s="38" t="str"/>
+      <x:c r="N32" s="33" t="str"/>
+      <x:c r="O32" s="36" t="str"/>
+      <x:c r="P32" s="39" t="str"/>
+      <x:c r="Q32" s="39" t="str"/>
+      <x:c r="S32" s="44" t="n">
+        <x:f>IF(31&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,31),"")</x:f>
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="T32" s="43"/>
+    </x:row>
+    <x:row r="33" ht="22" customHeight="1">
+      <x:c r="J33" s="37" t="str"/>
+      <x:c r="K33" s="33" t="str"/>
+      <x:c r="L33" s="33" t="str"/>
+      <x:c r="M33" s="38" t="str"/>
+      <x:c r="N33" s="33" t="str"/>
+      <x:c r="O33" s="36" t="str"/>
+      <x:c r="P33" s="39" t="str"/>
+      <x:c r="Q33" s="39" t="str"/>
+    </x:row>
+    <x:row r="34" ht="22" customHeight="1">
+      <x:c r="J34" s="37" t="str"/>
+      <x:c r="K34" s="33" t="str"/>
+      <x:c r="L34" s="33" t="str"/>
+      <x:c r="M34" s="38" t="str"/>
+      <x:c r="N34" s="33" t="str"/>
+      <x:c r="O34" s="36" t="str"/>
+      <x:c r="P34" s="39" t="str"/>
+      <x:c r="Q34" s="39" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3786,9 +4293,17 @@
       <x:formula>MONTH(B3)&lt;&gt;$H$1</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="J5:J34">
+      <x:formula1>$S$2:$S$32</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="N5:N34">
+      <x:formula1>$T$2:$T$8</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc90ee55832d947b0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70c0dc9ffcfd4754"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Show multiple events in larger Excel calendar
</commit_message>
<xml_diff>
--- a/app/template/캘린더(자동).xlsx
+++ b/app/template/캘린더(자동).xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="R09f9af01ded440b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26.8" sheetId="1" r:id="R9078901e1f4b44c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="Recd4d1d50b864195"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26.8" sheetId="1" r:id="R4d8dd71997184a62"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,7 +157,7 @@
     <x:numFmt numFmtId="201" formatCode="hh:mm"/>
     <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </x:numFmts>
-  <x:fonts count="19">
+  <x:fonts count="20">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -260,6 +260,11 @@
     <x:font>
       <x:sz val="9"/>
       <x:color rgb="FF98A2B3"/>
+      <x:name val="맑은 고딕"/>
+    </x:font>
+    <x:font>
+      <x:sz val="8"/>
+      <x:color rgb="FFC2C8D0"/>
       <x:name val="맑은 고딕"/>
     </x:font>
   </x:fonts>
@@ -551,7 +556,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="55">
+  <x:cellXfs count="56">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -681,6 +686,18 @@
     <x:xf numFmtId="200" fontId="18" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="176" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="176" fontId="7" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="176" fontId="12" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
@@ -692,15 +709,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="176" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="176" fontId="7" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="176" fontId="12" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -3415,6 +3423,15 @@
     <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="14" hidden="0" customWidth="1"/>
     <x:col min="20" max="20" width="11" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="9" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -3487,32 +3504,32 @@
         <x:v>파랑</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="17.25" customHeight="1">
-      <x:c r="B3" s="11" t="n">
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="B3" s="46" t="n">
         <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1</x:f>
         <x:v>46229</x:v>
       </x:c>
-      <x:c r="C3" s="12" t="n">
+      <x:c r="C3" s="47" t="n">
         <x:f t="shared" ref="C3:H3" si="0">B3+1</x:f>
         <x:v>46230</x:v>
       </x:c>
-      <x:c r="D3" s="12">
+      <x:c r="D3" s="47">
         <x:f t="shared" si="0"/>
         <x:v>46231</x:v>
       </x:c>
-      <x:c r="E3" s="12">
+      <x:c r="E3" s="47">
         <x:f t="shared" si="0"/>
         <x:v>46232</x:v>
       </x:c>
-      <x:c r="F3" s="12">
+      <x:c r="F3" s="47">
         <x:f t="shared" si="0"/>
         <x:v>46233</x:v>
       </x:c>
-      <x:c r="G3" s="12">
+      <x:c r="G3" s="47">
         <x:f t="shared" si="0"/>
         <x:v>46234</x:v>
       </x:c>
-      <x:c r="H3" s="22">
+      <x:c r="H3" s="48">
         <x:f t="shared" si="0"/>
         <x:v>46235</x:v>
       </x:c>
@@ -3525,27 +3542,27 @@
         <x:v>빨강</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="24" customHeight="1">
-      <x:c r="B4" s="45" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="C4" s="46" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="D4" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="E4" s="46" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="F4" s="46" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="G4" s="46" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="H4" s="48" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H3)*($Q$5:$Q$504=""),0),0)),"")</x:f>
+    <x:row r="4" ht="72" customHeight="1">
+      <x:c r="B4" s="49" t="str">
+        <x:f>XLOOKUP(B3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="C4" s="50" t="str">
+        <x:f>XLOOKUP(C3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="D4" s="51" t="str">
+        <x:f>XLOOKUP(D3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="E4" s="50" t="str">
+        <x:f>XLOOKUP(E3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="F4" s="50" t="str">
+        <x:f>XLOOKUP(F3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="G4" s="50" t="str">
+        <x:f>XLOOKUP(G3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="H4" s="52" t="str">
+        <x:f>XLOOKUP(H3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="I4" s="1"/>
       <x:c r="J4" s="30" t="str">
@@ -3572,6 +3589,9 @@
       <x:c r="Q4" s="30" t="str">
         <x:v>삭제시간</x:v>
       </x:c>
+      <x:c r="R4" s="45" t="str">
+        <x:v>내부 순번</x:v>
+      </x:c>
       <x:c r="S4" s="44" t="n">
         <x:f>IF(3&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,3),"")</x:f>
         <x:v>46237</x:v>
@@ -3579,33 +3599,36 @@
       <x:c r="T4" s="43" t="str">
         <x:v>초록</x:v>
       </x:c>
+      <x:c r="U4" s="45" t="str">
+        <x:v>내부 조회 키</x:v>
+      </x:c>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
-      <x:c r="B5" s="49" t="n">
+      <x:c r="B5" s="46" t="n">
         <x:f>H3+1</x:f>
         <x:v>46236</x:v>
       </x:c>
-      <x:c r="C5" s="50" t="n">
+      <x:c r="C5" s="47" t="n">
         <x:f t="shared" ref="C5:H5" si="1">B5+1</x:f>
         <x:v>46237</x:v>
       </x:c>
-      <x:c r="D5" s="50">
+      <x:c r="D5" s="47">
         <x:f t="shared" si="1"/>
         <x:v>46238</x:v>
       </x:c>
-      <x:c r="E5" s="50">
+      <x:c r="E5" s="47">
         <x:f t="shared" si="1"/>
         <x:v>46239</x:v>
       </x:c>
-      <x:c r="F5" s="50">
+      <x:c r="F5" s="47">
         <x:f t="shared" si="1"/>
         <x:v>46240</x:v>
       </x:c>
-      <x:c r="G5" s="50">
+      <x:c r="G5" s="47">
         <x:f t="shared" si="1"/>
         <x:v>46241</x:v>
       </x:c>
-      <x:c r="H5" s="51">
+      <x:c r="H5" s="48">
         <x:f t="shared" si="1"/>
         <x:v>46242</x:v>
       </x:c>
@@ -3618,6 +3641,9 @@
       <x:c r="O5" s="36" t="str"/>
       <x:c r="P5" s="39" t="str"/>
       <x:c r="Q5" s="39" t="str"/>
+      <x:c r="R5" s="45" t="str">
+        <x:f>IF(OR(J5="",Q5&lt;&gt;""),"",COUNTIF($J$5:J5,J5))</x:f>
+      </x:c>
       <x:c r="S5" s="44" t="n">
         <x:f>IF(4&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,4),"")</x:f>
         <x:v>46238</x:v>
@@ -3625,28 +3651,31 @@
       <x:c r="T5" s="43" t="str">
         <x:v>주황</x:v>
       </x:c>
-    </x:row>
-    <x:row r="6" ht="22" customHeight="1">
-      <x:c r="B6" s="45" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="C6" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="D6" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="E6" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="F6" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="G6" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="H6" s="48" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H5)*($Q$5:$Q$504=""),0),0)),"")</x:f>
+      <x:c r="U5" s="45" t="str">
+        <x:f>IF(OR(J5="",Q5&lt;&gt;""),"",J5&amp;"|"&amp;R5)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="72" customHeight="1">
+      <x:c r="B6" s="49" t="str">
+        <x:f>XLOOKUP(B5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="C6" s="51" t="str">
+        <x:f>XLOOKUP(C5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="D6" s="51" t="str">
+        <x:f>XLOOKUP(D5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="E6" s="51" t="str">
+        <x:f>XLOOKUP(E5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="F6" s="51" t="str">
+        <x:f>XLOOKUP(F5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="G6" s="51" t="str">
+        <x:f>XLOOKUP(G5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="H6" s="52" t="str">
+        <x:f>XLOOKUP(H5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="I6" s="1"/>
       <x:c r="J6" s="37" t="str"/>
@@ -3657,6 +3686,9 @@
       <x:c r="O6" s="36" t="str"/>
       <x:c r="P6" s="39" t="str"/>
       <x:c r="Q6" s="39" t="str"/>
+      <x:c r="R6" s="45" t="str">
+        <x:f>IF(OR(J6="",Q6&lt;&gt;""),"",COUNTIF($J$5:J6,J6))</x:f>
+      </x:c>
       <x:c r="S6" s="44" t="n">
         <x:f>IF(5&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,5),"")</x:f>
         <x:v>46239</x:v>
@@ -3664,33 +3696,36 @@
       <x:c r="T6" s="43" t="str">
         <x:v>보라</x:v>
       </x:c>
+      <x:c r="U6" s="45" t="str">
+        <x:f>IF(OR(J6="",Q6&lt;&gt;""),"",J6&amp;"|"&amp;R6)</x:f>
+      </x:c>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
-      <x:c r="B7" s="49" t="n">
+      <x:c r="B7" s="46" t="n">
         <x:f>H5+1</x:f>
         <x:v>46243</x:v>
       </x:c>
-      <x:c r="C7" s="50" t="n">
+      <x:c r="C7" s="47" t="n">
         <x:f t="shared" ref="C7:H7" si="2">B7+1</x:f>
         <x:v>46244</x:v>
       </x:c>
-      <x:c r="D7" s="50">
+      <x:c r="D7" s="47">
         <x:f t="shared" si="2"/>
         <x:v>46245</x:v>
       </x:c>
-      <x:c r="E7" s="50">
+      <x:c r="E7" s="47">
         <x:f t="shared" si="2"/>
         <x:v>46246</x:v>
       </x:c>
-      <x:c r="F7" s="50">
+      <x:c r="F7" s="47">
         <x:f t="shared" si="2"/>
         <x:v>46247</x:v>
       </x:c>
-      <x:c r="G7" s="50">
+      <x:c r="G7" s="47">
         <x:f t="shared" si="2"/>
         <x:v>46248</x:v>
       </x:c>
-      <x:c r="H7" s="51">
+      <x:c r="H7" s="48">
         <x:f t="shared" si="2"/>
         <x:v>46249</x:v>
       </x:c>
@@ -3703,6 +3738,9 @@
       <x:c r="O7" s="36" t="str"/>
       <x:c r="P7" s="39" t="str"/>
       <x:c r="Q7" s="39" t="str"/>
+      <x:c r="R7" s="45" t="str">
+        <x:f>IF(OR(J7="",Q7&lt;&gt;""),"",COUNTIF($J$5:J7,J7))</x:f>
+      </x:c>
       <x:c r="S7" s="44" t="n">
         <x:f>IF(6&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,6),"")</x:f>
         <x:v>46240</x:v>
@@ -3710,28 +3748,31 @@
       <x:c r="T7" s="43" t="str">
         <x:v>분홍</x:v>
       </x:c>
-    </x:row>
-    <x:row r="8" ht="22" customHeight="1">
-      <x:c r="B8" s="45" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="C8" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="D8" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="E8" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="F8" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="G8" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="H8" s="48" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H7)*($Q$5:$Q$504=""),0),0)),"")</x:f>
+      <x:c r="U7" s="45" t="str">
+        <x:f>IF(OR(J7="",Q7&lt;&gt;""),"",J7&amp;"|"&amp;R7)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="72" customHeight="1">
+      <x:c r="B8" s="49" t="str">
+        <x:f>XLOOKUP(B7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="C8" s="51" t="str">
+        <x:f>XLOOKUP(C7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="D8" s="51" t="str">
+        <x:f>XLOOKUP(D7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="E8" s="51" t="str">
+        <x:f>XLOOKUP(E7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="F8" s="51" t="str">
+        <x:f>XLOOKUP(F7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="G8" s="51" t="str">
+        <x:f>XLOOKUP(G7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="H8" s="52" t="str">
+        <x:f>XLOOKUP(H7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="I8" s="1"/>
       <x:c r="J8" s="37" t="str"/>
@@ -3742,6 +3783,9 @@
       <x:c r="O8" s="36" t="str"/>
       <x:c r="P8" s="39" t="str"/>
       <x:c r="Q8" s="39" t="str"/>
+      <x:c r="R8" s="45" t="str">
+        <x:f>IF(OR(J8="",Q8&lt;&gt;""),"",COUNTIF($J$5:J8,J8))</x:f>
+      </x:c>
       <x:c r="S8" s="44" t="n">
         <x:f>IF(7&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,7),"")</x:f>
         <x:v>46241</x:v>
@@ -3749,33 +3793,36 @@
       <x:c r="T8" s="43" t="str">
         <x:v>회색</x:v>
       </x:c>
+      <x:c r="U8" s="45" t="str">
+        <x:f>IF(OR(J8="",Q8&lt;&gt;""),"",J8&amp;"|"&amp;R8)</x:f>
+      </x:c>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
-      <x:c r="B9" s="49" t="n">
+      <x:c r="B9" s="46" t="n">
         <x:f>H7+1</x:f>
         <x:v>46250</x:v>
       </x:c>
-      <x:c r="C9" s="50" t="n">
+      <x:c r="C9" s="47" t="n">
         <x:f t="shared" ref="C9:H9" si="3">B9+1</x:f>
         <x:v>46251</x:v>
       </x:c>
-      <x:c r="D9" s="50">
+      <x:c r="D9" s="47">
         <x:f t="shared" si="3"/>
         <x:v>46252</x:v>
       </x:c>
-      <x:c r="E9" s="50">
+      <x:c r="E9" s="47">
         <x:f t="shared" si="3"/>
         <x:v>46253</x:v>
       </x:c>
-      <x:c r="F9" s="50">
+      <x:c r="F9" s="47">
         <x:f t="shared" si="3"/>
         <x:v>46254</x:v>
       </x:c>
-      <x:c r="G9" s="50">
+      <x:c r="G9" s="47">
         <x:f t="shared" si="3"/>
         <x:v>46255</x:v>
       </x:c>
-      <x:c r="H9" s="51">
+      <x:c r="H9" s="48">
         <x:f t="shared" si="3"/>
         <x:v>46256</x:v>
       </x:c>
@@ -3788,33 +3835,39 @@
       <x:c r="O9" s="36" t="str"/>
       <x:c r="P9" s="39" t="str"/>
       <x:c r="Q9" s="39" t="str"/>
+      <x:c r="R9" s="45" t="str">
+        <x:f>IF(OR(J9="",Q9&lt;&gt;""),"",COUNTIF($J$5:J9,J9))</x:f>
+      </x:c>
       <x:c r="S9" s="44" t="n">
         <x:f>IF(8&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,8),"")</x:f>
         <x:v>46242</x:v>
       </x:c>
       <x:c r="T9" s="43"/>
-    </x:row>
-    <x:row r="10" ht="22" customHeight="1">
-      <x:c r="B10" s="45" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="C10" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="D10" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="E10" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="F10" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="G10" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="H10" s="48" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H9)*($Q$5:$Q$504=""),0),0)),"")</x:f>
+      <x:c r="U9" s="45" t="str">
+        <x:f>IF(OR(J9="",Q9&lt;&gt;""),"",J9&amp;"|"&amp;R9)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="72" customHeight="1">
+      <x:c r="B10" s="49" t="str">
+        <x:f>XLOOKUP(B9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="C10" s="51" t="str">
+        <x:f>XLOOKUP(C9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="D10" s="51" t="str">
+        <x:f>XLOOKUP(D9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="E10" s="51" t="str">
+        <x:f>XLOOKUP(E9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="F10" s="51" t="str">
+        <x:f>XLOOKUP(F9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="G10" s="51" t="str">
+        <x:f>XLOOKUP(G9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="H10" s="52" t="str">
+        <x:f>XLOOKUP(H9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="I10" s="1"/>
       <x:c r="J10" s="37" t="str"/>
@@ -3825,38 +3878,44 @@
       <x:c r="O10" s="36" t="str"/>
       <x:c r="P10" s="39" t="str"/>
       <x:c r="Q10" s="39" t="str"/>
+      <x:c r="R10" s="45" t="str">
+        <x:f>IF(OR(J10="",Q10&lt;&gt;""),"",COUNTIF($J$5:J10,J10))</x:f>
+      </x:c>
       <x:c r="S10" s="44" t="n">
         <x:f>IF(9&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,9),"")</x:f>
         <x:v>46243</x:v>
       </x:c>
       <x:c r="T10" s="43"/>
+      <x:c r="U10" s="45" t="str">
+        <x:f>IF(OR(J10="",Q10&lt;&gt;""),"",J10&amp;"|"&amp;R10)</x:f>
+      </x:c>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
-      <x:c r="B11" s="49" t="n">
+      <x:c r="B11" s="46" t="n">
         <x:f>H9+1</x:f>
         <x:v>46257</x:v>
       </x:c>
-      <x:c r="C11" s="50" t="n">
+      <x:c r="C11" s="47" t="n">
         <x:f t="shared" ref="C11:H11" si="4">B11+1</x:f>
         <x:v>46258</x:v>
       </x:c>
-      <x:c r="D11" s="50">
+      <x:c r="D11" s="47">
         <x:f t="shared" si="4"/>
         <x:v>46259</x:v>
       </x:c>
-      <x:c r="E11" s="50">
+      <x:c r="E11" s="47">
         <x:f t="shared" si="4"/>
         <x:v>46260</x:v>
       </x:c>
-      <x:c r="F11" s="50">
+      <x:c r="F11" s="47">
         <x:f t="shared" si="4"/>
         <x:v>46261</x:v>
       </x:c>
-      <x:c r="G11" s="50">
+      <x:c r="G11" s="47">
         <x:f t="shared" si="4"/>
         <x:v>46262</x:v>
       </x:c>
-      <x:c r="H11" s="51">
+      <x:c r="H11" s="48">
         <x:f t="shared" si="4"/>
         <x:v>46263</x:v>
       </x:c>
@@ -3869,33 +3928,39 @@
       <x:c r="O11" s="36" t="str"/>
       <x:c r="P11" s="39" t="str"/>
       <x:c r="Q11" s="39" t="str"/>
+      <x:c r="R11" s="45" t="str">
+        <x:f>IF(OR(J11="",Q11&lt;&gt;""),"",COUNTIF($J$5:J11,J11))</x:f>
+      </x:c>
       <x:c r="S11" s="44" t="n">
         <x:f>IF(10&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,10),"")</x:f>
         <x:v>46244</x:v>
       </x:c>
       <x:c r="T11" s="43"/>
-    </x:row>
-    <x:row r="12" ht="22" customHeight="1">
-      <x:c r="B12" s="45" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="C12" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="D12" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="E12" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="F12" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="G12" s="47" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="H12" s="48" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H11)*($Q$5:$Q$504=""),0),0)),"")</x:f>
+      <x:c r="U11" s="45" t="str">
+        <x:f>IF(OR(J11="",Q11&lt;&gt;""),"",J11&amp;"|"&amp;R11)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="72" customHeight="1">
+      <x:c r="B12" s="49" t="str">
+        <x:f>XLOOKUP(B11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="C12" s="51" t="str">
+        <x:f>XLOOKUP(C11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="D12" s="51" t="str">
+        <x:f>XLOOKUP(D11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="E12" s="51" t="str">
+        <x:f>XLOOKUP(E11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="F12" s="51" t="str">
+        <x:f>XLOOKUP(F11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="G12" s="51" t="str">
+        <x:f>XLOOKUP(G11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="H12" s="52" t="str">
+        <x:f>XLOOKUP(H11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="I12" s="1"/>
       <x:c r="J12" s="37" t="str"/>
@@ -3906,38 +3971,44 @@
       <x:c r="O12" s="36" t="str"/>
       <x:c r="P12" s="39" t="str"/>
       <x:c r="Q12" s="39" t="str"/>
+      <x:c r="R12" s="45" t="str">
+        <x:f>IF(OR(J12="",Q12&lt;&gt;""),"",COUNTIF($J$5:J12,J12))</x:f>
+      </x:c>
       <x:c r="S12" s="44" t="n">
         <x:f>IF(11&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,11),"")</x:f>
         <x:v>46245</x:v>
       </x:c>
       <x:c r="T12" s="43"/>
+      <x:c r="U12" s="45" t="str">
+        <x:f>IF(OR(J12="",Q12&lt;&gt;""),"",J12&amp;"|"&amp;R12)</x:f>
+      </x:c>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
-      <x:c r="B13" s="49" t="n">
+      <x:c r="B13" s="46" t="n">
         <x:f>H11+1</x:f>
         <x:v>46264</x:v>
       </x:c>
-      <x:c r="C13" s="50" t="n">
+      <x:c r="C13" s="47" t="n">
         <x:f t="shared" ref="C13:H13" si="5">B13+1</x:f>
         <x:v>46265</x:v>
       </x:c>
-      <x:c r="D13" s="50">
+      <x:c r="D13" s="47">
         <x:f t="shared" si="5"/>
         <x:v>46266</x:v>
       </x:c>
-      <x:c r="E13" s="50">
+      <x:c r="E13" s="47">
         <x:f t="shared" si="5"/>
         <x:v>46267</x:v>
       </x:c>
-      <x:c r="F13" s="50">
+      <x:c r="F13" s="47">
         <x:f t="shared" si="5"/>
         <x:v>46268</x:v>
       </x:c>
-      <x:c r="G13" s="50">
+      <x:c r="G13" s="47">
         <x:f t="shared" si="5"/>
         <x:v>46269</x:v>
       </x:c>
-      <x:c r="H13" s="51">
+      <x:c r="H13" s="48">
         <x:f t="shared" si="5"/>
         <x:v>46270</x:v>
       </x:c>
@@ -3950,33 +4021,39 @@
       <x:c r="O13" s="36" t="str"/>
       <x:c r="P13" s="39" t="str"/>
       <x:c r="Q13" s="39" t="str"/>
+      <x:c r="R13" s="45" t="str">
+        <x:f>IF(OR(J13="",Q13&lt;&gt;""),"",COUNTIF($J$5:J13,J13))</x:f>
+      </x:c>
       <x:c r="S13" s="44" t="n">
         <x:f>IF(12&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,12),"")</x:f>
         <x:v>46246</x:v>
       </x:c>
       <x:c r="T13" s="43"/>
-    </x:row>
-    <x:row r="14" ht="22" customHeight="1">
-      <x:c r="B14" s="52" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=B13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="C14" s="53" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=C13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="D14" s="53" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=D13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="E14" s="53" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=E13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="F14" s="53" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=F13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="G14" s="53" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=G13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
-      </x:c>
-      <x:c r="H14" s="54" t="str">
-        <x:f>IFERROR(INDEX($K$5:$K$504,MATCH(1,INDEX(($J$5:$J$504=H13)*($Q$5:$Q$504=""),0),0)),"")</x:f>
+      <x:c r="U13" s="45" t="str">
+        <x:f>IF(OR(J13="",Q13&lt;&gt;""),"",J13&amp;"|"&amp;R13)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="72" customHeight="1">
+      <x:c r="B14" s="53" t="str">
+        <x:f>XLOOKUP(B13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="C14" s="54" t="str">
+        <x:f>XLOOKUP(C13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="D14" s="54" t="str">
+        <x:f>XLOOKUP(D13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="E14" s="54" t="str">
+        <x:f>XLOOKUP(E13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="F14" s="54" t="str">
+        <x:f>XLOOKUP(F13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="G14" s="54" t="str">
+        <x:f>XLOOKUP(G13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="H14" s="55" t="str">
+        <x:f>XLOOKUP(H13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="I14" s="2"/>
       <x:c r="J14" s="37" t="str"/>
@@ -3987,11 +4064,17 @@
       <x:c r="O14" s="36" t="str"/>
       <x:c r="P14" s="39" t="str"/>
       <x:c r="Q14" s="39" t="str"/>
+      <x:c r="R14" s="45" t="str">
+        <x:f>IF(OR(J14="",Q14&lt;&gt;""),"",COUNTIF($J$5:J14,J14))</x:f>
+      </x:c>
       <x:c r="S14" s="44" t="n">
         <x:f>IF(13&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,13),"")</x:f>
         <x:v>46247</x:v>
       </x:c>
       <x:c r="T14" s="43"/>
+      <x:c r="U14" s="45" t="str">
+        <x:f>IF(OR(J14="",Q14&lt;&gt;""),"",J14&amp;"|"&amp;R14)</x:f>
+      </x:c>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
       <x:c r="J15" s="37" t="str"/>
@@ -4002,11 +4085,17 @@
       <x:c r="O15" s="36" t="str"/>
       <x:c r="P15" s="39" t="str"/>
       <x:c r="Q15" s="39" t="str"/>
+      <x:c r="R15" s="45" t="str">
+        <x:f>IF(OR(J15="",Q15&lt;&gt;""),"",COUNTIF($J$5:J15,J15))</x:f>
+      </x:c>
       <x:c r="S15" s="44" t="n">
         <x:f>IF(14&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,14),"")</x:f>
         <x:v>46248</x:v>
       </x:c>
       <x:c r="T15" s="43"/>
+      <x:c r="U15" s="45" t="str">
+        <x:f>IF(OR(J15="",Q15&lt;&gt;""),"",J15&amp;"|"&amp;R15)</x:f>
+      </x:c>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="J16" s="37" t="str"/>
@@ -4017,11 +4106,17 @@
       <x:c r="O16" s="36" t="str"/>
       <x:c r="P16" s="39" t="str"/>
       <x:c r="Q16" s="39" t="str"/>
+      <x:c r="R16" s="45" t="str">
+        <x:f>IF(OR(J16="",Q16&lt;&gt;""),"",COUNTIF($J$5:J16,J16))</x:f>
+      </x:c>
       <x:c r="S16" s="44" t="n">
         <x:f>IF(15&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,15),"")</x:f>
         <x:v>46249</x:v>
       </x:c>
       <x:c r="T16" s="43"/>
+      <x:c r="U16" s="45" t="str">
+        <x:f>IF(OR(J16="",Q16&lt;&gt;""),"",J16&amp;"|"&amp;R16)</x:f>
+      </x:c>
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
       <x:c r="J17" s="37" t="str"/>
@@ -4032,11 +4127,17 @@
       <x:c r="O17" s="36" t="str"/>
       <x:c r="P17" s="39" t="str"/>
       <x:c r="Q17" s="39" t="str"/>
+      <x:c r="R17" s="45" t="str">
+        <x:f>IF(OR(J17="",Q17&lt;&gt;""),"",COUNTIF($J$5:J17,J17))</x:f>
+      </x:c>
       <x:c r="S17" s="44" t="n">
         <x:f>IF(16&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,16),"")</x:f>
         <x:v>46250</x:v>
       </x:c>
       <x:c r="T17" s="43"/>
+      <x:c r="U17" s="45" t="str">
+        <x:f>IF(OR(J17="",Q17&lt;&gt;""),"",J17&amp;"|"&amp;R17)</x:f>
+      </x:c>
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
       <x:c r="J18" s="37" t="str"/>
@@ -4047,11 +4148,17 @@
       <x:c r="O18" s="36" t="str"/>
       <x:c r="P18" s="39" t="str"/>
       <x:c r="Q18" s="39" t="str"/>
+      <x:c r="R18" s="45" t="str">
+        <x:f>IF(OR(J18="",Q18&lt;&gt;""),"",COUNTIF($J$5:J18,J18))</x:f>
+      </x:c>
       <x:c r="S18" s="44" t="n">
         <x:f>IF(17&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,17),"")</x:f>
         <x:v>46251</x:v>
       </x:c>
       <x:c r="T18" s="43"/>
+      <x:c r="U18" s="45" t="str">
+        <x:f>IF(OR(J18="",Q18&lt;&gt;""),"",J18&amp;"|"&amp;R18)</x:f>
+      </x:c>
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
       <x:c r="J19" s="37" t="str"/>
@@ -4062,11 +4169,17 @@
       <x:c r="O19" s="36" t="str"/>
       <x:c r="P19" s="39" t="str"/>
       <x:c r="Q19" s="39" t="str"/>
+      <x:c r="R19" s="45" t="str">
+        <x:f>IF(OR(J19="",Q19&lt;&gt;""),"",COUNTIF($J$5:J19,J19))</x:f>
+      </x:c>
       <x:c r="S19" s="44" t="n">
         <x:f>IF(18&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,18),"")</x:f>
         <x:v>46252</x:v>
       </x:c>
       <x:c r="T19" s="43"/>
+      <x:c r="U19" s="45" t="str">
+        <x:f>IF(OR(J19="",Q19&lt;&gt;""),"",J19&amp;"|"&amp;R19)</x:f>
+      </x:c>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
       <x:c r="J20" s="37" t="str"/>
@@ -4077,11 +4190,17 @@
       <x:c r="O20" s="36" t="str"/>
       <x:c r="P20" s="39" t="str"/>
       <x:c r="Q20" s="39" t="str"/>
+      <x:c r="R20" s="45" t="str">
+        <x:f>IF(OR(J20="",Q20&lt;&gt;""),"",COUNTIF($J$5:J20,J20))</x:f>
+      </x:c>
       <x:c r="S20" s="44" t="n">
         <x:f>IF(19&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,19),"")</x:f>
         <x:v>46253</x:v>
       </x:c>
       <x:c r="T20" s="43"/>
+      <x:c r="U20" s="45" t="str">
+        <x:f>IF(OR(J20="",Q20&lt;&gt;""),"",J20&amp;"|"&amp;R20)</x:f>
+      </x:c>
     </x:row>
     <x:row r="21" ht="22" customHeight="1">
       <x:c r="J21" s="37" t="str"/>
@@ -4092,11 +4211,17 @@
       <x:c r="O21" s="36" t="str"/>
       <x:c r="P21" s="39" t="str"/>
       <x:c r="Q21" s="39" t="str"/>
+      <x:c r="R21" s="45" t="str">
+        <x:f>IF(OR(J21="",Q21&lt;&gt;""),"",COUNTIF($J$5:J21,J21))</x:f>
+      </x:c>
       <x:c r="S21" s="44" t="n">
         <x:f>IF(20&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,20),"")</x:f>
         <x:v>46254</x:v>
       </x:c>
       <x:c r="T21" s="43"/>
+      <x:c r="U21" s="45" t="str">
+        <x:f>IF(OR(J21="",Q21&lt;&gt;""),"",J21&amp;"|"&amp;R21)</x:f>
+      </x:c>
     </x:row>
     <x:row r="22" ht="22" customHeight="1">
       <x:c r="J22" s="37" t="str"/>
@@ -4107,11 +4232,17 @@
       <x:c r="O22" s="36" t="str"/>
       <x:c r="P22" s="39" t="str"/>
       <x:c r="Q22" s="39" t="str"/>
+      <x:c r="R22" s="45" t="str">
+        <x:f>IF(OR(J22="",Q22&lt;&gt;""),"",COUNTIF($J$5:J22,J22))</x:f>
+      </x:c>
       <x:c r="S22" s="44" t="n">
         <x:f>IF(21&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,21),"")</x:f>
         <x:v>46255</x:v>
       </x:c>
       <x:c r="T22" s="43"/>
+      <x:c r="U22" s="45" t="str">
+        <x:f>IF(OR(J22="",Q22&lt;&gt;""),"",J22&amp;"|"&amp;R22)</x:f>
+      </x:c>
     </x:row>
     <x:row r="23" ht="22" customHeight="1">
       <x:c r="J23" s="37" t="str"/>
@@ -4122,11 +4253,17 @@
       <x:c r="O23" s="36" t="str"/>
       <x:c r="P23" s="39" t="str"/>
       <x:c r="Q23" s="39" t="str"/>
+      <x:c r="R23" s="45" t="str">
+        <x:f>IF(OR(J23="",Q23&lt;&gt;""),"",COUNTIF($J$5:J23,J23))</x:f>
+      </x:c>
       <x:c r="S23" s="44" t="n">
         <x:f>IF(22&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,22),"")</x:f>
         <x:v>46256</x:v>
       </x:c>
       <x:c r="T23" s="43"/>
+      <x:c r="U23" s="45" t="str">
+        <x:f>IF(OR(J23="",Q23&lt;&gt;""),"",J23&amp;"|"&amp;R23)</x:f>
+      </x:c>
     </x:row>
     <x:row r="24" ht="22" customHeight="1">
       <x:c r="J24" s="37" t="str"/>
@@ -4137,11 +4274,17 @@
       <x:c r="O24" s="36" t="str"/>
       <x:c r="P24" s="39" t="str"/>
       <x:c r="Q24" s="39" t="str"/>
+      <x:c r="R24" s="45" t="str">
+        <x:f>IF(OR(J24="",Q24&lt;&gt;""),"",COUNTIF($J$5:J24,J24))</x:f>
+      </x:c>
       <x:c r="S24" s="44" t="n">
         <x:f>IF(23&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,23),"")</x:f>
         <x:v>46257</x:v>
       </x:c>
       <x:c r="T24" s="43"/>
+      <x:c r="U24" s="45" t="str">
+        <x:f>IF(OR(J24="",Q24&lt;&gt;""),"",J24&amp;"|"&amp;R24)</x:f>
+      </x:c>
     </x:row>
     <x:row r="25" ht="22" customHeight="1">
       <x:c r="J25" s="37" t="str"/>
@@ -4152,11 +4295,17 @@
       <x:c r="O25" s="36" t="str"/>
       <x:c r="P25" s="39" t="str"/>
       <x:c r="Q25" s="39" t="str"/>
+      <x:c r="R25" s="45" t="str">
+        <x:f>IF(OR(J25="",Q25&lt;&gt;""),"",COUNTIF($J$5:J25,J25))</x:f>
+      </x:c>
       <x:c r="S25" s="44" t="n">
         <x:f>IF(24&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,24),"")</x:f>
         <x:v>46258</x:v>
       </x:c>
       <x:c r="T25" s="43"/>
+      <x:c r="U25" s="45" t="str">
+        <x:f>IF(OR(J25="",Q25&lt;&gt;""),"",J25&amp;"|"&amp;R25)</x:f>
+      </x:c>
     </x:row>
     <x:row r="26" ht="22" customHeight="1">
       <x:c r="J26" s="37" t="str"/>
@@ -4167,11 +4316,17 @@
       <x:c r="O26" s="36" t="str"/>
       <x:c r="P26" s="39" t="str"/>
       <x:c r="Q26" s="39" t="str"/>
+      <x:c r="R26" s="45" t="str">
+        <x:f>IF(OR(J26="",Q26&lt;&gt;""),"",COUNTIF($J$5:J26,J26))</x:f>
+      </x:c>
       <x:c r="S26" s="44" t="n">
         <x:f>IF(25&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,25),"")</x:f>
         <x:v>46259</x:v>
       </x:c>
       <x:c r="T26" s="43"/>
+      <x:c r="U26" s="45" t="str">
+        <x:f>IF(OR(J26="",Q26&lt;&gt;""),"",J26&amp;"|"&amp;R26)</x:f>
+      </x:c>
     </x:row>
     <x:row r="27" ht="22" customHeight="1">
       <x:c r="J27" s="37" t="str"/>
@@ -4182,11 +4337,17 @@
       <x:c r="O27" s="36" t="str"/>
       <x:c r="P27" s="39" t="str"/>
       <x:c r="Q27" s="39" t="str"/>
+      <x:c r="R27" s="45" t="str">
+        <x:f>IF(OR(J27="",Q27&lt;&gt;""),"",COUNTIF($J$5:J27,J27))</x:f>
+      </x:c>
       <x:c r="S27" s="44" t="n">
         <x:f>IF(26&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,26),"")</x:f>
         <x:v>46260</x:v>
       </x:c>
       <x:c r="T27" s="43"/>
+      <x:c r="U27" s="45" t="str">
+        <x:f>IF(OR(J27="",Q27&lt;&gt;""),"",J27&amp;"|"&amp;R27)</x:f>
+      </x:c>
     </x:row>
     <x:row r="28" ht="22" customHeight="1">
       <x:c r="J28" s="37" t="str"/>
@@ -4197,11 +4358,17 @@
       <x:c r="O28" s="36" t="str"/>
       <x:c r="P28" s="39" t="str"/>
       <x:c r="Q28" s="39" t="str"/>
+      <x:c r="R28" s="45" t="str">
+        <x:f>IF(OR(J28="",Q28&lt;&gt;""),"",COUNTIF($J$5:J28,J28))</x:f>
+      </x:c>
       <x:c r="S28" s="44" t="n">
         <x:f>IF(27&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,27),"")</x:f>
         <x:v>46261</x:v>
       </x:c>
       <x:c r="T28" s="43"/>
+      <x:c r="U28" s="45" t="str">
+        <x:f>IF(OR(J28="",Q28&lt;&gt;""),"",J28&amp;"|"&amp;R28)</x:f>
+      </x:c>
     </x:row>
     <x:row r="29" ht="22" customHeight="1">
       <x:c r="J29" s="37" t="str"/>
@@ -4212,11 +4379,17 @@
       <x:c r="O29" s="36" t="str"/>
       <x:c r="P29" s="39" t="str"/>
       <x:c r="Q29" s="39" t="str"/>
+      <x:c r="R29" s="45" t="str">
+        <x:f>IF(OR(J29="",Q29&lt;&gt;""),"",COUNTIF($J$5:J29,J29))</x:f>
+      </x:c>
       <x:c r="S29" s="44" t="n">
         <x:f>IF(28&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,28),"")</x:f>
         <x:v>46262</x:v>
       </x:c>
       <x:c r="T29" s="43"/>
+      <x:c r="U29" s="45" t="str">
+        <x:f>IF(OR(J29="",Q29&lt;&gt;""),"",J29&amp;"|"&amp;R29)</x:f>
+      </x:c>
     </x:row>
     <x:row r="30" ht="22" customHeight="1">
       <x:c r="J30" s="37" t="str"/>
@@ -4227,11 +4400,17 @@
       <x:c r="O30" s="36" t="str"/>
       <x:c r="P30" s="39" t="str"/>
       <x:c r="Q30" s="39" t="str"/>
+      <x:c r="R30" s="45" t="str">
+        <x:f>IF(OR(J30="",Q30&lt;&gt;""),"",COUNTIF($J$5:J30,J30))</x:f>
+      </x:c>
       <x:c r="S30" s="44" t="n">
         <x:f>IF(29&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,29),"")</x:f>
         <x:v>46263</x:v>
       </x:c>
       <x:c r="T30" s="43"/>
+      <x:c r="U30" s="45" t="str">
+        <x:f>IF(OR(J30="",Q30&lt;&gt;""),"",J30&amp;"|"&amp;R30)</x:f>
+      </x:c>
     </x:row>
     <x:row r="31" ht="22" customHeight="1">
       <x:c r="J31" s="37" t="str"/>
@@ -4242,11 +4421,17 @@
       <x:c r="O31" s="36" t="str"/>
       <x:c r="P31" s="39" t="str"/>
       <x:c r="Q31" s="39" t="str"/>
+      <x:c r="R31" s="45" t="str">
+        <x:f>IF(OR(J31="",Q31&lt;&gt;""),"",COUNTIF($J$5:J31,J31))</x:f>
+      </x:c>
       <x:c r="S31" s="44" t="n">
         <x:f>IF(30&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,30),"")</x:f>
         <x:v>46264</x:v>
       </x:c>
       <x:c r="T31" s="43"/>
+      <x:c r="U31" s="45" t="str">
+        <x:f>IF(OR(J31="",Q31&lt;&gt;""),"",J31&amp;"|"&amp;R31)</x:f>
+      </x:c>
     </x:row>
     <x:row r="32" ht="22" customHeight="1">
       <x:c r="J32" s="37" t="str"/>
@@ -4257,11 +4442,17 @@
       <x:c r="O32" s="36" t="str"/>
       <x:c r="P32" s="39" t="str"/>
       <x:c r="Q32" s="39" t="str"/>
+      <x:c r="R32" s="45" t="str">
+        <x:f>IF(OR(J32="",Q32&lt;&gt;""),"",COUNTIF($J$5:J32,J32))</x:f>
+      </x:c>
       <x:c r="S32" s="44" t="n">
         <x:f>IF(31&lt;=DAY(EOMONTH(DATE($G$1,$H$1,1),0)),DATE($G$1,$H$1,31),"")</x:f>
         <x:v>46265</x:v>
       </x:c>
       <x:c r="T32" s="43"/>
+      <x:c r="U32" s="45" t="str">
+        <x:f>IF(OR(J32="",Q32&lt;&gt;""),"",J32&amp;"|"&amp;R32)</x:f>
+      </x:c>
     </x:row>
     <x:row r="33" ht="22" customHeight="1">
       <x:c r="J33" s="37" t="str"/>
@@ -4272,6 +4463,12 @@
       <x:c r="O33" s="36" t="str"/>
       <x:c r="P33" s="39" t="str"/>
       <x:c r="Q33" s="39" t="str"/>
+      <x:c r="R33" s="45" t="str">
+        <x:f>IF(OR(J33="",Q33&lt;&gt;""),"",COUNTIF($J$5:J33,J33))</x:f>
+      </x:c>
+      <x:c r="U33" s="45" t="str">
+        <x:f>IF(OR(J33="",Q33&lt;&gt;""),"",J33&amp;"|"&amp;R33)</x:f>
+      </x:c>
     </x:row>
     <x:row r="34" ht="22" customHeight="1">
       <x:c r="J34" s="37" t="str"/>
@@ -4282,6 +4479,3772 @@
       <x:c r="O34" s="36" t="str"/>
       <x:c r="P34" s="39" t="str"/>
       <x:c r="Q34" s="39" t="str"/>
+      <x:c r="R34" s="45" t="str">
+        <x:f>IF(OR(J34="",Q34&lt;&gt;""),"",COUNTIF($J$5:J34,J34))</x:f>
+      </x:c>
+      <x:c r="U34" s="45" t="str">
+        <x:f>IF(OR(J34="",Q34&lt;&gt;""),"",J34&amp;"|"&amp;R34)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="R35" s="45" t="str">
+        <x:f>IF(OR(J35="",Q35&lt;&gt;""),"",COUNTIF($J$5:J35,J35))</x:f>
+      </x:c>
+      <x:c r="U35" s="45" t="str">
+        <x:f>IF(OR(J35="",Q35&lt;&gt;""),"",J35&amp;"|"&amp;R35)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="R36" s="45" t="str">
+        <x:f>IF(OR(J36="",Q36&lt;&gt;""),"",COUNTIF($J$5:J36,J36))</x:f>
+      </x:c>
+      <x:c r="U36" s="45" t="str">
+        <x:f>IF(OR(J36="",Q36&lt;&gt;""),"",J36&amp;"|"&amp;R36)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="R37" s="45" t="str">
+        <x:f>IF(OR(J37="",Q37&lt;&gt;""),"",COUNTIF($J$5:J37,J37))</x:f>
+      </x:c>
+      <x:c r="U37" s="45" t="str">
+        <x:f>IF(OR(J37="",Q37&lt;&gt;""),"",J37&amp;"|"&amp;R37)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="R38" s="45" t="str">
+        <x:f>IF(OR(J38="",Q38&lt;&gt;""),"",COUNTIF($J$5:J38,J38))</x:f>
+      </x:c>
+      <x:c r="U38" s="45" t="str">
+        <x:f>IF(OR(J38="",Q38&lt;&gt;""),"",J38&amp;"|"&amp;R38)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="R39" s="45" t="str">
+        <x:f>IF(OR(J39="",Q39&lt;&gt;""),"",COUNTIF($J$5:J39,J39))</x:f>
+      </x:c>
+      <x:c r="U39" s="45" t="str">
+        <x:f>IF(OR(J39="",Q39&lt;&gt;""),"",J39&amp;"|"&amp;R39)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="R40" s="45" t="str">
+        <x:f>IF(OR(J40="",Q40&lt;&gt;""),"",COUNTIF($J$5:J40,J40))</x:f>
+      </x:c>
+      <x:c r="U40" s="45" t="str">
+        <x:f>IF(OR(J40="",Q40&lt;&gt;""),"",J40&amp;"|"&amp;R40)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="R41" s="45" t="str">
+        <x:f>IF(OR(J41="",Q41&lt;&gt;""),"",COUNTIF($J$5:J41,J41))</x:f>
+      </x:c>
+      <x:c r="U41" s="45" t="str">
+        <x:f>IF(OR(J41="",Q41&lt;&gt;""),"",J41&amp;"|"&amp;R41)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="R42" s="45" t="str">
+        <x:f>IF(OR(J42="",Q42&lt;&gt;""),"",COUNTIF($J$5:J42,J42))</x:f>
+      </x:c>
+      <x:c r="U42" s="45" t="str">
+        <x:f>IF(OR(J42="",Q42&lt;&gt;""),"",J42&amp;"|"&amp;R42)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="R43" s="45" t="str">
+        <x:f>IF(OR(J43="",Q43&lt;&gt;""),"",COUNTIF($J$5:J43,J43))</x:f>
+      </x:c>
+      <x:c r="U43" s="45" t="str">
+        <x:f>IF(OR(J43="",Q43&lt;&gt;""),"",J43&amp;"|"&amp;R43)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="R44" s="45" t="str">
+        <x:f>IF(OR(J44="",Q44&lt;&gt;""),"",COUNTIF($J$5:J44,J44))</x:f>
+      </x:c>
+      <x:c r="U44" s="45" t="str">
+        <x:f>IF(OR(J44="",Q44&lt;&gt;""),"",J44&amp;"|"&amp;R44)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="R45" s="45" t="str">
+        <x:f>IF(OR(J45="",Q45&lt;&gt;""),"",COUNTIF($J$5:J45,J45))</x:f>
+      </x:c>
+      <x:c r="U45" s="45" t="str">
+        <x:f>IF(OR(J45="",Q45&lt;&gt;""),"",J45&amp;"|"&amp;R45)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="R46" s="45" t="str">
+        <x:f>IF(OR(J46="",Q46&lt;&gt;""),"",COUNTIF($J$5:J46,J46))</x:f>
+      </x:c>
+      <x:c r="U46" s="45" t="str">
+        <x:f>IF(OR(J46="",Q46&lt;&gt;""),"",J46&amp;"|"&amp;R46)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="R47" s="45" t="str">
+        <x:f>IF(OR(J47="",Q47&lt;&gt;""),"",COUNTIF($J$5:J47,J47))</x:f>
+      </x:c>
+      <x:c r="U47" s="45" t="str">
+        <x:f>IF(OR(J47="",Q47&lt;&gt;""),"",J47&amp;"|"&amp;R47)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="R48" s="45" t="str">
+        <x:f>IF(OR(J48="",Q48&lt;&gt;""),"",COUNTIF($J$5:J48,J48))</x:f>
+      </x:c>
+      <x:c r="U48" s="45" t="str">
+        <x:f>IF(OR(J48="",Q48&lt;&gt;""),"",J48&amp;"|"&amp;R48)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="R49" s="45" t="str">
+        <x:f>IF(OR(J49="",Q49&lt;&gt;""),"",COUNTIF($J$5:J49,J49))</x:f>
+      </x:c>
+      <x:c r="U49" s="45" t="str">
+        <x:f>IF(OR(J49="",Q49&lt;&gt;""),"",J49&amp;"|"&amp;R49)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="R50" s="45" t="str">
+        <x:f>IF(OR(J50="",Q50&lt;&gt;""),"",COUNTIF($J$5:J50,J50))</x:f>
+      </x:c>
+      <x:c r="U50" s="45" t="str">
+        <x:f>IF(OR(J50="",Q50&lt;&gt;""),"",J50&amp;"|"&amp;R50)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="R51" s="45" t="str">
+        <x:f>IF(OR(J51="",Q51&lt;&gt;""),"",COUNTIF($J$5:J51,J51))</x:f>
+      </x:c>
+      <x:c r="U51" s="45" t="str">
+        <x:f>IF(OR(J51="",Q51&lt;&gt;""),"",J51&amp;"|"&amp;R51)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="R52" s="45" t="str">
+        <x:f>IF(OR(J52="",Q52&lt;&gt;""),"",COUNTIF($J$5:J52,J52))</x:f>
+      </x:c>
+      <x:c r="U52" s="45" t="str">
+        <x:f>IF(OR(J52="",Q52&lt;&gt;""),"",J52&amp;"|"&amp;R52)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="R53" s="45" t="str">
+        <x:f>IF(OR(J53="",Q53&lt;&gt;""),"",COUNTIF($J$5:J53,J53))</x:f>
+      </x:c>
+      <x:c r="U53" s="45" t="str">
+        <x:f>IF(OR(J53="",Q53&lt;&gt;""),"",J53&amp;"|"&amp;R53)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="R54" s="45" t="str">
+        <x:f>IF(OR(J54="",Q54&lt;&gt;""),"",COUNTIF($J$5:J54,J54))</x:f>
+      </x:c>
+      <x:c r="U54" s="45" t="str">
+        <x:f>IF(OR(J54="",Q54&lt;&gt;""),"",J54&amp;"|"&amp;R54)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="R55" s="45" t="str">
+        <x:f>IF(OR(J55="",Q55&lt;&gt;""),"",COUNTIF($J$5:J55,J55))</x:f>
+      </x:c>
+      <x:c r="U55" s="45" t="str">
+        <x:f>IF(OR(J55="",Q55&lt;&gt;""),"",J55&amp;"|"&amp;R55)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="R56" s="45" t="str">
+        <x:f>IF(OR(J56="",Q56&lt;&gt;""),"",COUNTIF($J$5:J56,J56))</x:f>
+      </x:c>
+      <x:c r="U56" s="45" t="str">
+        <x:f>IF(OR(J56="",Q56&lt;&gt;""),"",J56&amp;"|"&amp;R56)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="R57" s="45" t="str">
+        <x:f>IF(OR(J57="",Q57&lt;&gt;""),"",COUNTIF($J$5:J57,J57))</x:f>
+      </x:c>
+      <x:c r="U57" s="45" t="str">
+        <x:f>IF(OR(J57="",Q57&lt;&gt;""),"",J57&amp;"|"&amp;R57)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="R58" s="45" t="str">
+        <x:f>IF(OR(J58="",Q58&lt;&gt;""),"",COUNTIF($J$5:J58,J58))</x:f>
+      </x:c>
+      <x:c r="U58" s="45" t="str">
+        <x:f>IF(OR(J58="",Q58&lt;&gt;""),"",J58&amp;"|"&amp;R58)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="R59" s="45" t="str">
+        <x:f>IF(OR(J59="",Q59&lt;&gt;""),"",COUNTIF($J$5:J59,J59))</x:f>
+      </x:c>
+      <x:c r="U59" s="45" t="str">
+        <x:f>IF(OR(J59="",Q59&lt;&gt;""),"",J59&amp;"|"&amp;R59)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="R60" s="45" t="str">
+        <x:f>IF(OR(J60="",Q60&lt;&gt;""),"",COUNTIF($J$5:J60,J60))</x:f>
+      </x:c>
+      <x:c r="U60" s="45" t="str">
+        <x:f>IF(OR(J60="",Q60&lt;&gt;""),"",J60&amp;"|"&amp;R60)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="R61" s="45" t="str">
+        <x:f>IF(OR(J61="",Q61&lt;&gt;""),"",COUNTIF($J$5:J61,J61))</x:f>
+      </x:c>
+      <x:c r="U61" s="45" t="str">
+        <x:f>IF(OR(J61="",Q61&lt;&gt;""),"",J61&amp;"|"&amp;R61)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="R62" s="45" t="str">
+        <x:f>IF(OR(J62="",Q62&lt;&gt;""),"",COUNTIF($J$5:J62,J62))</x:f>
+      </x:c>
+      <x:c r="U62" s="45" t="str">
+        <x:f>IF(OR(J62="",Q62&lt;&gt;""),"",J62&amp;"|"&amp;R62)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="R63" s="45" t="str">
+        <x:f>IF(OR(J63="",Q63&lt;&gt;""),"",COUNTIF($J$5:J63,J63))</x:f>
+      </x:c>
+      <x:c r="U63" s="45" t="str">
+        <x:f>IF(OR(J63="",Q63&lt;&gt;""),"",J63&amp;"|"&amp;R63)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="R64" s="45" t="str">
+        <x:f>IF(OR(J64="",Q64&lt;&gt;""),"",COUNTIF($J$5:J64,J64))</x:f>
+      </x:c>
+      <x:c r="U64" s="45" t="str">
+        <x:f>IF(OR(J64="",Q64&lt;&gt;""),"",J64&amp;"|"&amp;R64)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="R65" s="45" t="str">
+        <x:f>IF(OR(J65="",Q65&lt;&gt;""),"",COUNTIF($J$5:J65,J65))</x:f>
+      </x:c>
+      <x:c r="U65" s="45" t="str">
+        <x:f>IF(OR(J65="",Q65&lt;&gt;""),"",J65&amp;"|"&amp;R65)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="R66" s="45" t="str">
+        <x:f>IF(OR(J66="",Q66&lt;&gt;""),"",COUNTIF($J$5:J66,J66))</x:f>
+      </x:c>
+      <x:c r="U66" s="45" t="str">
+        <x:f>IF(OR(J66="",Q66&lt;&gt;""),"",J66&amp;"|"&amp;R66)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="R67" s="45" t="str">
+        <x:f>IF(OR(J67="",Q67&lt;&gt;""),"",COUNTIF($J$5:J67,J67))</x:f>
+      </x:c>
+      <x:c r="U67" s="45" t="str">
+        <x:f>IF(OR(J67="",Q67&lt;&gt;""),"",J67&amp;"|"&amp;R67)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="R68" s="45" t="str">
+        <x:f>IF(OR(J68="",Q68&lt;&gt;""),"",COUNTIF($J$5:J68,J68))</x:f>
+      </x:c>
+      <x:c r="U68" s="45" t="str">
+        <x:f>IF(OR(J68="",Q68&lt;&gt;""),"",J68&amp;"|"&amp;R68)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="R69" s="45" t="str">
+        <x:f>IF(OR(J69="",Q69&lt;&gt;""),"",COUNTIF($J$5:J69,J69))</x:f>
+      </x:c>
+      <x:c r="U69" s="45" t="str">
+        <x:f>IF(OR(J69="",Q69&lt;&gt;""),"",J69&amp;"|"&amp;R69)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="R70" s="45" t="str">
+        <x:f>IF(OR(J70="",Q70&lt;&gt;""),"",COUNTIF($J$5:J70,J70))</x:f>
+      </x:c>
+      <x:c r="U70" s="45" t="str">
+        <x:f>IF(OR(J70="",Q70&lt;&gt;""),"",J70&amp;"|"&amp;R70)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="R71" s="45" t="str">
+        <x:f>IF(OR(J71="",Q71&lt;&gt;""),"",COUNTIF($J$5:J71,J71))</x:f>
+      </x:c>
+      <x:c r="U71" s="45" t="str">
+        <x:f>IF(OR(J71="",Q71&lt;&gt;""),"",J71&amp;"|"&amp;R71)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="R72" s="45" t="str">
+        <x:f>IF(OR(J72="",Q72&lt;&gt;""),"",COUNTIF($J$5:J72,J72))</x:f>
+      </x:c>
+      <x:c r="U72" s="45" t="str">
+        <x:f>IF(OR(J72="",Q72&lt;&gt;""),"",J72&amp;"|"&amp;R72)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="R73" s="45" t="str">
+        <x:f>IF(OR(J73="",Q73&lt;&gt;""),"",COUNTIF($J$5:J73,J73))</x:f>
+      </x:c>
+      <x:c r="U73" s="45" t="str">
+        <x:f>IF(OR(J73="",Q73&lt;&gt;""),"",J73&amp;"|"&amp;R73)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="R74" s="45" t="str">
+        <x:f>IF(OR(J74="",Q74&lt;&gt;""),"",COUNTIF($J$5:J74,J74))</x:f>
+      </x:c>
+      <x:c r="U74" s="45" t="str">
+        <x:f>IF(OR(J74="",Q74&lt;&gt;""),"",J74&amp;"|"&amp;R74)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="R75" s="45" t="str">
+        <x:f>IF(OR(J75="",Q75&lt;&gt;""),"",COUNTIF($J$5:J75,J75))</x:f>
+      </x:c>
+      <x:c r="U75" s="45" t="str">
+        <x:f>IF(OR(J75="",Q75&lt;&gt;""),"",J75&amp;"|"&amp;R75)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="R76" s="45" t="str">
+        <x:f>IF(OR(J76="",Q76&lt;&gt;""),"",COUNTIF($J$5:J76,J76))</x:f>
+      </x:c>
+      <x:c r="U76" s="45" t="str">
+        <x:f>IF(OR(J76="",Q76&lt;&gt;""),"",J76&amp;"|"&amp;R76)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="R77" s="45" t="str">
+        <x:f>IF(OR(J77="",Q77&lt;&gt;""),"",COUNTIF($J$5:J77,J77))</x:f>
+      </x:c>
+      <x:c r="U77" s="45" t="str">
+        <x:f>IF(OR(J77="",Q77&lt;&gt;""),"",J77&amp;"|"&amp;R77)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="R78" s="45" t="str">
+        <x:f>IF(OR(J78="",Q78&lt;&gt;""),"",COUNTIF($J$5:J78,J78))</x:f>
+      </x:c>
+      <x:c r="U78" s="45" t="str">
+        <x:f>IF(OR(J78="",Q78&lt;&gt;""),"",J78&amp;"|"&amp;R78)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="R79" s="45" t="str">
+        <x:f>IF(OR(J79="",Q79&lt;&gt;""),"",COUNTIF($J$5:J79,J79))</x:f>
+      </x:c>
+      <x:c r="U79" s="45" t="str">
+        <x:f>IF(OR(J79="",Q79&lt;&gt;""),"",J79&amp;"|"&amp;R79)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="R80" s="45" t="str">
+        <x:f>IF(OR(J80="",Q80&lt;&gt;""),"",COUNTIF($J$5:J80,J80))</x:f>
+      </x:c>
+      <x:c r="U80" s="45" t="str">
+        <x:f>IF(OR(J80="",Q80&lt;&gt;""),"",J80&amp;"|"&amp;R80)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="R81" s="45" t="str">
+        <x:f>IF(OR(J81="",Q81&lt;&gt;""),"",COUNTIF($J$5:J81,J81))</x:f>
+      </x:c>
+      <x:c r="U81" s="45" t="str">
+        <x:f>IF(OR(J81="",Q81&lt;&gt;""),"",J81&amp;"|"&amp;R81)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="R82" s="45" t="str">
+        <x:f>IF(OR(J82="",Q82&lt;&gt;""),"",COUNTIF($J$5:J82,J82))</x:f>
+      </x:c>
+      <x:c r="U82" s="45" t="str">
+        <x:f>IF(OR(J82="",Q82&lt;&gt;""),"",J82&amp;"|"&amp;R82)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="R83" s="45" t="str">
+        <x:f>IF(OR(J83="",Q83&lt;&gt;""),"",COUNTIF($J$5:J83,J83))</x:f>
+      </x:c>
+      <x:c r="U83" s="45" t="str">
+        <x:f>IF(OR(J83="",Q83&lt;&gt;""),"",J83&amp;"|"&amp;R83)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="R84" s="45" t="str">
+        <x:f>IF(OR(J84="",Q84&lt;&gt;""),"",COUNTIF($J$5:J84,J84))</x:f>
+      </x:c>
+      <x:c r="U84" s="45" t="str">
+        <x:f>IF(OR(J84="",Q84&lt;&gt;""),"",J84&amp;"|"&amp;R84)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="R85" s="45" t="str">
+        <x:f>IF(OR(J85="",Q85&lt;&gt;""),"",COUNTIF($J$5:J85,J85))</x:f>
+      </x:c>
+      <x:c r="U85" s="45" t="str">
+        <x:f>IF(OR(J85="",Q85&lt;&gt;""),"",J85&amp;"|"&amp;R85)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="R86" s="45" t="str">
+        <x:f>IF(OR(J86="",Q86&lt;&gt;""),"",COUNTIF($J$5:J86,J86))</x:f>
+      </x:c>
+      <x:c r="U86" s="45" t="str">
+        <x:f>IF(OR(J86="",Q86&lt;&gt;""),"",J86&amp;"|"&amp;R86)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="R87" s="45" t="str">
+        <x:f>IF(OR(J87="",Q87&lt;&gt;""),"",COUNTIF($J$5:J87,J87))</x:f>
+      </x:c>
+      <x:c r="U87" s="45" t="str">
+        <x:f>IF(OR(J87="",Q87&lt;&gt;""),"",J87&amp;"|"&amp;R87)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="R88" s="45" t="str">
+        <x:f>IF(OR(J88="",Q88&lt;&gt;""),"",COUNTIF($J$5:J88,J88))</x:f>
+      </x:c>
+      <x:c r="U88" s="45" t="str">
+        <x:f>IF(OR(J88="",Q88&lt;&gt;""),"",J88&amp;"|"&amp;R88)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="R89" s="45" t="str">
+        <x:f>IF(OR(J89="",Q89&lt;&gt;""),"",COUNTIF($J$5:J89,J89))</x:f>
+      </x:c>
+      <x:c r="U89" s="45" t="str">
+        <x:f>IF(OR(J89="",Q89&lt;&gt;""),"",J89&amp;"|"&amp;R89)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="R90" s="45" t="str">
+        <x:f>IF(OR(J90="",Q90&lt;&gt;""),"",COUNTIF($J$5:J90,J90))</x:f>
+      </x:c>
+      <x:c r="U90" s="45" t="str">
+        <x:f>IF(OR(J90="",Q90&lt;&gt;""),"",J90&amp;"|"&amp;R90)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="R91" s="45" t="str">
+        <x:f>IF(OR(J91="",Q91&lt;&gt;""),"",COUNTIF($J$5:J91,J91))</x:f>
+      </x:c>
+      <x:c r="U91" s="45" t="str">
+        <x:f>IF(OR(J91="",Q91&lt;&gt;""),"",J91&amp;"|"&amp;R91)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="R92" s="45" t="str">
+        <x:f>IF(OR(J92="",Q92&lt;&gt;""),"",COUNTIF($J$5:J92,J92))</x:f>
+      </x:c>
+      <x:c r="U92" s="45" t="str">
+        <x:f>IF(OR(J92="",Q92&lt;&gt;""),"",J92&amp;"|"&amp;R92)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="R93" s="45" t="str">
+        <x:f>IF(OR(J93="",Q93&lt;&gt;""),"",COUNTIF($J$5:J93,J93))</x:f>
+      </x:c>
+      <x:c r="U93" s="45" t="str">
+        <x:f>IF(OR(J93="",Q93&lt;&gt;""),"",J93&amp;"|"&amp;R93)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="R94" s="45" t="str">
+        <x:f>IF(OR(J94="",Q94&lt;&gt;""),"",COUNTIF($J$5:J94,J94))</x:f>
+      </x:c>
+      <x:c r="U94" s="45" t="str">
+        <x:f>IF(OR(J94="",Q94&lt;&gt;""),"",J94&amp;"|"&amp;R94)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="R95" s="45" t="str">
+        <x:f>IF(OR(J95="",Q95&lt;&gt;""),"",COUNTIF($J$5:J95,J95))</x:f>
+      </x:c>
+      <x:c r="U95" s="45" t="str">
+        <x:f>IF(OR(J95="",Q95&lt;&gt;""),"",J95&amp;"|"&amp;R95)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="R96" s="45" t="str">
+        <x:f>IF(OR(J96="",Q96&lt;&gt;""),"",COUNTIF($J$5:J96,J96))</x:f>
+      </x:c>
+      <x:c r="U96" s="45" t="str">
+        <x:f>IF(OR(J96="",Q96&lt;&gt;""),"",J96&amp;"|"&amp;R96)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="R97" s="45" t="str">
+        <x:f>IF(OR(J97="",Q97&lt;&gt;""),"",COUNTIF($J$5:J97,J97))</x:f>
+      </x:c>
+      <x:c r="U97" s="45" t="str">
+        <x:f>IF(OR(J97="",Q97&lt;&gt;""),"",J97&amp;"|"&amp;R97)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="R98" s="45" t="str">
+        <x:f>IF(OR(J98="",Q98&lt;&gt;""),"",COUNTIF($J$5:J98,J98))</x:f>
+      </x:c>
+      <x:c r="U98" s="45" t="str">
+        <x:f>IF(OR(J98="",Q98&lt;&gt;""),"",J98&amp;"|"&amp;R98)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="R99" s="45" t="str">
+        <x:f>IF(OR(J99="",Q99&lt;&gt;""),"",COUNTIF($J$5:J99,J99))</x:f>
+      </x:c>
+      <x:c r="U99" s="45" t="str">
+        <x:f>IF(OR(J99="",Q99&lt;&gt;""),"",J99&amp;"|"&amp;R99)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="R100" s="45" t="str">
+        <x:f>IF(OR(J100="",Q100&lt;&gt;""),"",COUNTIF($J$5:J100,J100))</x:f>
+      </x:c>
+      <x:c r="U100" s="45" t="str">
+        <x:f>IF(OR(J100="",Q100&lt;&gt;""),"",J100&amp;"|"&amp;R100)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="R101" s="45" t="str">
+        <x:f>IF(OR(J101="",Q101&lt;&gt;""),"",COUNTIF($J$5:J101,J101))</x:f>
+      </x:c>
+      <x:c r="U101" s="45" t="str">
+        <x:f>IF(OR(J101="",Q101&lt;&gt;""),"",J101&amp;"|"&amp;R101)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="102">
+      <x:c r="R102" s="45" t="str">
+        <x:f>IF(OR(J102="",Q102&lt;&gt;""),"",COUNTIF($J$5:J102,J102))</x:f>
+      </x:c>
+      <x:c r="U102" s="45" t="str">
+        <x:f>IF(OR(J102="",Q102&lt;&gt;""),"",J102&amp;"|"&amp;R102)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="103">
+      <x:c r="R103" s="45" t="str">
+        <x:f>IF(OR(J103="",Q103&lt;&gt;""),"",COUNTIF($J$5:J103,J103))</x:f>
+      </x:c>
+      <x:c r="U103" s="45" t="str">
+        <x:f>IF(OR(J103="",Q103&lt;&gt;""),"",J103&amp;"|"&amp;R103)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="R104" s="45" t="str">
+        <x:f>IF(OR(J104="",Q104&lt;&gt;""),"",COUNTIF($J$5:J104,J104))</x:f>
+      </x:c>
+      <x:c r="U104" s="45" t="str">
+        <x:f>IF(OR(J104="",Q104&lt;&gt;""),"",J104&amp;"|"&amp;R104)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="105">
+      <x:c r="R105" s="45" t="str">
+        <x:f>IF(OR(J105="",Q105&lt;&gt;""),"",COUNTIF($J$5:J105,J105))</x:f>
+      </x:c>
+      <x:c r="U105" s="45" t="str">
+        <x:f>IF(OR(J105="",Q105&lt;&gt;""),"",J105&amp;"|"&amp;R105)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="R106" s="45" t="str">
+        <x:f>IF(OR(J106="",Q106&lt;&gt;""),"",COUNTIF($J$5:J106,J106))</x:f>
+      </x:c>
+      <x:c r="U106" s="45" t="str">
+        <x:f>IF(OR(J106="",Q106&lt;&gt;""),"",J106&amp;"|"&amp;R106)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="R107" s="45" t="str">
+        <x:f>IF(OR(J107="",Q107&lt;&gt;""),"",COUNTIF($J$5:J107,J107))</x:f>
+      </x:c>
+      <x:c r="U107" s="45" t="str">
+        <x:f>IF(OR(J107="",Q107&lt;&gt;""),"",J107&amp;"|"&amp;R107)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="R108" s="45" t="str">
+        <x:f>IF(OR(J108="",Q108&lt;&gt;""),"",COUNTIF($J$5:J108,J108))</x:f>
+      </x:c>
+      <x:c r="U108" s="45" t="str">
+        <x:f>IF(OR(J108="",Q108&lt;&gt;""),"",J108&amp;"|"&amp;R108)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="R109" s="45" t="str">
+        <x:f>IF(OR(J109="",Q109&lt;&gt;""),"",COUNTIF($J$5:J109,J109))</x:f>
+      </x:c>
+      <x:c r="U109" s="45" t="str">
+        <x:f>IF(OR(J109="",Q109&lt;&gt;""),"",J109&amp;"|"&amp;R109)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="R110" s="45" t="str">
+        <x:f>IF(OR(J110="",Q110&lt;&gt;""),"",COUNTIF($J$5:J110,J110))</x:f>
+      </x:c>
+      <x:c r="U110" s="45" t="str">
+        <x:f>IF(OR(J110="",Q110&lt;&gt;""),"",J110&amp;"|"&amp;R110)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="R111" s="45" t="str">
+        <x:f>IF(OR(J111="",Q111&lt;&gt;""),"",COUNTIF($J$5:J111,J111))</x:f>
+      </x:c>
+      <x:c r="U111" s="45" t="str">
+        <x:f>IF(OR(J111="",Q111&lt;&gt;""),"",J111&amp;"|"&amp;R111)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="112">
+      <x:c r="R112" s="45" t="str">
+        <x:f>IF(OR(J112="",Q112&lt;&gt;""),"",COUNTIF($J$5:J112,J112))</x:f>
+      </x:c>
+      <x:c r="U112" s="45" t="str">
+        <x:f>IF(OR(J112="",Q112&lt;&gt;""),"",J112&amp;"|"&amp;R112)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="113">
+      <x:c r="R113" s="45" t="str">
+        <x:f>IF(OR(J113="",Q113&lt;&gt;""),"",COUNTIF($J$5:J113,J113))</x:f>
+      </x:c>
+      <x:c r="U113" s="45" t="str">
+        <x:f>IF(OR(J113="",Q113&lt;&gt;""),"",J113&amp;"|"&amp;R113)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="114">
+      <x:c r="R114" s="45" t="str">
+        <x:f>IF(OR(J114="",Q114&lt;&gt;""),"",COUNTIF($J$5:J114,J114))</x:f>
+      </x:c>
+      <x:c r="U114" s="45" t="str">
+        <x:f>IF(OR(J114="",Q114&lt;&gt;""),"",J114&amp;"|"&amp;R114)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="115">
+      <x:c r="R115" s="45" t="str">
+        <x:f>IF(OR(J115="",Q115&lt;&gt;""),"",COUNTIF($J$5:J115,J115))</x:f>
+      </x:c>
+      <x:c r="U115" s="45" t="str">
+        <x:f>IF(OR(J115="",Q115&lt;&gt;""),"",J115&amp;"|"&amp;R115)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="116">
+      <x:c r="R116" s="45" t="str">
+        <x:f>IF(OR(J116="",Q116&lt;&gt;""),"",COUNTIF($J$5:J116,J116))</x:f>
+      </x:c>
+      <x:c r="U116" s="45" t="str">
+        <x:f>IF(OR(J116="",Q116&lt;&gt;""),"",J116&amp;"|"&amp;R116)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="117">
+      <x:c r="R117" s="45" t="str">
+        <x:f>IF(OR(J117="",Q117&lt;&gt;""),"",COUNTIF($J$5:J117,J117))</x:f>
+      </x:c>
+      <x:c r="U117" s="45" t="str">
+        <x:f>IF(OR(J117="",Q117&lt;&gt;""),"",J117&amp;"|"&amp;R117)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="118">
+      <x:c r="R118" s="45" t="str">
+        <x:f>IF(OR(J118="",Q118&lt;&gt;""),"",COUNTIF($J$5:J118,J118))</x:f>
+      </x:c>
+      <x:c r="U118" s="45" t="str">
+        <x:f>IF(OR(J118="",Q118&lt;&gt;""),"",J118&amp;"|"&amp;R118)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="119">
+      <x:c r="R119" s="45" t="str">
+        <x:f>IF(OR(J119="",Q119&lt;&gt;""),"",COUNTIF($J$5:J119,J119))</x:f>
+      </x:c>
+      <x:c r="U119" s="45" t="str">
+        <x:f>IF(OR(J119="",Q119&lt;&gt;""),"",J119&amp;"|"&amp;R119)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="120">
+      <x:c r="R120" s="45" t="str">
+        <x:f>IF(OR(J120="",Q120&lt;&gt;""),"",COUNTIF($J$5:J120,J120))</x:f>
+      </x:c>
+      <x:c r="U120" s="45" t="str">
+        <x:f>IF(OR(J120="",Q120&lt;&gt;""),"",J120&amp;"|"&amp;R120)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="121">
+      <x:c r="R121" s="45" t="str">
+        <x:f>IF(OR(J121="",Q121&lt;&gt;""),"",COUNTIF($J$5:J121,J121))</x:f>
+      </x:c>
+      <x:c r="U121" s="45" t="str">
+        <x:f>IF(OR(J121="",Q121&lt;&gt;""),"",J121&amp;"|"&amp;R121)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="122">
+      <x:c r="R122" s="45" t="str">
+        <x:f>IF(OR(J122="",Q122&lt;&gt;""),"",COUNTIF($J$5:J122,J122))</x:f>
+      </x:c>
+      <x:c r="U122" s="45" t="str">
+        <x:f>IF(OR(J122="",Q122&lt;&gt;""),"",J122&amp;"|"&amp;R122)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="123">
+      <x:c r="R123" s="45" t="str">
+        <x:f>IF(OR(J123="",Q123&lt;&gt;""),"",COUNTIF($J$5:J123,J123))</x:f>
+      </x:c>
+      <x:c r="U123" s="45" t="str">
+        <x:f>IF(OR(J123="",Q123&lt;&gt;""),"",J123&amp;"|"&amp;R123)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="124">
+      <x:c r="R124" s="45" t="str">
+        <x:f>IF(OR(J124="",Q124&lt;&gt;""),"",COUNTIF($J$5:J124,J124))</x:f>
+      </x:c>
+      <x:c r="U124" s="45" t="str">
+        <x:f>IF(OR(J124="",Q124&lt;&gt;""),"",J124&amp;"|"&amp;R124)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="125">
+      <x:c r="R125" s="45" t="str">
+        <x:f>IF(OR(J125="",Q125&lt;&gt;""),"",COUNTIF($J$5:J125,J125))</x:f>
+      </x:c>
+      <x:c r="U125" s="45" t="str">
+        <x:f>IF(OR(J125="",Q125&lt;&gt;""),"",J125&amp;"|"&amp;R125)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="126">
+      <x:c r="R126" s="45" t="str">
+        <x:f>IF(OR(J126="",Q126&lt;&gt;""),"",COUNTIF($J$5:J126,J126))</x:f>
+      </x:c>
+      <x:c r="U126" s="45" t="str">
+        <x:f>IF(OR(J126="",Q126&lt;&gt;""),"",J126&amp;"|"&amp;R126)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="127">
+      <x:c r="R127" s="45" t="str">
+        <x:f>IF(OR(J127="",Q127&lt;&gt;""),"",COUNTIF($J$5:J127,J127))</x:f>
+      </x:c>
+      <x:c r="U127" s="45" t="str">
+        <x:f>IF(OR(J127="",Q127&lt;&gt;""),"",J127&amp;"|"&amp;R127)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="128">
+      <x:c r="R128" s="45" t="str">
+        <x:f>IF(OR(J128="",Q128&lt;&gt;""),"",COUNTIF($J$5:J128,J128))</x:f>
+      </x:c>
+      <x:c r="U128" s="45" t="str">
+        <x:f>IF(OR(J128="",Q128&lt;&gt;""),"",J128&amp;"|"&amp;R128)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="129">
+      <x:c r="R129" s="45" t="str">
+        <x:f>IF(OR(J129="",Q129&lt;&gt;""),"",COUNTIF($J$5:J129,J129))</x:f>
+      </x:c>
+      <x:c r="U129" s="45" t="str">
+        <x:f>IF(OR(J129="",Q129&lt;&gt;""),"",J129&amp;"|"&amp;R129)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="130">
+      <x:c r="R130" s="45" t="str">
+        <x:f>IF(OR(J130="",Q130&lt;&gt;""),"",COUNTIF($J$5:J130,J130))</x:f>
+      </x:c>
+      <x:c r="U130" s="45" t="str">
+        <x:f>IF(OR(J130="",Q130&lt;&gt;""),"",J130&amp;"|"&amp;R130)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="131">
+      <x:c r="R131" s="45" t="str">
+        <x:f>IF(OR(J131="",Q131&lt;&gt;""),"",COUNTIF($J$5:J131,J131))</x:f>
+      </x:c>
+      <x:c r="U131" s="45" t="str">
+        <x:f>IF(OR(J131="",Q131&lt;&gt;""),"",J131&amp;"|"&amp;R131)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="132">
+      <x:c r="R132" s="45" t="str">
+        <x:f>IF(OR(J132="",Q132&lt;&gt;""),"",COUNTIF($J$5:J132,J132))</x:f>
+      </x:c>
+      <x:c r="U132" s="45" t="str">
+        <x:f>IF(OR(J132="",Q132&lt;&gt;""),"",J132&amp;"|"&amp;R132)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="133">
+      <x:c r="R133" s="45" t="str">
+        <x:f>IF(OR(J133="",Q133&lt;&gt;""),"",COUNTIF($J$5:J133,J133))</x:f>
+      </x:c>
+      <x:c r="U133" s="45" t="str">
+        <x:f>IF(OR(J133="",Q133&lt;&gt;""),"",J133&amp;"|"&amp;R133)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="R134" s="45" t="str">
+        <x:f>IF(OR(J134="",Q134&lt;&gt;""),"",COUNTIF($J$5:J134,J134))</x:f>
+      </x:c>
+      <x:c r="U134" s="45" t="str">
+        <x:f>IF(OR(J134="",Q134&lt;&gt;""),"",J134&amp;"|"&amp;R134)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="R135" s="45" t="str">
+        <x:f>IF(OR(J135="",Q135&lt;&gt;""),"",COUNTIF($J$5:J135,J135))</x:f>
+      </x:c>
+      <x:c r="U135" s="45" t="str">
+        <x:f>IF(OR(J135="",Q135&lt;&gt;""),"",J135&amp;"|"&amp;R135)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="R136" s="45" t="str">
+        <x:f>IF(OR(J136="",Q136&lt;&gt;""),"",COUNTIF($J$5:J136,J136))</x:f>
+      </x:c>
+      <x:c r="U136" s="45" t="str">
+        <x:f>IF(OR(J136="",Q136&lt;&gt;""),"",J136&amp;"|"&amp;R136)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="R137" s="45" t="str">
+        <x:f>IF(OR(J137="",Q137&lt;&gt;""),"",COUNTIF($J$5:J137,J137))</x:f>
+      </x:c>
+      <x:c r="U137" s="45" t="str">
+        <x:f>IF(OR(J137="",Q137&lt;&gt;""),"",J137&amp;"|"&amp;R137)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="138">
+      <x:c r="R138" s="45" t="str">
+        <x:f>IF(OR(J138="",Q138&lt;&gt;""),"",COUNTIF($J$5:J138,J138))</x:f>
+      </x:c>
+      <x:c r="U138" s="45" t="str">
+        <x:f>IF(OR(J138="",Q138&lt;&gt;""),"",J138&amp;"|"&amp;R138)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="139">
+      <x:c r="R139" s="45" t="str">
+        <x:f>IF(OR(J139="",Q139&lt;&gt;""),"",COUNTIF($J$5:J139,J139))</x:f>
+      </x:c>
+      <x:c r="U139" s="45" t="str">
+        <x:f>IF(OR(J139="",Q139&lt;&gt;""),"",J139&amp;"|"&amp;R139)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="R140" s="45" t="str">
+        <x:f>IF(OR(J140="",Q140&lt;&gt;""),"",COUNTIF($J$5:J140,J140))</x:f>
+      </x:c>
+      <x:c r="U140" s="45" t="str">
+        <x:f>IF(OR(J140="",Q140&lt;&gt;""),"",J140&amp;"|"&amp;R140)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="141">
+      <x:c r="R141" s="45" t="str">
+        <x:f>IF(OR(J141="",Q141&lt;&gt;""),"",COUNTIF($J$5:J141,J141))</x:f>
+      </x:c>
+      <x:c r="U141" s="45" t="str">
+        <x:f>IF(OR(J141="",Q141&lt;&gt;""),"",J141&amp;"|"&amp;R141)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="R142" s="45" t="str">
+        <x:f>IF(OR(J142="",Q142&lt;&gt;""),"",COUNTIF($J$5:J142,J142))</x:f>
+      </x:c>
+      <x:c r="U142" s="45" t="str">
+        <x:f>IF(OR(J142="",Q142&lt;&gt;""),"",J142&amp;"|"&amp;R142)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="R143" s="45" t="str">
+        <x:f>IF(OR(J143="",Q143&lt;&gt;""),"",COUNTIF($J$5:J143,J143))</x:f>
+      </x:c>
+      <x:c r="U143" s="45" t="str">
+        <x:f>IF(OR(J143="",Q143&lt;&gt;""),"",J143&amp;"|"&amp;R143)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="R144" s="45" t="str">
+        <x:f>IF(OR(J144="",Q144&lt;&gt;""),"",COUNTIF($J$5:J144,J144))</x:f>
+      </x:c>
+      <x:c r="U144" s="45" t="str">
+        <x:f>IF(OR(J144="",Q144&lt;&gt;""),"",J144&amp;"|"&amp;R144)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="R145" s="45" t="str">
+        <x:f>IF(OR(J145="",Q145&lt;&gt;""),"",COUNTIF($J$5:J145,J145))</x:f>
+      </x:c>
+      <x:c r="U145" s="45" t="str">
+        <x:f>IF(OR(J145="",Q145&lt;&gt;""),"",J145&amp;"|"&amp;R145)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="R146" s="45" t="str">
+        <x:f>IF(OR(J146="",Q146&lt;&gt;""),"",COUNTIF($J$5:J146,J146))</x:f>
+      </x:c>
+      <x:c r="U146" s="45" t="str">
+        <x:f>IF(OR(J146="",Q146&lt;&gt;""),"",J146&amp;"|"&amp;R146)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="R147" s="45" t="str">
+        <x:f>IF(OR(J147="",Q147&lt;&gt;""),"",COUNTIF($J$5:J147,J147))</x:f>
+      </x:c>
+      <x:c r="U147" s="45" t="str">
+        <x:f>IF(OR(J147="",Q147&lt;&gt;""),"",J147&amp;"|"&amp;R147)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="R148" s="45" t="str">
+        <x:f>IF(OR(J148="",Q148&lt;&gt;""),"",COUNTIF($J$5:J148,J148))</x:f>
+      </x:c>
+      <x:c r="U148" s="45" t="str">
+        <x:f>IF(OR(J148="",Q148&lt;&gt;""),"",J148&amp;"|"&amp;R148)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="R149" s="45" t="str">
+        <x:f>IF(OR(J149="",Q149&lt;&gt;""),"",COUNTIF($J$5:J149,J149))</x:f>
+      </x:c>
+      <x:c r="U149" s="45" t="str">
+        <x:f>IF(OR(J149="",Q149&lt;&gt;""),"",J149&amp;"|"&amp;R149)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="R150" s="45" t="str">
+        <x:f>IF(OR(J150="",Q150&lt;&gt;""),"",COUNTIF($J$5:J150,J150))</x:f>
+      </x:c>
+      <x:c r="U150" s="45" t="str">
+        <x:f>IF(OR(J150="",Q150&lt;&gt;""),"",J150&amp;"|"&amp;R150)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="151">
+      <x:c r="R151" s="45" t="str">
+        <x:f>IF(OR(J151="",Q151&lt;&gt;""),"",COUNTIF($J$5:J151,J151))</x:f>
+      </x:c>
+      <x:c r="U151" s="45" t="str">
+        <x:f>IF(OR(J151="",Q151&lt;&gt;""),"",J151&amp;"|"&amp;R151)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="152">
+      <x:c r="R152" s="45" t="str">
+        <x:f>IF(OR(J152="",Q152&lt;&gt;""),"",COUNTIF($J$5:J152,J152))</x:f>
+      </x:c>
+      <x:c r="U152" s="45" t="str">
+        <x:f>IF(OR(J152="",Q152&lt;&gt;""),"",J152&amp;"|"&amp;R152)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="153">
+      <x:c r="R153" s="45" t="str">
+        <x:f>IF(OR(J153="",Q153&lt;&gt;""),"",COUNTIF($J$5:J153,J153))</x:f>
+      </x:c>
+      <x:c r="U153" s="45" t="str">
+        <x:f>IF(OR(J153="",Q153&lt;&gt;""),"",J153&amp;"|"&amp;R153)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="154">
+      <x:c r="R154" s="45" t="str">
+        <x:f>IF(OR(J154="",Q154&lt;&gt;""),"",COUNTIF($J$5:J154,J154))</x:f>
+      </x:c>
+      <x:c r="U154" s="45" t="str">
+        <x:f>IF(OR(J154="",Q154&lt;&gt;""),"",J154&amp;"|"&amp;R154)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="155">
+      <x:c r="R155" s="45" t="str">
+        <x:f>IF(OR(J155="",Q155&lt;&gt;""),"",COUNTIF($J$5:J155,J155))</x:f>
+      </x:c>
+      <x:c r="U155" s="45" t="str">
+        <x:f>IF(OR(J155="",Q155&lt;&gt;""),"",J155&amp;"|"&amp;R155)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="156">
+      <x:c r="R156" s="45" t="str">
+        <x:f>IF(OR(J156="",Q156&lt;&gt;""),"",COUNTIF($J$5:J156,J156))</x:f>
+      </x:c>
+      <x:c r="U156" s="45" t="str">
+        <x:f>IF(OR(J156="",Q156&lt;&gt;""),"",J156&amp;"|"&amp;R156)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="157">
+      <x:c r="R157" s="45" t="str">
+        <x:f>IF(OR(J157="",Q157&lt;&gt;""),"",COUNTIF($J$5:J157,J157))</x:f>
+      </x:c>
+      <x:c r="U157" s="45" t="str">
+        <x:f>IF(OR(J157="",Q157&lt;&gt;""),"",J157&amp;"|"&amp;R157)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="158">
+      <x:c r="R158" s="45" t="str">
+        <x:f>IF(OR(J158="",Q158&lt;&gt;""),"",COUNTIF($J$5:J158,J158))</x:f>
+      </x:c>
+      <x:c r="U158" s="45" t="str">
+        <x:f>IF(OR(J158="",Q158&lt;&gt;""),"",J158&amp;"|"&amp;R158)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="159">
+      <x:c r="R159" s="45" t="str">
+        <x:f>IF(OR(J159="",Q159&lt;&gt;""),"",COUNTIF($J$5:J159,J159))</x:f>
+      </x:c>
+      <x:c r="U159" s="45" t="str">
+        <x:f>IF(OR(J159="",Q159&lt;&gt;""),"",J159&amp;"|"&amp;R159)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="160">
+      <x:c r="R160" s="45" t="str">
+        <x:f>IF(OR(J160="",Q160&lt;&gt;""),"",COUNTIF($J$5:J160,J160))</x:f>
+      </x:c>
+      <x:c r="U160" s="45" t="str">
+        <x:f>IF(OR(J160="",Q160&lt;&gt;""),"",J160&amp;"|"&amp;R160)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="161">
+      <x:c r="R161" s="45" t="str">
+        <x:f>IF(OR(J161="",Q161&lt;&gt;""),"",COUNTIF($J$5:J161,J161))</x:f>
+      </x:c>
+      <x:c r="U161" s="45" t="str">
+        <x:f>IF(OR(J161="",Q161&lt;&gt;""),"",J161&amp;"|"&amp;R161)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="162">
+      <x:c r="R162" s="45" t="str">
+        <x:f>IF(OR(J162="",Q162&lt;&gt;""),"",COUNTIF($J$5:J162,J162))</x:f>
+      </x:c>
+      <x:c r="U162" s="45" t="str">
+        <x:f>IF(OR(J162="",Q162&lt;&gt;""),"",J162&amp;"|"&amp;R162)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="163">
+      <x:c r="R163" s="45" t="str">
+        <x:f>IF(OR(J163="",Q163&lt;&gt;""),"",COUNTIF($J$5:J163,J163))</x:f>
+      </x:c>
+      <x:c r="U163" s="45" t="str">
+        <x:f>IF(OR(J163="",Q163&lt;&gt;""),"",J163&amp;"|"&amp;R163)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="164">
+      <x:c r="R164" s="45" t="str">
+        <x:f>IF(OR(J164="",Q164&lt;&gt;""),"",COUNTIF($J$5:J164,J164))</x:f>
+      </x:c>
+      <x:c r="U164" s="45" t="str">
+        <x:f>IF(OR(J164="",Q164&lt;&gt;""),"",J164&amp;"|"&amp;R164)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="165">
+      <x:c r="R165" s="45" t="str">
+        <x:f>IF(OR(J165="",Q165&lt;&gt;""),"",COUNTIF($J$5:J165,J165))</x:f>
+      </x:c>
+      <x:c r="U165" s="45" t="str">
+        <x:f>IF(OR(J165="",Q165&lt;&gt;""),"",J165&amp;"|"&amp;R165)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="166">
+      <x:c r="R166" s="45" t="str">
+        <x:f>IF(OR(J166="",Q166&lt;&gt;""),"",COUNTIF($J$5:J166,J166))</x:f>
+      </x:c>
+      <x:c r="U166" s="45" t="str">
+        <x:f>IF(OR(J166="",Q166&lt;&gt;""),"",J166&amp;"|"&amp;R166)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="167">
+      <x:c r="R167" s="45" t="str">
+        <x:f>IF(OR(J167="",Q167&lt;&gt;""),"",COUNTIF($J$5:J167,J167))</x:f>
+      </x:c>
+      <x:c r="U167" s="45" t="str">
+        <x:f>IF(OR(J167="",Q167&lt;&gt;""),"",J167&amp;"|"&amp;R167)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="168">
+      <x:c r="R168" s="45" t="str">
+        <x:f>IF(OR(J168="",Q168&lt;&gt;""),"",COUNTIF($J$5:J168,J168))</x:f>
+      </x:c>
+      <x:c r="U168" s="45" t="str">
+        <x:f>IF(OR(J168="",Q168&lt;&gt;""),"",J168&amp;"|"&amp;R168)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="169">
+      <x:c r="R169" s="45" t="str">
+        <x:f>IF(OR(J169="",Q169&lt;&gt;""),"",COUNTIF($J$5:J169,J169))</x:f>
+      </x:c>
+      <x:c r="U169" s="45" t="str">
+        <x:f>IF(OR(J169="",Q169&lt;&gt;""),"",J169&amp;"|"&amp;R169)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="170">
+      <x:c r="R170" s="45" t="str">
+        <x:f>IF(OR(J170="",Q170&lt;&gt;""),"",COUNTIF($J$5:J170,J170))</x:f>
+      </x:c>
+      <x:c r="U170" s="45" t="str">
+        <x:f>IF(OR(J170="",Q170&lt;&gt;""),"",J170&amp;"|"&amp;R170)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="171">
+      <x:c r="R171" s="45" t="str">
+        <x:f>IF(OR(J171="",Q171&lt;&gt;""),"",COUNTIF($J$5:J171,J171))</x:f>
+      </x:c>
+      <x:c r="U171" s="45" t="str">
+        <x:f>IF(OR(J171="",Q171&lt;&gt;""),"",J171&amp;"|"&amp;R171)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="172">
+      <x:c r="R172" s="45" t="str">
+        <x:f>IF(OR(J172="",Q172&lt;&gt;""),"",COUNTIF($J$5:J172,J172))</x:f>
+      </x:c>
+      <x:c r="U172" s="45" t="str">
+        <x:f>IF(OR(J172="",Q172&lt;&gt;""),"",J172&amp;"|"&amp;R172)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="173">
+      <x:c r="R173" s="45" t="str">
+        <x:f>IF(OR(J173="",Q173&lt;&gt;""),"",COUNTIF($J$5:J173,J173))</x:f>
+      </x:c>
+      <x:c r="U173" s="45" t="str">
+        <x:f>IF(OR(J173="",Q173&lt;&gt;""),"",J173&amp;"|"&amp;R173)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="174">
+      <x:c r="R174" s="45" t="str">
+        <x:f>IF(OR(J174="",Q174&lt;&gt;""),"",COUNTIF($J$5:J174,J174))</x:f>
+      </x:c>
+      <x:c r="U174" s="45" t="str">
+        <x:f>IF(OR(J174="",Q174&lt;&gt;""),"",J174&amp;"|"&amp;R174)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="175">
+      <x:c r="R175" s="45" t="str">
+        <x:f>IF(OR(J175="",Q175&lt;&gt;""),"",COUNTIF($J$5:J175,J175))</x:f>
+      </x:c>
+      <x:c r="U175" s="45" t="str">
+        <x:f>IF(OR(J175="",Q175&lt;&gt;""),"",J175&amp;"|"&amp;R175)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="176">
+      <x:c r="R176" s="45" t="str">
+        <x:f>IF(OR(J176="",Q176&lt;&gt;""),"",COUNTIF($J$5:J176,J176))</x:f>
+      </x:c>
+      <x:c r="U176" s="45" t="str">
+        <x:f>IF(OR(J176="",Q176&lt;&gt;""),"",J176&amp;"|"&amp;R176)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="177">
+      <x:c r="R177" s="45" t="str">
+        <x:f>IF(OR(J177="",Q177&lt;&gt;""),"",COUNTIF($J$5:J177,J177))</x:f>
+      </x:c>
+      <x:c r="U177" s="45" t="str">
+        <x:f>IF(OR(J177="",Q177&lt;&gt;""),"",J177&amp;"|"&amp;R177)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="178">
+      <x:c r="R178" s="45" t="str">
+        <x:f>IF(OR(J178="",Q178&lt;&gt;""),"",COUNTIF($J$5:J178,J178))</x:f>
+      </x:c>
+      <x:c r="U178" s="45" t="str">
+        <x:f>IF(OR(J178="",Q178&lt;&gt;""),"",J178&amp;"|"&amp;R178)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="179">
+      <x:c r="R179" s="45" t="str">
+        <x:f>IF(OR(J179="",Q179&lt;&gt;""),"",COUNTIF($J$5:J179,J179))</x:f>
+      </x:c>
+      <x:c r="U179" s="45" t="str">
+        <x:f>IF(OR(J179="",Q179&lt;&gt;""),"",J179&amp;"|"&amp;R179)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="180">
+      <x:c r="R180" s="45" t="str">
+        <x:f>IF(OR(J180="",Q180&lt;&gt;""),"",COUNTIF($J$5:J180,J180))</x:f>
+      </x:c>
+      <x:c r="U180" s="45" t="str">
+        <x:f>IF(OR(J180="",Q180&lt;&gt;""),"",J180&amp;"|"&amp;R180)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="181">
+      <x:c r="R181" s="45" t="str">
+        <x:f>IF(OR(J181="",Q181&lt;&gt;""),"",COUNTIF($J$5:J181,J181))</x:f>
+      </x:c>
+      <x:c r="U181" s="45" t="str">
+        <x:f>IF(OR(J181="",Q181&lt;&gt;""),"",J181&amp;"|"&amp;R181)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="182">
+      <x:c r="R182" s="45" t="str">
+        <x:f>IF(OR(J182="",Q182&lt;&gt;""),"",COUNTIF($J$5:J182,J182))</x:f>
+      </x:c>
+      <x:c r="U182" s="45" t="str">
+        <x:f>IF(OR(J182="",Q182&lt;&gt;""),"",J182&amp;"|"&amp;R182)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="183">
+      <x:c r="R183" s="45" t="str">
+        <x:f>IF(OR(J183="",Q183&lt;&gt;""),"",COUNTIF($J$5:J183,J183))</x:f>
+      </x:c>
+      <x:c r="U183" s="45" t="str">
+        <x:f>IF(OR(J183="",Q183&lt;&gt;""),"",J183&amp;"|"&amp;R183)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="184">
+      <x:c r="R184" s="45" t="str">
+        <x:f>IF(OR(J184="",Q184&lt;&gt;""),"",COUNTIF($J$5:J184,J184))</x:f>
+      </x:c>
+      <x:c r="U184" s="45" t="str">
+        <x:f>IF(OR(J184="",Q184&lt;&gt;""),"",J184&amp;"|"&amp;R184)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="185">
+      <x:c r="R185" s="45" t="str">
+        <x:f>IF(OR(J185="",Q185&lt;&gt;""),"",COUNTIF($J$5:J185,J185))</x:f>
+      </x:c>
+      <x:c r="U185" s="45" t="str">
+        <x:f>IF(OR(J185="",Q185&lt;&gt;""),"",J185&amp;"|"&amp;R185)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="186">
+      <x:c r="R186" s="45" t="str">
+        <x:f>IF(OR(J186="",Q186&lt;&gt;""),"",COUNTIF($J$5:J186,J186))</x:f>
+      </x:c>
+      <x:c r="U186" s="45" t="str">
+        <x:f>IF(OR(J186="",Q186&lt;&gt;""),"",J186&amp;"|"&amp;R186)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="187">
+      <x:c r="R187" s="45" t="str">
+        <x:f>IF(OR(J187="",Q187&lt;&gt;""),"",COUNTIF($J$5:J187,J187))</x:f>
+      </x:c>
+      <x:c r="U187" s="45" t="str">
+        <x:f>IF(OR(J187="",Q187&lt;&gt;""),"",J187&amp;"|"&amp;R187)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="188">
+      <x:c r="R188" s="45" t="str">
+        <x:f>IF(OR(J188="",Q188&lt;&gt;""),"",COUNTIF($J$5:J188,J188))</x:f>
+      </x:c>
+      <x:c r="U188" s="45" t="str">
+        <x:f>IF(OR(J188="",Q188&lt;&gt;""),"",J188&amp;"|"&amp;R188)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="189">
+      <x:c r="R189" s="45" t="str">
+        <x:f>IF(OR(J189="",Q189&lt;&gt;""),"",COUNTIF($J$5:J189,J189))</x:f>
+      </x:c>
+      <x:c r="U189" s="45" t="str">
+        <x:f>IF(OR(J189="",Q189&lt;&gt;""),"",J189&amp;"|"&amp;R189)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="190">
+      <x:c r="R190" s="45" t="str">
+        <x:f>IF(OR(J190="",Q190&lt;&gt;""),"",COUNTIF($J$5:J190,J190))</x:f>
+      </x:c>
+      <x:c r="U190" s="45" t="str">
+        <x:f>IF(OR(J190="",Q190&lt;&gt;""),"",J190&amp;"|"&amp;R190)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="191">
+      <x:c r="R191" s="45" t="str">
+        <x:f>IF(OR(J191="",Q191&lt;&gt;""),"",COUNTIF($J$5:J191,J191))</x:f>
+      </x:c>
+      <x:c r="U191" s="45" t="str">
+        <x:f>IF(OR(J191="",Q191&lt;&gt;""),"",J191&amp;"|"&amp;R191)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="192">
+      <x:c r="R192" s="45" t="str">
+        <x:f>IF(OR(J192="",Q192&lt;&gt;""),"",COUNTIF($J$5:J192,J192))</x:f>
+      </x:c>
+      <x:c r="U192" s="45" t="str">
+        <x:f>IF(OR(J192="",Q192&lt;&gt;""),"",J192&amp;"|"&amp;R192)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="193">
+      <x:c r="R193" s="45" t="str">
+        <x:f>IF(OR(J193="",Q193&lt;&gt;""),"",COUNTIF($J$5:J193,J193))</x:f>
+      </x:c>
+      <x:c r="U193" s="45" t="str">
+        <x:f>IF(OR(J193="",Q193&lt;&gt;""),"",J193&amp;"|"&amp;R193)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="194">
+      <x:c r="R194" s="45" t="str">
+        <x:f>IF(OR(J194="",Q194&lt;&gt;""),"",COUNTIF($J$5:J194,J194))</x:f>
+      </x:c>
+      <x:c r="U194" s="45" t="str">
+        <x:f>IF(OR(J194="",Q194&lt;&gt;""),"",J194&amp;"|"&amp;R194)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="195">
+      <x:c r="R195" s="45" t="str">
+        <x:f>IF(OR(J195="",Q195&lt;&gt;""),"",COUNTIF($J$5:J195,J195))</x:f>
+      </x:c>
+      <x:c r="U195" s="45" t="str">
+        <x:f>IF(OR(J195="",Q195&lt;&gt;""),"",J195&amp;"|"&amp;R195)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="196">
+      <x:c r="R196" s="45" t="str">
+        <x:f>IF(OR(J196="",Q196&lt;&gt;""),"",COUNTIF($J$5:J196,J196))</x:f>
+      </x:c>
+      <x:c r="U196" s="45" t="str">
+        <x:f>IF(OR(J196="",Q196&lt;&gt;""),"",J196&amp;"|"&amp;R196)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="197">
+      <x:c r="R197" s="45" t="str">
+        <x:f>IF(OR(J197="",Q197&lt;&gt;""),"",COUNTIF($J$5:J197,J197))</x:f>
+      </x:c>
+      <x:c r="U197" s="45" t="str">
+        <x:f>IF(OR(J197="",Q197&lt;&gt;""),"",J197&amp;"|"&amp;R197)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="198">
+      <x:c r="R198" s="45" t="str">
+        <x:f>IF(OR(J198="",Q198&lt;&gt;""),"",COUNTIF($J$5:J198,J198))</x:f>
+      </x:c>
+      <x:c r="U198" s="45" t="str">
+        <x:f>IF(OR(J198="",Q198&lt;&gt;""),"",J198&amp;"|"&amp;R198)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="199">
+      <x:c r="R199" s="45" t="str">
+        <x:f>IF(OR(J199="",Q199&lt;&gt;""),"",COUNTIF($J$5:J199,J199))</x:f>
+      </x:c>
+      <x:c r="U199" s="45" t="str">
+        <x:f>IF(OR(J199="",Q199&lt;&gt;""),"",J199&amp;"|"&amp;R199)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="200">
+      <x:c r="R200" s="45" t="str">
+        <x:f>IF(OR(J200="",Q200&lt;&gt;""),"",COUNTIF($J$5:J200,J200))</x:f>
+      </x:c>
+      <x:c r="U200" s="45" t="str">
+        <x:f>IF(OR(J200="",Q200&lt;&gt;""),"",J200&amp;"|"&amp;R200)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="201">
+      <x:c r="R201" s="45" t="str">
+        <x:f>IF(OR(J201="",Q201&lt;&gt;""),"",COUNTIF($J$5:J201,J201))</x:f>
+      </x:c>
+      <x:c r="U201" s="45" t="str">
+        <x:f>IF(OR(J201="",Q201&lt;&gt;""),"",J201&amp;"|"&amp;R201)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="202">
+      <x:c r="R202" s="45" t="str">
+        <x:f>IF(OR(J202="",Q202&lt;&gt;""),"",COUNTIF($J$5:J202,J202))</x:f>
+      </x:c>
+      <x:c r="U202" s="45" t="str">
+        <x:f>IF(OR(J202="",Q202&lt;&gt;""),"",J202&amp;"|"&amp;R202)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="203">
+      <x:c r="R203" s="45" t="str">
+        <x:f>IF(OR(J203="",Q203&lt;&gt;""),"",COUNTIF($J$5:J203,J203))</x:f>
+      </x:c>
+      <x:c r="U203" s="45" t="str">
+        <x:f>IF(OR(J203="",Q203&lt;&gt;""),"",J203&amp;"|"&amp;R203)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="204">
+      <x:c r="R204" s="45" t="str">
+        <x:f>IF(OR(J204="",Q204&lt;&gt;""),"",COUNTIF($J$5:J204,J204))</x:f>
+      </x:c>
+      <x:c r="U204" s="45" t="str">
+        <x:f>IF(OR(J204="",Q204&lt;&gt;""),"",J204&amp;"|"&amp;R204)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="205">
+      <x:c r="R205" s="45" t="str">
+        <x:f>IF(OR(J205="",Q205&lt;&gt;""),"",COUNTIF($J$5:J205,J205))</x:f>
+      </x:c>
+      <x:c r="U205" s="45" t="str">
+        <x:f>IF(OR(J205="",Q205&lt;&gt;""),"",J205&amp;"|"&amp;R205)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="206">
+      <x:c r="R206" s="45" t="str">
+        <x:f>IF(OR(J206="",Q206&lt;&gt;""),"",COUNTIF($J$5:J206,J206))</x:f>
+      </x:c>
+      <x:c r="U206" s="45" t="str">
+        <x:f>IF(OR(J206="",Q206&lt;&gt;""),"",J206&amp;"|"&amp;R206)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="207">
+      <x:c r="R207" s="45" t="str">
+        <x:f>IF(OR(J207="",Q207&lt;&gt;""),"",COUNTIF($J$5:J207,J207))</x:f>
+      </x:c>
+      <x:c r="U207" s="45" t="str">
+        <x:f>IF(OR(J207="",Q207&lt;&gt;""),"",J207&amp;"|"&amp;R207)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="208">
+      <x:c r="R208" s="45" t="str">
+        <x:f>IF(OR(J208="",Q208&lt;&gt;""),"",COUNTIF($J$5:J208,J208))</x:f>
+      </x:c>
+      <x:c r="U208" s="45" t="str">
+        <x:f>IF(OR(J208="",Q208&lt;&gt;""),"",J208&amp;"|"&amp;R208)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="209">
+      <x:c r="R209" s="45" t="str">
+        <x:f>IF(OR(J209="",Q209&lt;&gt;""),"",COUNTIF($J$5:J209,J209))</x:f>
+      </x:c>
+      <x:c r="U209" s="45" t="str">
+        <x:f>IF(OR(J209="",Q209&lt;&gt;""),"",J209&amp;"|"&amp;R209)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="210">
+      <x:c r="R210" s="45" t="str">
+        <x:f>IF(OR(J210="",Q210&lt;&gt;""),"",COUNTIF($J$5:J210,J210))</x:f>
+      </x:c>
+      <x:c r="U210" s="45" t="str">
+        <x:f>IF(OR(J210="",Q210&lt;&gt;""),"",J210&amp;"|"&amp;R210)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="211">
+      <x:c r="R211" s="45" t="str">
+        <x:f>IF(OR(J211="",Q211&lt;&gt;""),"",COUNTIF($J$5:J211,J211))</x:f>
+      </x:c>
+      <x:c r="U211" s="45" t="str">
+        <x:f>IF(OR(J211="",Q211&lt;&gt;""),"",J211&amp;"|"&amp;R211)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="212">
+      <x:c r="R212" s="45" t="str">
+        <x:f>IF(OR(J212="",Q212&lt;&gt;""),"",COUNTIF($J$5:J212,J212))</x:f>
+      </x:c>
+      <x:c r="U212" s="45" t="str">
+        <x:f>IF(OR(J212="",Q212&lt;&gt;""),"",J212&amp;"|"&amp;R212)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="213">
+      <x:c r="R213" s="45" t="str">
+        <x:f>IF(OR(J213="",Q213&lt;&gt;""),"",COUNTIF($J$5:J213,J213))</x:f>
+      </x:c>
+      <x:c r="U213" s="45" t="str">
+        <x:f>IF(OR(J213="",Q213&lt;&gt;""),"",J213&amp;"|"&amp;R213)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="214">
+      <x:c r="R214" s="45" t="str">
+        <x:f>IF(OR(J214="",Q214&lt;&gt;""),"",COUNTIF($J$5:J214,J214))</x:f>
+      </x:c>
+      <x:c r="U214" s="45" t="str">
+        <x:f>IF(OR(J214="",Q214&lt;&gt;""),"",J214&amp;"|"&amp;R214)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="215">
+      <x:c r="R215" s="45" t="str">
+        <x:f>IF(OR(J215="",Q215&lt;&gt;""),"",COUNTIF($J$5:J215,J215))</x:f>
+      </x:c>
+      <x:c r="U215" s="45" t="str">
+        <x:f>IF(OR(J215="",Q215&lt;&gt;""),"",J215&amp;"|"&amp;R215)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="216">
+      <x:c r="R216" s="45" t="str">
+        <x:f>IF(OR(J216="",Q216&lt;&gt;""),"",COUNTIF($J$5:J216,J216))</x:f>
+      </x:c>
+      <x:c r="U216" s="45" t="str">
+        <x:f>IF(OR(J216="",Q216&lt;&gt;""),"",J216&amp;"|"&amp;R216)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="217">
+      <x:c r="R217" s="45" t="str">
+        <x:f>IF(OR(J217="",Q217&lt;&gt;""),"",COUNTIF($J$5:J217,J217))</x:f>
+      </x:c>
+      <x:c r="U217" s="45" t="str">
+        <x:f>IF(OR(J217="",Q217&lt;&gt;""),"",J217&amp;"|"&amp;R217)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="218">
+      <x:c r="R218" s="45" t="str">
+        <x:f>IF(OR(J218="",Q218&lt;&gt;""),"",COUNTIF($J$5:J218,J218))</x:f>
+      </x:c>
+      <x:c r="U218" s="45" t="str">
+        <x:f>IF(OR(J218="",Q218&lt;&gt;""),"",J218&amp;"|"&amp;R218)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="219">
+      <x:c r="R219" s="45" t="str">
+        <x:f>IF(OR(J219="",Q219&lt;&gt;""),"",COUNTIF($J$5:J219,J219))</x:f>
+      </x:c>
+      <x:c r="U219" s="45" t="str">
+        <x:f>IF(OR(J219="",Q219&lt;&gt;""),"",J219&amp;"|"&amp;R219)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="220">
+      <x:c r="R220" s="45" t="str">
+        <x:f>IF(OR(J220="",Q220&lt;&gt;""),"",COUNTIF($J$5:J220,J220))</x:f>
+      </x:c>
+      <x:c r="U220" s="45" t="str">
+        <x:f>IF(OR(J220="",Q220&lt;&gt;""),"",J220&amp;"|"&amp;R220)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="221">
+      <x:c r="R221" s="45" t="str">
+        <x:f>IF(OR(J221="",Q221&lt;&gt;""),"",COUNTIF($J$5:J221,J221))</x:f>
+      </x:c>
+      <x:c r="U221" s="45" t="str">
+        <x:f>IF(OR(J221="",Q221&lt;&gt;""),"",J221&amp;"|"&amp;R221)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="222">
+      <x:c r="R222" s="45" t="str">
+        <x:f>IF(OR(J222="",Q222&lt;&gt;""),"",COUNTIF($J$5:J222,J222))</x:f>
+      </x:c>
+      <x:c r="U222" s="45" t="str">
+        <x:f>IF(OR(J222="",Q222&lt;&gt;""),"",J222&amp;"|"&amp;R222)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="223">
+      <x:c r="R223" s="45" t="str">
+        <x:f>IF(OR(J223="",Q223&lt;&gt;""),"",COUNTIF($J$5:J223,J223))</x:f>
+      </x:c>
+      <x:c r="U223" s="45" t="str">
+        <x:f>IF(OR(J223="",Q223&lt;&gt;""),"",J223&amp;"|"&amp;R223)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="224">
+      <x:c r="R224" s="45" t="str">
+        <x:f>IF(OR(J224="",Q224&lt;&gt;""),"",COUNTIF($J$5:J224,J224))</x:f>
+      </x:c>
+      <x:c r="U224" s="45" t="str">
+        <x:f>IF(OR(J224="",Q224&lt;&gt;""),"",J224&amp;"|"&amp;R224)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="225">
+      <x:c r="R225" s="45" t="str">
+        <x:f>IF(OR(J225="",Q225&lt;&gt;""),"",COUNTIF($J$5:J225,J225))</x:f>
+      </x:c>
+      <x:c r="U225" s="45" t="str">
+        <x:f>IF(OR(J225="",Q225&lt;&gt;""),"",J225&amp;"|"&amp;R225)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="226">
+      <x:c r="R226" s="45" t="str">
+        <x:f>IF(OR(J226="",Q226&lt;&gt;""),"",COUNTIF($J$5:J226,J226))</x:f>
+      </x:c>
+      <x:c r="U226" s="45" t="str">
+        <x:f>IF(OR(J226="",Q226&lt;&gt;""),"",J226&amp;"|"&amp;R226)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="227">
+      <x:c r="R227" s="45" t="str">
+        <x:f>IF(OR(J227="",Q227&lt;&gt;""),"",COUNTIF($J$5:J227,J227))</x:f>
+      </x:c>
+      <x:c r="U227" s="45" t="str">
+        <x:f>IF(OR(J227="",Q227&lt;&gt;""),"",J227&amp;"|"&amp;R227)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="228">
+      <x:c r="R228" s="45" t="str">
+        <x:f>IF(OR(J228="",Q228&lt;&gt;""),"",COUNTIF($J$5:J228,J228))</x:f>
+      </x:c>
+      <x:c r="U228" s="45" t="str">
+        <x:f>IF(OR(J228="",Q228&lt;&gt;""),"",J228&amp;"|"&amp;R228)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="229">
+      <x:c r="R229" s="45" t="str">
+        <x:f>IF(OR(J229="",Q229&lt;&gt;""),"",COUNTIF($J$5:J229,J229))</x:f>
+      </x:c>
+      <x:c r="U229" s="45" t="str">
+        <x:f>IF(OR(J229="",Q229&lt;&gt;""),"",J229&amp;"|"&amp;R229)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="230">
+      <x:c r="R230" s="45" t="str">
+        <x:f>IF(OR(J230="",Q230&lt;&gt;""),"",COUNTIF($J$5:J230,J230))</x:f>
+      </x:c>
+      <x:c r="U230" s="45" t="str">
+        <x:f>IF(OR(J230="",Q230&lt;&gt;""),"",J230&amp;"|"&amp;R230)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="231">
+      <x:c r="R231" s="45" t="str">
+        <x:f>IF(OR(J231="",Q231&lt;&gt;""),"",COUNTIF($J$5:J231,J231))</x:f>
+      </x:c>
+      <x:c r="U231" s="45" t="str">
+        <x:f>IF(OR(J231="",Q231&lt;&gt;""),"",J231&amp;"|"&amp;R231)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="232">
+      <x:c r="R232" s="45" t="str">
+        <x:f>IF(OR(J232="",Q232&lt;&gt;""),"",COUNTIF($J$5:J232,J232))</x:f>
+      </x:c>
+      <x:c r="U232" s="45" t="str">
+        <x:f>IF(OR(J232="",Q232&lt;&gt;""),"",J232&amp;"|"&amp;R232)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="233">
+      <x:c r="R233" s="45" t="str">
+        <x:f>IF(OR(J233="",Q233&lt;&gt;""),"",COUNTIF($J$5:J233,J233))</x:f>
+      </x:c>
+      <x:c r="U233" s="45" t="str">
+        <x:f>IF(OR(J233="",Q233&lt;&gt;""),"",J233&amp;"|"&amp;R233)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="234">
+      <x:c r="R234" s="45" t="str">
+        <x:f>IF(OR(J234="",Q234&lt;&gt;""),"",COUNTIF($J$5:J234,J234))</x:f>
+      </x:c>
+      <x:c r="U234" s="45" t="str">
+        <x:f>IF(OR(J234="",Q234&lt;&gt;""),"",J234&amp;"|"&amp;R234)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="235">
+      <x:c r="R235" s="45" t="str">
+        <x:f>IF(OR(J235="",Q235&lt;&gt;""),"",COUNTIF($J$5:J235,J235))</x:f>
+      </x:c>
+      <x:c r="U235" s="45" t="str">
+        <x:f>IF(OR(J235="",Q235&lt;&gt;""),"",J235&amp;"|"&amp;R235)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="236">
+      <x:c r="R236" s="45" t="str">
+        <x:f>IF(OR(J236="",Q236&lt;&gt;""),"",COUNTIF($J$5:J236,J236))</x:f>
+      </x:c>
+      <x:c r="U236" s="45" t="str">
+        <x:f>IF(OR(J236="",Q236&lt;&gt;""),"",J236&amp;"|"&amp;R236)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="237">
+      <x:c r="R237" s="45" t="str">
+        <x:f>IF(OR(J237="",Q237&lt;&gt;""),"",COUNTIF($J$5:J237,J237))</x:f>
+      </x:c>
+      <x:c r="U237" s="45" t="str">
+        <x:f>IF(OR(J237="",Q237&lt;&gt;""),"",J237&amp;"|"&amp;R237)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="238">
+      <x:c r="R238" s="45" t="str">
+        <x:f>IF(OR(J238="",Q238&lt;&gt;""),"",COUNTIF($J$5:J238,J238))</x:f>
+      </x:c>
+      <x:c r="U238" s="45" t="str">
+        <x:f>IF(OR(J238="",Q238&lt;&gt;""),"",J238&amp;"|"&amp;R238)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="239">
+      <x:c r="R239" s="45" t="str">
+        <x:f>IF(OR(J239="",Q239&lt;&gt;""),"",COUNTIF($J$5:J239,J239))</x:f>
+      </x:c>
+      <x:c r="U239" s="45" t="str">
+        <x:f>IF(OR(J239="",Q239&lt;&gt;""),"",J239&amp;"|"&amp;R239)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="240">
+      <x:c r="R240" s="45" t="str">
+        <x:f>IF(OR(J240="",Q240&lt;&gt;""),"",COUNTIF($J$5:J240,J240))</x:f>
+      </x:c>
+      <x:c r="U240" s="45" t="str">
+        <x:f>IF(OR(J240="",Q240&lt;&gt;""),"",J240&amp;"|"&amp;R240)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="241">
+      <x:c r="R241" s="45" t="str">
+        <x:f>IF(OR(J241="",Q241&lt;&gt;""),"",COUNTIF($J$5:J241,J241))</x:f>
+      </x:c>
+      <x:c r="U241" s="45" t="str">
+        <x:f>IF(OR(J241="",Q241&lt;&gt;""),"",J241&amp;"|"&amp;R241)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="242">
+      <x:c r="R242" s="45" t="str">
+        <x:f>IF(OR(J242="",Q242&lt;&gt;""),"",COUNTIF($J$5:J242,J242))</x:f>
+      </x:c>
+      <x:c r="U242" s="45" t="str">
+        <x:f>IF(OR(J242="",Q242&lt;&gt;""),"",J242&amp;"|"&amp;R242)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="243">
+      <x:c r="R243" s="45" t="str">
+        <x:f>IF(OR(J243="",Q243&lt;&gt;""),"",COUNTIF($J$5:J243,J243))</x:f>
+      </x:c>
+      <x:c r="U243" s="45" t="str">
+        <x:f>IF(OR(J243="",Q243&lt;&gt;""),"",J243&amp;"|"&amp;R243)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="244">
+      <x:c r="R244" s="45" t="str">
+        <x:f>IF(OR(J244="",Q244&lt;&gt;""),"",COUNTIF($J$5:J244,J244))</x:f>
+      </x:c>
+      <x:c r="U244" s="45" t="str">
+        <x:f>IF(OR(J244="",Q244&lt;&gt;""),"",J244&amp;"|"&amp;R244)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="245">
+      <x:c r="R245" s="45" t="str">
+        <x:f>IF(OR(J245="",Q245&lt;&gt;""),"",COUNTIF($J$5:J245,J245))</x:f>
+      </x:c>
+      <x:c r="U245" s="45" t="str">
+        <x:f>IF(OR(J245="",Q245&lt;&gt;""),"",J245&amp;"|"&amp;R245)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="246">
+      <x:c r="R246" s="45" t="str">
+        <x:f>IF(OR(J246="",Q246&lt;&gt;""),"",COUNTIF($J$5:J246,J246))</x:f>
+      </x:c>
+      <x:c r="U246" s="45" t="str">
+        <x:f>IF(OR(J246="",Q246&lt;&gt;""),"",J246&amp;"|"&amp;R246)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="247">
+      <x:c r="R247" s="45" t="str">
+        <x:f>IF(OR(J247="",Q247&lt;&gt;""),"",COUNTIF($J$5:J247,J247))</x:f>
+      </x:c>
+      <x:c r="U247" s="45" t="str">
+        <x:f>IF(OR(J247="",Q247&lt;&gt;""),"",J247&amp;"|"&amp;R247)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="248">
+      <x:c r="R248" s="45" t="str">
+        <x:f>IF(OR(J248="",Q248&lt;&gt;""),"",COUNTIF($J$5:J248,J248))</x:f>
+      </x:c>
+      <x:c r="U248" s="45" t="str">
+        <x:f>IF(OR(J248="",Q248&lt;&gt;""),"",J248&amp;"|"&amp;R248)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="249">
+      <x:c r="R249" s="45" t="str">
+        <x:f>IF(OR(J249="",Q249&lt;&gt;""),"",COUNTIF($J$5:J249,J249))</x:f>
+      </x:c>
+      <x:c r="U249" s="45" t="str">
+        <x:f>IF(OR(J249="",Q249&lt;&gt;""),"",J249&amp;"|"&amp;R249)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="250">
+      <x:c r="R250" s="45" t="str">
+        <x:f>IF(OR(J250="",Q250&lt;&gt;""),"",COUNTIF($J$5:J250,J250))</x:f>
+      </x:c>
+      <x:c r="U250" s="45" t="str">
+        <x:f>IF(OR(J250="",Q250&lt;&gt;""),"",J250&amp;"|"&amp;R250)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="251">
+      <x:c r="R251" s="45" t="str">
+        <x:f>IF(OR(J251="",Q251&lt;&gt;""),"",COUNTIF($J$5:J251,J251))</x:f>
+      </x:c>
+      <x:c r="U251" s="45" t="str">
+        <x:f>IF(OR(J251="",Q251&lt;&gt;""),"",J251&amp;"|"&amp;R251)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="252">
+      <x:c r="R252" s="45" t="str">
+        <x:f>IF(OR(J252="",Q252&lt;&gt;""),"",COUNTIF($J$5:J252,J252))</x:f>
+      </x:c>
+      <x:c r="U252" s="45" t="str">
+        <x:f>IF(OR(J252="",Q252&lt;&gt;""),"",J252&amp;"|"&amp;R252)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="253">
+      <x:c r="R253" s="45" t="str">
+        <x:f>IF(OR(J253="",Q253&lt;&gt;""),"",COUNTIF($J$5:J253,J253))</x:f>
+      </x:c>
+      <x:c r="U253" s="45" t="str">
+        <x:f>IF(OR(J253="",Q253&lt;&gt;""),"",J253&amp;"|"&amp;R253)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="254">
+      <x:c r="R254" s="45" t="str">
+        <x:f>IF(OR(J254="",Q254&lt;&gt;""),"",COUNTIF($J$5:J254,J254))</x:f>
+      </x:c>
+      <x:c r="U254" s="45" t="str">
+        <x:f>IF(OR(J254="",Q254&lt;&gt;""),"",J254&amp;"|"&amp;R254)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="255">
+      <x:c r="R255" s="45" t="str">
+        <x:f>IF(OR(J255="",Q255&lt;&gt;""),"",COUNTIF($J$5:J255,J255))</x:f>
+      </x:c>
+      <x:c r="U255" s="45" t="str">
+        <x:f>IF(OR(J255="",Q255&lt;&gt;""),"",J255&amp;"|"&amp;R255)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="256">
+      <x:c r="R256" s="45" t="str">
+        <x:f>IF(OR(J256="",Q256&lt;&gt;""),"",COUNTIF($J$5:J256,J256))</x:f>
+      </x:c>
+      <x:c r="U256" s="45" t="str">
+        <x:f>IF(OR(J256="",Q256&lt;&gt;""),"",J256&amp;"|"&amp;R256)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="257">
+      <x:c r="R257" s="45" t="str">
+        <x:f>IF(OR(J257="",Q257&lt;&gt;""),"",COUNTIF($J$5:J257,J257))</x:f>
+      </x:c>
+      <x:c r="U257" s="45" t="str">
+        <x:f>IF(OR(J257="",Q257&lt;&gt;""),"",J257&amp;"|"&amp;R257)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="258">
+      <x:c r="R258" s="45" t="str">
+        <x:f>IF(OR(J258="",Q258&lt;&gt;""),"",COUNTIF($J$5:J258,J258))</x:f>
+      </x:c>
+      <x:c r="U258" s="45" t="str">
+        <x:f>IF(OR(J258="",Q258&lt;&gt;""),"",J258&amp;"|"&amp;R258)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="259">
+      <x:c r="R259" s="45" t="str">
+        <x:f>IF(OR(J259="",Q259&lt;&gt;""),"",COUNTIF($J$5:J259,J259))</x:f>
+      </x:c>
+      <x:c r="U259" s="45" t="str">
+        <x:f>IF(OR(J259="",Q259&lt;&gt;""),"",J259&amp;"|"&amp;R259)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="260">
+      <x:c r="R260" s="45" t="str">
+        <x:f>IF(OR(J260="",Q260&lt;&gt;""),"",COUNTIF($J$5:J260,J260))</x:f>
+      </x:c>
+      <x:c r="U260" s="45" t="str">
+        <x:f>IF(OR(J260="",Q260&lt;&gt;""),"",J260&amp;"|"&amp;R260)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="261">
+      <x:c r="R261" s="45" t="str">
+        <x:f>IF(OR(J261="",Q261&lt;&gt;""),"",COUNTIF($J$5:J261,J261))</x:f>
+      </x:c>
+      <x:c r="U261" s="45" t="str">
+        <x:f>IF(OR(J261="",Q261&lt;&gt;""),"",J261&amp;"|"&amp;R261)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="262">
+      <x:c r="R262" s="45" t="str">
+        <x:f>IF(OR(J262="",Q262&lt;&gt;""),"",COUNTIF($J$5:J262,J262))</x:f>
+      </x:c>
+      <x:c r="U262" s="45" t="str">
+        <x:f>IF(OR(J262="",Q262&lt;&gt;""),"",J262&amp;"|"&amp;R262)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="263">
+      <x:c r="R263" s="45" t="str">
+        <x:f>IF(OR(J263="",Q263&lt;&gt;""),"",COUNTIF($J$5:J263,J263))</x:f>
+      </x:c>
+      <x:c r="U263" s="45" t="str">
+        <x:f>IF(OR(J263="",Q263&lt;&gt;""),"",J263&amp;"|"&amp;R263)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="264">
+      <x:c r="R264" s="45" t="str">
+        <x:f>IF(OR(J264="",Q264&lt;&gt;""),"",COUNTIF($J$5:J264,J264))</x:f>
+      </x:c>
+      <x:c r="U264" s="45" t="str">
+        <x:f>IF(OR(J264="",Q264&lt;&gt;""),"",J264&amp;"|"&amp;R264)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="265">
+      <x:c r="R265" s="45" t="str">
+        <x:f>IF(OR(J265="",Q265&lt;&gt;""),"",COUNTIF($J$5:J265,J265))</x:f>
+      </x:c>
+      <x:c r="U265" s="45" t="str">
+        <x:f>IF(OR(J265="",Q265&lt;&gt;""),"",J265&amp;"|"&amp;R265)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="266">
+      <x:c r="R266" s="45" t="str">
+        <x:f>IF(OR(J266="",Q266&lt;&gt;""),"",COUNTIF($J$5:J266,J266))</x:f>
+      </x:c>
+      <x:c r="U266" s="45" t="str">
+        <x:f>IF(OR(J266="",Q266&lt;&gt;""),"",J266&amp;"|"&amp;R266)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="267">
+      <x:c r="R267" s="45" t="str">
+        <x:f>IF(OR(J267="",Q267&lt;&gt;""),"",COUNTIF($J$5:J267,J267))</x:f>
+      </x:c>
+      <x:c r="U267" s="45" t="str">
+        <x:f>IF(OR(J267="",Q267&lt;&gt;""),"",J267&amp;"|"&amp;R267)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="268">
+      <x:c r="R268" s="45" t="str">
+        <x:f>IF(OR(J268="",Q268&lt;&gt;""),"",COUNTIF($J$5:J268,J268))</x:f>
+      </x:c>
+      <x:c r="U268" s="45" t="str">
+        <x:f>IF(OR(J268="",Q268&lt;&gt;""),"",J268&amp;"|"&amp;R268)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="269">
+      <x:c r="R269" s="45" t="str">
+        <x:f>IF(OR(J269="",Q269&lt;&gt;""),"",COUNTIF($J$5:J269,J269))</x:f>
+      </x:c>
+      <x:c r="U269" s="45" t="str">
+        <x:f>IF(OR(J269="",Q269&lt;&gt;""),"",J269&amp;"|"&amp;R269)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="270">
+      <x:c r="R270" s="45" t="str">
+        <x:f>IF(OR(J270="",Q270&lt;&gt;""),"",COUNTIF($J$5:J270,J270))</x:f>
+      </x:c>
+      <x:c r="U270" s="45" t="str">
+        <x:f>IF(OR(J270="",Q270&lt;&gt;""),"",J270&amp;"|"&amp;R270)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="271">
+      <x:c r="R271" s="45" t="str">
+        <x:f>IF(OR(J271="",Q271&lt;&gt;""),"",COUNTIF($J$5:J271,J271))</x:f>
+      </x:c>
+      <x:c r="U271" s="45" t="str">
+        <x:f>IF(OR(J271="",Q271&lt;&gt;""),"",J271&amp;"|"&amp;R271)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="272">
+      <x:c r="R272" s="45" t="str">
+        <x:f>IF(OR(J272="",Q272&lt;&gt;""),"",COUNTIF($J$5:J272,J272))</x:f>
+      </x:c>
+      <x:c r="U272" s="45" t="str">
+        <x:f>IF(OR(J272="",Q272&lt;&gt;""),"",J272&amp;"|"&amp;R272)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="273">
+      <x:c r="R273" s="45" t="str">
+        <x:f>IF(OR(J273="",Q273&lt;&gt;""),"",COUNTIF($J$5:J273,J273))</x:f>
+      </x:c>
+      <x:c r="U273" s="45" t="str">
+        <x:f>IF(OR(J273="",Q273&lt;&gt;""),"",J273&amp;"|"&amp;R273)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="274">
+      <x:c r="R274" s="45" t="str">
+        <x:f>IF(OR(J274="",Q274&lt;&gt;""),"",COUNTIF($J$5:J274,J274))</x:f>
+      </x:c>
+      <x:c r="U274" s="45" t="str">
+        <x:f>IF(OR(J274="",Q274&lt;&gt;""),"",J274&amp;"|"&amp;R274)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="275">
+      <x:c r="R275" s="45" t="str">
+        <x:f>IF(OR(J275="",Q275&lt;&gt;""),"",COUNTIF($J$5:J275,J275))</x:f>
+      </x:c>
+      <x:c r="U275" s="45" t="str">
+        <x:f>IF(OR(J275="",Q275&lt;&gt;""),"",J275&amp;"|"&amp;R275)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="276">
+      <x:c r="R276" s="45" t="str">
+        <x:f>IF(OR(J276="",Q276&lt;&gt;""),"",COUNTIF($J$5:J276,J276))</x:f>
+      </x:c>
+      <x:c r="U276" s="45" t="str">
+        <x:f>IF(OR(J276="",Q276&lt;&gt;""),"",J276&amp;"|"&amp;R276)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="277">
+      <x:c r="R277" s="45" t="str">
+        <x:f>IF(OR(J277="",Q277&lt;&gt;""),"",COUNTIF($J$5:J277,J277))</x:f>
+      </x:c>
+      <x:c r="U277" s="45" t="str">
+        <x:f>IF(OR(J277="",Q277&lt;&gt;""),"",J277&amp;"|"&amp;R277)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="278">
+      <x:c r="R278" s="45" t="str">
+        <x:f>IF(OR(J278="",Q278&lt;&gt;""),"",COUNTIF($J$5:J278,J278))</x:f>
+      </x:c>
+      <x:c r="U278" s="45" t="str">
+        <x:f>IF(OR(J278="",Q278&lt;&gt;""),"",J278&amp;"|"&amp;R278)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="279">
+      <x:c r="R279" s="45" t="str">
+        <x:f>IF(OR(J279="",Q279&lt;&gt;""),"",COUNTIF($J$5:J279,J279))</x:f>
+      </x:c>
+      <x:c r="U279" s="45" t="str">
+        <x:f>IF(OR(J279="",Q279&lt;&gt;""),"",J279&amp;"|"&amp;R279)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="280">
+      <x:c r="R280" s="45" t="str">
+        <x:f>IF(OR(J280="",Q280&lt;&gt;""),"",COUNTIF($J$5:J280,J280))</x:f>
+      </x:c>
+      <x:c r="U280" s="45" t="str">
+        <x:f>IF(OR(J280="",Q280&lt;&gt;""),"",J280&amp;"|"&amp;R280)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="281">
+      <x:c r="R281" s="45" t="str">
+        <x:f>IF(OR(J281="",Q281&lt;&gt;""),"",COUNTIF($J$5:J281,J281))</x:f>
+      </x:c>
+      <x:c r="U281" s="45" t="str">
+        <x:f>IF(OR(J281="",Q281&lt;&gt;""),"",J281&amp;"|"&amp;R281)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="282">
+      <x:c r="R282" s="45" t="str">
+        <x:f>IF(OR(J282="",Q282&lt;&gt;""),"",COUNTIF($J$5:J282,J282))</x:f>
+      </x:c>
+      <x:c r="U282" s="45" t="str">
+        <x:f>IF(OR(J282="",Q282&lt;&gt;""),"",J282&amp;"|"&amp;R282)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="283">
+      <x:c r="R283" s="45" t="str">
+        <x:f>IF(OR(J283="",Q283&lt;&gt;""),"",COUNTIF($J$5:J283,J283))</x:f>
+      </x:c>
+      <x:c r="U283" s="45" t="str">
+        <x:f>IF(OR(J283="",Q283&lt;&gt;""),"",J283&amp;"|"&amp;R283)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="284">
+      <x:c r="R284" s="45" t="str">
+        <x:f>IF(OR(J284="",Q284&lt;&gt;""),"",COUNTIF($J$5:J284,J284))</x:f>
+      </x:c>
+      <x:c r="U284" s="45" t="str">
+        <x:f>IF(OR(J284="",Q284&lt;&gt;""),"",J284&amp;"|"&amp;R284)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="285">
+      <x:c r="R285" s="45" t="str">
+        <x:f>IF(OR(J285="",Q285&lt;&gt;""),"",COUNTIF($J$5:J285,J285))</x:f>
+      </x:c>
+      <x:c r="U285" s="45" t="str">
+        <x:f>IF(OR(J285="",Q285&lt;&gt;""),"",J285&amp;"|"&amp;R285)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="286">
+      <x:c r="R286" s="45" t="str">
+        <x:f>IF(OR(J286="",Q286&lt;&gt;""),"",COUNTIF($J$5:J286,J286))</x:f>
+      </x:c>
+      <x:c r="U286" s="45" t="str">
+        <x:f>IF(OR(J286="",Q286&lt;&gt;""),"",J286&amp;"|"&amp;R286)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="287">
+      <x:c r="R287" s="45" t="str">
+        <x:f>IF(OR(J287="",Q287&lt;&gt;""),"",COUNTIF($J$5:J287,J287))</x:f>
+      </x:c>
+      <x:c r="U287" s="45" t="str">
+        <x:f>IF(OR(J287="",Q287&lt;&gt;""),"",J287&amp;"|"&amp;R287)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="288">
+      <x:c r="R288" s="45" t="str">
+        <x:f>IF(OR(J288="",Q288&lt;&gt;""),"",COUNTIF($J$5:J288,J288))</x:f>
+      </x:c>
+      <x:c r="U288" s="45" t="str">
+        <x:f>IF(OR(J288="",Q288&lt;&gt;""),"",J288&amp;"|"&amp;R288)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="289">
+      <x:c r="R289" s="45" t="str">
+        <x:f>IF(OR(J289="",Q289&lt;&gt;""),"",COUNTIF($J$5:J289,J289))</x:f>
+      </x:c>
+      <x:c r="U289" s="45" t="str">
+        <x:f>IF(OR(J289="",Q289&lt;&gt;""),"",J289&amp;"|"&amp;R289)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="290">
+      <x:c r="R290" s="45" t="str">
+        <x:f>IF(OR(J290="",Q290&lt;&gt;""),"",COUNTIF($J$5:J290,J290))</x:f>
+      </x:c>
+      <x:c r="U290" s="45" t="str">
+        <x:f>IF(OR(J290="",Q290&lt;&gt;""),"",J290&amp;"|"&amp;R290)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="291">
+      <x:c r="R291" s="45" t="str">
+        <x:f>IF(OR(J291="",Q291&lt;&gt;""),"",COUNTIF($J$5:J291,J291))</x:f>
+      </x:c>
+      <x:c r="U291" s="45" t="str">
+        <x:f>IF(OR(J291="",Q291&lt;&gt;""),"",J291&amp;"|"&amp;R291)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="292">
+      <x:c r="R292" s="45" t="str">
+        <x:f>IF(OR(J292="",Q292&lt;&gt;""),"",COUNTIF($J$5:J292,J292))</x:f>
+      </x:c>
+      <x:c r="U292" s="45" t="str">
+        <x:f>IF(OR(J292="",Q292&lt;&gt;""),"",J292&amp;"|"&amp;R292)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="293">
+      <x:c r="R293" s="45" t="str">
+        <x:f>IF(OR(J293="",Q293&lt;&gt;""),"",COUNTIF($J$5:J293,J293))</x:f>
+      </x:c>
+      <x:c r="U293" s="45" t="str">
+        <x:f>IF(OR(J293="",Q293&lt;&gt;""),"",J293&amp;"|"&amp;R293)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="294">
+      <x:c r="R294" s="45" t="str">
+        <x:f>IF(OR(J294="",Q294&lt;&gt;""),"",COUNTIF($J$5:J294,J294))</x:f>
+      </x:c>
+      <x:c r="U294" s="45" t="str">
+        <x:f>IF(OR(J294="",Q294&lt;&gt;""),"",J294&amp;"|"&amp;R294)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="295">
+      <x:c r="R295" s="45" t="str">
+        <x:f>IF(OR(J295="",Q295&lt;&gt;""),"",COUNTIF($J$5:J295,J295))</x:f>
+      </x:c>
+      <x:c r="U295" s="45" t="str">
+        <x:f>IF(OR(J295="",Q295&lt;&gt;""),"",J295&amp;"|"&amp;R295)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="296">
+      <x:c r="R296" s="45" t="str">
+        <x:f>IF(OR(J296="",Q296&lt;&gt;""),"",COUNTIF($J$5:J296,J296))</x:f>
+      </x:c>
+      <x:c r="U296" s="45" t="str">
+        <x:f>IF(OR(J296="",Q296&lt;&gt;""),"",J296&amp;"|"&amp;R296)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="297">
+      <x:c r="R297" s="45" t="str">
+        <x:f>IF(OR(J297="",Q297&lt;&gt;""),"",COUNTIF($J$5:J297,J297))</x:f>
+      </x:c>
+      <x:c r="U297" s="45" t="str">
+        <x:f>IF(OR(J297="",Q297&lt;&gt;""),"",J297&amp;"|"&amp;R297)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="298">
+      <x:c r="R298" s="45" t="str">
+        <x:f>IF(OR(J298="",Q298&lt;&gt;""),"",COUNTIF($J$5:J298,J298))</x:f>
+      </x:c>
+      <x:c r="U298" s="45" t="str">
+        <x:f>IF(OR(J298="",Q298&lt;&gt;""),"",J298&amp;"|"&amp;R298)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="299">
+      <x:c r="R299" s="45" t="str">
+        <x:f>IF(OR(J299="",Q299&lt;&gt;""),"",COUNTIF($J$5:J299,J299))</x:f>
+      </x:c>
+      <x:c r="U299" s="45" t="str">
+        <x:f>IF(OR(J299="",Q299&lt;&gt;""),"",J299&amp;"|"&amp;R299)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="300">
+      <x:c r="R300" s="45" t="str">
+        <x:f>IF(OR(J300="",Q300&lt;&gt;""),"",COUNTIF($J$5:J300,J300))</x:f>
+      </x:c>
+      <x:c r="U300" s="45" t="str">
+        <x:f>IF(OR(J300="",Q300&lt;&gt;""),"",J300&amp;"|"&amp;R300)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="301">
+      <x:c r="R301" s="45" t="str">
+        <x:f>IF(OR(J301="",Q301&lt;&gt;""),"",COUNTIF($J$5:J301,J301))</x:f>
+      </x:c>
+      <x:c r="U301" s="45" t="str">
+        <x:f>IF(OR(J301="",Q301&lt;&gt;""),"",J301&amp;"|"&amp;R301)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="302">
+      <x:c r="R302" s="45" t="str">
+        <x:f>IF(OR(J302="",Q302&lt;&gt;""),"",COUNTIF($J$5:J302,J302))</x:f>
+      </x:c>
+      <x:c r="U302" s="45" t="str">
+        <x:f>IF(OR(J302="",Q302&lt;&gt;""),"",J302&amp;"|"&amp;R302)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="303">
+      <x:c r="R303" s="45" t="str">
+        <x:f>IF(OR(J303="",Q303&lt;&gt;""),"",COUNTIF($J$5:J303,J303))</x:f>
+      </x:c>
+      <x:c r="U303" s="45" t="str">
+        <x:f>IF(OR(J303="",Q303&lt;&gt;""),"",J303&amp;"|"&amp;R303)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="304">
+      <x:c r="R304" s="45" t="str">
+        <x:f>IF(OR(J304="",Q304&lt;&gt;""),"",COUNTIF($J$5:J304,J304))</x:f>
+      </x:c>
+      <x:c r="U304" s="45" t="str">
+        <x:f>IF(OR(J304="",Q304&lt;&gt;""),"",J304&amp;"|"&amp;R304)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="305">
+      <x:c r="R305" s="45" t="str">
+        <x:f>IF(OR(J305="",Q305&lt;&gt;""),"",COUNTIF($J$5:J305,J305))</x:f>
+      </x:c>
+      <x:c r="U305" s="45" t="str">
+        <x:f>IF(OR(J305="",Q305&lt;&gt;""),"",J305&amp;"|"&amp;R305)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="306">
+      <x:c r="R306" s="45" t="str">
+        <x:f>IF(OR(J306="",Q306&lt;&gt;""),"",COUNTIF($J$5:J306,J306))</x:f>
+      </x:c>
+      <x:c r="U306" s="45" t="str">
+        <x:f>IF(OR(J306="",Q306&lt;&gt;""),"",J306&amp;"|"&amp;R306)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="307">
+      <x:c r="R307" s="45" t="str">
+        <x:f>IF(OR(J307="",Q307&lt;&gt;""),"",COUNTIF($J$5:J307,J307))</x:f>
+      </x:c>
+      <x:c r="U307" s="45" t="str">
+        <x:f>IF(OR(J307="",Q307&lt;&gt;""),"",J307&amp;"|"&amp;R307)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="308">
+      <x:c r="R308" s="45" t="str">
+        <x:f>IF(OR(J308="",Q308&lt;&gt;""),"",COUNTIF($J$5:J308,J308))</x:f>
+      </x:c>
+      <x:c r="U308" s="45" t="str">
+        <x:f>IF(OR(J308="",Q308&lt;&gt;""),"",J308&amp;"|"&amp;R308)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="309">
+      <x:c r="R309" s="45" t="str">
+        <x:f>IF(OR(J309="",Q309&lt;&gt;""),"",COUNTIF($J$5:J309,J309))</x:f>
+      </x:c>
+      <x:c r="U309" s="45" t="str">
+        <x:f>IF(OR(J309="",Q309&lt;&gt;""),"",J309&amp;"|"&amp;R309)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="310">
+      <x:c r="R310" s="45" t="str">
+        <x:f>IF(OR(J310="",Q310&lt;&gt;""),"",COUNTIF($J$5:J310,J310))</x:f>
+      </x:c>
+      <x:c r="U310" s="45" t="str">
+        <x:f>IF(OR(J310="",Q310&lt;&gt;""),"",J310&amp;"|"&amp;R310)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="311">
+      <x:c r="R311" s="45" t="str">
+        <x:f>IF(OR(J311="",Q311&lt;&gt;""),"",COUNTIF($J$5:J311,J311))</x:f>
+      </x:c>
+      <x:c r="U311" s="45" t="str">
+        <x:f>IF(OR(J311="",Q311&lt;&gt;""),"",J311&amp;"|"&amp;R311)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="312">
+      <x:c r="R312" s="45" t="str">
+        <x:f>IF(OR(J312="",Q312&lt;&gt;""),"",COUNTIF($J$5:J312,J312))</x:f>
+      </x:c>
+      <x:c r="U312" s="45" t="str">
+        <x:f>IF(OR(J312="",Q312&lt;&gt;""),"",J312&amp;"|"&amp;R312)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="313">
+      <x:c r="R313" s="45" t="str">
+        <x:f>IF(OR(J313="",Q313&lt;&gt;""),"",COUNTIF($J$5:J313,J313))</x:f>
+      </x:c>
+      <x:c r="U313" s="45" t="str">
+        <x:f>IF(OR(J313="",Q313&lt;&gt;""),"",J313&amp;"|"&amp;R313)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="314">
+      <x:c r="R314" s="45" t="str">
+        <x:f>IF(OR(J314="",Q314&lt;&gt;""),"",COUNTIF($J$5:J314,J314))</x:f>
+      </x:c>
+      <x:c r="U314" s="45" t="str">
+        <x:f>IF(OR(J314="",Q314&lt;&gt;""),"",J314&amp;"|"&amp;R314)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="315">
+      <x:c r="R315" s="45" t="str">
+        <x:f>IF(OR(J315="",Q315&lt;&gt;""),"",COUNTIF($J$5:J315,J315))</x:f>
+      </x:c>
+      <x:c r="U315" s="45" t="str">
+        <x:f>IF(OR(J315="",Q315&lt;&gt;""),"",J315&amp;"|"&amp;R315)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="316">
+      <x:c r="R316" s="45" t="str">
+        <x:f>IF(OR(J316="",Q316&lt;&gt;""),"",COUNTIF($J$5:J316,J316))</x:f>
+      </x:c>
+      <x:c r="U316" s="45" t="str">
+        <x:f>IF(OR(J316="",Q316&lt;&gt;""),"",J316&amp;"|"&amp;R316)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="317">
+      <x:c r="R317" s="45" t="str">
+        <x:f>IF(OR(J317="",Q317&lt;&gt;""),"",COUNTIF($J$5:J317,J317))</x:f>
+      </x:c>
+      <x:c r="U317" s="45" t="str">
+        <x:f>IF(OR(J317="",Q317&lt;&gt;""),"",J317&amp;"|"&amp;R317)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="318">
+      <x:c r="R318" s="45" t="str">
+        <x:f>IF(OR(J318="",Q318&lt;&gt;""),"",COUNTIF($J$5:J318,J318))</x:f>
+      </x:c>
+      <x:c r="U318" s="45" t="str">
+        <x:f>IF(OR(J318="",Q318&lt;&gt;""),"",J318&amp;"|"&amp;R318)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="319">
+      <x:c r="R319" s="45" t="str">
+        <x:f>IF(OR(J319="",Q319&lt;&gt;""),"",COUNTIF($J$5:J319,J319))</x:f>
+      </x:c>
+      <x:c r="U319" s="45" t="str">
+        <x:f>IF(OR(J319="",Q319&lt;&gt;""),"",J319&amp;"|"&amp;R319)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="320">
+      <x:c r="R320" s="45" t="str">
+        <x:f>IF(OR(J320="",Q320&lt;&gt;""),"",COUNTIF($J$5:J320,J320))</x:f>
+      </x:c>
+      <x:c r="U320" s="45" t="str">
+        <x:f>IF(OR(J320="",Q320&lt;&gt;""),"",J320&amp;"|"&amp;R320)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="321">
+      <x:c r="R321" s="45" t="str">
+        <x:f>IF(OR(J321="",Q321&lt;&gt;""),"",COUNTIF($J$5:J321,J321))</x:f>
+      </x:c>
+      <x:c r="U321" s="45" t="str">
+        <x:f>IF(OR(J321="",Q321&lt;&gt;""),"",J321&amp;"|"&amp;R321)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="322">
+      <x:c r="R322" s="45" t="str">
+        <x:f>IF(OR(J322="",Q322&lt;&gt;""),"",COUNTIF($J$5:J322,J322))</x:f>
+      </x:c>
+      <x:c r="U322" s="45" t="str">
+        <x:f>IF(OR(J322="",Q322&lt;&gt;""),"",J322&amp;"|"&amp;R322)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="323">
+      <x:c r="R323" s="45" t="str">
+        <x:f>IF(OR(J323="",Q323&lt;&gt;""),"",COUNTIF($J$5:J323,J323))</x:f>
+      </x:c>
+      <x:c r="U323" s="45" t="str">
+        <x:f>IF(OR(J323="",Q323&lt;&gt;""),"",J323&amp;"|"&amp;R323)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="324">
+      <x:c r="R324" s="45" t="str">
+        <x:f>IF(OR(J324="",Q324&lt;&gt;""),"",COUNTIF($J$5:J324,J324))</x:f>
+      </x:c>
+      <x:c r="U324" s="45" t="str">
+        <x:f>IF(OR(J324="",Q324&lt;&gt;""),"",J324&amp;"|"&amp;R324)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="325">
+      <x:c r="R325" s="45" t="str">
+        <x:f>IF(OR(J325="",Q325&lt;&gt;""),"",COUNTIF($J$5:J325,J325))</x:f>
+      </x:c>
+      <x:c r="U325" s="45" t="str">
+        <x:f>IF(OR(J325="",Q325&lt;&gt;""),"",J325&amp;"|"&amp;R325)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="326">
+      <x:c r="R326" s="45" t="str">
+        <x:f>IF(OR(J326="",Q326&lt;&gt;""),"",COUNTIF($J$5:J326,J326))</x:f>
+      </x:c>
+      <x:c r="U326" s="45" t="str">
+        <x:f>IF(OR(J326="",Q326&lt;&gt;""),"",J326&amp;"|"&amp;R326)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="327">
+      <x:c r="R327" s="45" t="str">
+        <x:f>IF(OR(J327="",Q327&lt;&gt;""),"",COUNTIF($J$5:J327,J327))</x:f>
+      </x:c>
+      <x:c r="U327" s="45" t="str">
+        <x:f>IF(OR(J327="",Q327&lt;&gt;""),"",J327&amp;"|"&amp;R327)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="328">
+      <x:c r="R328" s="45" t="str">
+        <x:f>IF(OR(J328="",Q328&lt;&gt;""),"",COUNTIF($J$5:J328,J328))</x:f>
+      </x:c>
+      <x:c r="U328" s="45" t="str">
+        <x:f>IF(OR(J328="",Q328&lt;&gt;""),"",J328&amp;"|"&amp;R328)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="329">
+      <x:c r="R329" s="45" t="str">
+        <x:f>IF(OR(J329="",Q329&lt;&gt;""),"",COUNTIF($J$5:J329,J329))</x:f>
+      </x:c>
+      <x:c r="U329" s="45" t="str">
+        <x:f>IF(OR(J329="",Q329&lt;&gt;""),"",J329&amp;"|"&amp;R329)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="330">
+      <x:c r="R330" s="45" t="str">
+        <x:f>IF(OR(J330="",Q330&lt;&gt;""),"",COUNTIF($J$5:J330,J330))</x:f>
+      </x:c>
+      <x:c r="U330" s="45" t="str">
+        <x:f>IF(OR(J330="",Q330&lt;&gt;""),"",J330&amp;"|"&amp;R330)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="331">
+      <x:c r="R331" s="45" t="str">
+        <x:f>IF(OR(J331="",Q331&lt;&gt;""),"",COUNTIF($J$5:J331,J331))</x:f>
+      </x:c>
+      <x:c r="U331" s="45" t="str">
+        <x:f>IF(OR(J331="",Q331&lt;&gt;""),"",J331&amp;"|"&amp;R331)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="332">
+      <x:c r="R332" s="45" t="str">
+        <x:f>IF(OR(J332="",Q332&lt;&gt;""),"",COUNTIF($J$5:J332,J332))</x:f>
+      </x:c>
+      <x:c r="U332" s="45" t="str">
+        <x:f>IF(OR(J332="",Q332&lt;&gt;""),"",J332&amp;"|"&amp;R332)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="333">
+      <x:c r="R333" s="45" t="str">
+        <x:f>IF(OR(J333="",Q333&lt;&gt;""),"",COUNTIF($J$5:J333,J333))</x:f>
+      </x:c>
+      <x:c r="U333" s="45" t="str">
+        <x:f>IF(OR(J333="",Q333&lt;&gt;""),"",J333&amp;"|"&amp;R333)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="334">
+      <x:c r="R334" s="45" t="str">
+        <x:f>IF(OR(J334="",Q334&lt;&gt;""),"",COUNTIF($J$5:J334,J334))</x:f>
+      </x:c>
+      <x:c r="U334" s="45" t="str">
+        <x:f>IF(OR(J334="",Q334&lt;&gt;""),"",J334&amp;"|"&amp;R334)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="335">
+      <x:c r="R335" s="45" t="str">
+        <x:f>IF(OR(J335="",Q335&lt;&gt;""),"",COUNTIF($J$5:J335,J335))</x:f>
+      </x:c>
+      <x:c r="U335" s="45" t="str">
+        <x:f>IF(OR(J335="",Q335&lt;&gt;""),"",J335&amp;"|"&amp;R335)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="336">
+      <x:c r="R336" s="45" t="str">
+        <x:f>IF(OR(J336="",Q336&lt;&gt;""),"",COUNTIF($J$5:J336,J336))</x:f>
+      </x:c>
+      <x:c r="U336" s="45" t="str">
+        <x:f>IF(OR(J336="",Q336&lt;&gt;""),"",J336&amp;"|"&amp;R336)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="337">
+      <x:c r="R337" s="45" t="str">
+        <x:f>IF(OR(J337="",Q337&lt;&gt;""),"",COUNTIF($J$5:J337,J337))</x:f>
+      </x:c>
+      <x:c r="U337" s="45" t="str">
+        <x:f>IF(OR(J337="",Q337&lt;&gt;""),"",J337&amp;"|"&amp;R337)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="338">
+      <x:c r="R338" s="45" t="str">
+        <x:f>IF(OR(J338="",Q338&lt;&gt;""),"",COUNTIF($J$5:J338,J338))</x:f>
+      </x:c>
+      <x:c r="U338" s="45" t="str">
+        <x:f>IF(OR(J338="",Q338&lt;&gt;""),"",J338&amp;"|"&amp;R338)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="339">
+      <x:c r="R339" s="45" t="str">
+        <x:f>IF(OR(J339="",Q339&lt;&gt;""),"",COUNTIF($J$5:J339,J339))</x:f>
+      </x:c>
+      <x:c r="U339" s="45" t="str">
+        <x:f>IF(OR(J339="",Q339&lt;&gt;""),"",J339&amp;"|"&amp;R339)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="340">
+      <x:c r="R340" s="45" t="str">
+        <x:f>IF(OR(J340="",Q340&lt;&gt;""),"",COUNTIF($J$5:J340,J340))</x:f>
+      </x:c>
+      <x:c r="U340" s="45" t="str">
+        <x:f>IF(OR(J340="",Q340&lt;&gt;""),"",J340&amp;"|"&amp;R340)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="341">
+      <x:c r="R341" s="45" t="str">
+        <x:f>IF(OR(J341="",Q341&lt;&gt;""),"",COUNTIF($J$5:J341,J341))</x:f>
+      </x:c>
+      <x:c r="U341" s="45" t="str">
+        <x:f>IF(OR(J341="",Q341&lt;&gt;""),"",J341&amp;"|"&amp;R341)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="342">
+      <x:c r="R342" s="45" t="str">
+        <x:f>IF(OR(J342="",Q342&lt;&gt;""),"",COUNTIF($J$5:J342,J342))</x:f>
+      </x:c>
+      <x:c r="U342" s="45" t="str">
+        <x:f>IF(OR(J342="",Q342&lt;&gt;""),"",J342&amp;"|"&amp;R342)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="343">
+      <x:c r="R343" s="45" t="str">
+        <x:f>IF(OR(J343="",Q343&lt;&gt;""),"",COUNTIF($J$5:J343,J343))</x:f>
+      </x:c>
+      <x:c r="U343" s="45" t="str">
+        <x:f>IF(OR(J343="",Q343&lt;&gt;""),"",J343&amp;"|"&amp;R343)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="344">
+      <x:c r="R344" s="45" t="str">
+        <x:f>IF(OR(J344="",Q344&lt;&gt;""),"",COUNTIF($J$5:J344,J344))</x:f>
+      </x:c>
+      <x:c r="U344" s="45" t="str">
+        <x:f>IF(OR(J344="",Q344&lt;&gt;""),"",J344&amp;"|"&amp;R344)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="345">
+      <x:c r="R345" s="45" t="str">
+        <x:f>IF(OR(J345="",Q345&lt;&gt;""),"",COUNTIF($J$5:J345,J345))</x:f>
+      </x:c>
+      <x:c r="U345" s="45" t="str">
+        <x:f>IF(OR(J345="",Q345&lt;&gt;""),"",J345&amp;"|"&amp;R345)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="346">
+      <x:c r="R346" s="45" t="str">
+        <x:f>IF(OR(J346="",Q346&lt;&gt;""),"",COUNTIF($J$5:J346,J346))</x:f>
+      </x:c>
+      <x:c r="U346" s="45" t="str">
+        <x:f>IF(OR(J346="",Q346&lt;&gt;""),"",J346&amp;"|"&amp;R346)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="347">
+      <x:c r="R347" s="45" t="str">
+        <x:f>IF(OR(J347="",Q347&lt;&gt;""),"",COUNTIF($J$5:J347,J347))</x:f>
+      </x:c>
+      <x:c r="U347" s="45" t="str">
+        <x:f>IF(OR(J347="",Q347&lt;&gt;""),"",J347&amp;"|"&amp;R347)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="348">
+      <x:c r="R348" s="45" t="str">
+        <x:f>IF(OR(J348="",Q348&lt;&gt;""),"",COUNTIF($J$5:J348,J348))</x:f>
+      </x:c>
+      <x:c r="U348" s="45" t="str">
+        <x:f>IF(OR(J348="",Q348&lt;&gt;""),"",J348&amp;"|"&amp;R348)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="349">
+      <x:c r="R349" s="45" t="str">
+        <x:f>IF(OR(J349="",Q349&lt;&gt;""),"",COUNTIF($J$5:J349,J349))</x:f>
+      </x:c>
+      <x:c r="U349" s="45" t="str">
+        <x:f>IF(OR(J349="",Q349&lt;&gt;""),"",J349&amp;"|"&amp;R349)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="350">
+      <x:c r="R350" s="45" t="str">
+        <x:f>IF(OR(J350="",Q350&lt;&gt;""),"",COUNTIF($J$5:J350,J350))</x:f>
+      </x:c>
+      <x:c r="U350" s="45" t="str">
+        <x:f>IF(OR(J350="",Q350&lt;&gt;""),"",J350&amp;"|"&amp;R350)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="351">
+      <x:c r="R351" s="45" t="str">
+        <x:f>IF(OR(J351="",Q351&lt;&gt;""),"",COUNTIF($J$5:J351,J351))</x:f>
+      </x:c>
+      <x:c r="U351" s="45" t="str">
+        <x:f>IF(OR(J351="",Q351&lt;&gt;""),"",J351&amp;"|"&amp;R351)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="352">
+      <x:c r="R352" s="45" t="str">
+        <x:f>IF(OR(J352="",Q352&lt;&gt;""),"",COUNTIF($J$5:J352,J352))</x:f>
+      </x:c>
+      <x:c r="U352" s="45" t="str">
+        <x:f>IF(OR(J352="",Q352&lt;&gt;""),"",J352&amp;"|"&amp;R352)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="353">
+      <x:c r="R353" s="45" t="str">
+        <x:f>IF(OR(J353="",Q353&lt;&gt;""),"",COUNTIF($J$5:J353,J353))</x:f>
+      </x:c>
+      <x:c r="U353" s="45" t="str">
+        <x:f>IF(OR(J353="",Q353&lt;&gt;""),"",J353&amp;"|"&amp;R353)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="354">
+      <x:c r="R354" s="45" t="str">
+        <x:f>IF(OR(J354="",Q354&lt;&gt;""),"",COUNTIF($J$5:J354,J354))</x:f>
+      </x:c>
+      <x:c r="U354" s="45" t="str">
+        <x:f>IF(OR(J354="",Q354&lt;&gt;""),"",J354&amp;"|"&amp;R354)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="355">
+      <x:c r="R355" s="45" t="str">
+        <x:f>IF(OR(J355="",Q355&lt;&gt;""),"",COUNTIF($J$5:J355,J355))</x:f>
+      </x:c>
+      <x:c r="U355" s="45" t="str">
+        <x:f>IF(OR(J355="",Q355&lt;&gt;""),"",J355&amp;"|"&amp;R355)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="356">
+      <x:c r="R356" s="45" t="str">
+        <x:f>IF(OR(J356="",Q356&lt;&gt;""),"",COUNTIF($J$5:J356,J356))</x:f>
+      </x:c>
+      <x:c r="U356" s="45" t="str">
+        <x:f>IF(OR(J356="",Q356&lt;&gt;""),"",J356&amp;"|"&amp;R356)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="357">
+      <x:c r="R357" s="45" t="str">
+        <x:f>IF(OR(J357="",Q357&lt;&gt;""),"",COUNTIF($J$5:J357,J357))</x:f>
+      </x:c>
+      <x:c r="U357" s="45" t="str">
+        <x:f>IF(OR(J357="",Q357&lt;&gt;""),"",J357&amp;"|"&amp;R357)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="358">
+      <x:c r="R358" s="45" t="str">
+        <x:f>IF(OR(J358="",Q358&lt;&gt;""),"",COUNTIF($J$5:J358,J358))</x:f>
+      </x:c>
+      <x:c r="U358" s="45" t="str">
+        <x:f>IF(OR(J358="",Q358&lt;&gt;""),"",J358&amp;"|"&amp;R358)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="359">
+      <x:c r="R359" s="45" t="str">
+        <x:f>IF(OR(J359="",Q359&lt;&gt;""),"",COUNTIF($J$5:J359,J359))</x:f>
+      </x:c>
+      <x:c r="U359" s="45" t="str">
+        <x:f>IF(OR(J359="",Q359&lt;&gt;""),"",J359&amp;"|"&amp;R359)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="360">
+      <x:c r="R360" s="45" t="str">
+        <x:f>IF(OR(J360="",Q360&lt;&gt;""),"",COUNTIF($J$5:J360,J360))</x:f>
+      </x:c>
+      <x:c r="U360" s="45" t="str">
+        <x:f>IF(OR(J360="",Q360&lt;&gt;""),"",J360&amp;"|"&amp;R360)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="361">
+      <x:c r="R361" s="45" t="str">
+        <x:f>IF(OR(J361="",Q361&lt;&gt;""),"",COUNTIF($J$5:J361,J361))</x:f>
+      </x:c>
+      <x:c r="U361" s="45" t="str">
+        <x:f>IF(OR(J361="",Q361&lt;&gt;""),"",J361&amp;"|"&amp;R361)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="362">
+      <x:c r="R362" s="45" t="str">
+        <x:f>IF(OR(J362="",Q362&lt;&gt;""),"",COUNTIF($J$5:J362,J362))</x:f>
+      </x:c>
+      <x:c r="U362" s="45" t="str">
+        <x:f>IF(OR(J362="",Q362&lt;&gt;""),"",J362&amp;"|"&amp;R362)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="363">
+      <x:c r="R363" s="45" t="str">
+        <x:f>IF(OR(J363="",Q363&lt;&gt;""),"",COUNTIF($J$5:J363,J363))</x:f>
+      </x:c>
+      <x:c r="U363" s="45" t="str">
+        <x:f>IF(OR(J363="",Q363&lt;&gt;""),"",J363&amp;"|"&amp;R363)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="364">
+      <x:c r="R364" s="45" t="str">
+        <x:f>IF(OR(J364="",Q364&lt;&gt;""),"",COUNTIF($J$5:J364,J364))</x:f>
+      </x:c>
+      <x:c r="U364" s="45" t="str">
+        <x:f>IF(OR(J364="",Q364&lt;&gt;""),"",J364&amp;"|"&amp;R364)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="365">
+      <x:c r="R365" s="45" t="str">
+        <x:f>IF(OR(J365="",Q365&lt;&gt;""),"",COUNTIF($J$5:J365,J365))</x:f>
+      </x:c>
+      <x:c r="U365" s="45" t="str">
+        <x:f>IF(OR(J365="",Q365&lt;&gt;""),"",J365&amp;"|"&amp;R365)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="366">
+      <x:c r="R366" s="45" t="str">
+        <x:f>IF(OR(J366="",Q366&lt;&gt;""),"",COUNTIF($J$5:J366,J366))</x:f>
+      </x:c>
+      <x:c r="U366" s="45" t="str">
+        <x:f>IF(OR(J366="",Q366&lt;&gt;""),"",J366&amp;"|"&amp;R366)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="367">
+      <x:c r="R367" s="45" t="str">
+        <x:f>IF(OR(J367="",Q367&lt;&gt;""),"",COUNTIF($J$5:J367,J367))</x:f>
+      </x:c>
+      <x:c r="U367" s="45" t="str">
+        <x:f>IF(OR(J367="",Q367&lt;&gt;""),"",J367&amp;"|"&amp;R367)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="368">
+      <x:c r="R368" s="45" t="str">
+        <x:f>IF(OR(J368="",Q368&lt;&gt;""),"",COUNTIF($J$5:J368,J368))</x:f>
+      </x:c>
+      <x:c r="U368" s="45" t="str">
+        <x:f>IF(OR(J368="",Q368&lt;&gt;""),"",J368&amp;"|"&amp;R368)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="369">
+      <x:c r="R369" s="45" t="str">
+        <x:f>IF(OR(J369="",Q369&lt;&gt;""),"",COUNTIF($J$5:J369,J369))</x:f>
+      </x:c>
+      <x:c r="U369" s="45" t="str">
+        <x:f>IF(OR(J369="",Q369&lt;&gt;""),"",J369&amp;"|"&amp;R369)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="370">
+      <x:c r="R370" s="45" t="str">
+        <x:f>IF(OR(J370="",Q370&lt;&gt;""),"",COUNTIF($J$5:J370,J370))</x:f>
+      </x:c>
+      <x:c r="U370" s="45" t="str">
+        <x:f>IF(OR(J370="",Q370&lt;&gt;""),"",J370&amp;"|"&amp;R370)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="371">
+      <x:c r="R371" s="45" t="str">
+        <x:f>IF(OR(J371="",Q371&lt;&gt;""),"",COUNTIF($J$5:J371,J371))</x:f>
+      </x:c>
+      <x:c r="U371" s="45" t="str">
+        <x:f>IF(OR(J371="",Q371&lt;&gt;""),"",J371&amp;"|"&amp;R371)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="372">
+      <x:c r="R372" s="45" t="str">
+        <x:f>IF(OR(J372="",Q372&lt;&gt;""),"",COUNTIF($J$5:J372,J372))</x:f>
+      </x:c>
+      <x:c r="U372" s="45" t="str">
+        <x:f>IF(OR(J372="",Q372&lt;&gt;""),"",J372&amp;"|"&amp;R372)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="373">
+      <x:c r="R373" s="45" t="str">
+        <x:f>IF(OR(J373="",Q373&lt;&gt;""),"",COUNTIF($J$5:J373,J373))</x:f>
+      </x:c>
+      <x:c r="U373" s="45" t="str">
+        <x:f>IF(OR(J373="",Q373&lt;&gt;""),"",J373&amp;"|"&amp;R373)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="374">
+      <x:c r="R374" s="45" t="str">
+        <x:f>IF(OR(J374="",Q374&lt;&gt;""),"",COUNTIF($J$5:J374,J374))</x:f>
+      </x:c>
+      <x:c r="U374" s="45" t="str">
+        <x:f>IF(OR(J374="",Q374&lt;&gt;""),"",J374&amp;"|"&amp;R374)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="375">
+      <x:c r="R375" s="45" t="str">
+        <x:f>IF(OR(J375="",Q375&lt;&gt;""),"",COUNTIF($J$5:J375,J375))</x:f>
+      </x:c>
+      <x:c r="U375" s="45" t="str">
+        <x:f>IF(OR(J375="",Q375&lt;&gt;""),"",J375&amp;"|"&amp;R375)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="376">
+      <x:c r="R376" s="45" t="str">
+        <x:f>IF(OR(J376="",Q376&lt;&gt;""),"",COUNTIF($J$5:J376,J376))</x:f>
+      </x:c>
+      <x:c r="U376" s="45" t="str">
+        <x:f>IF(OR(J376="",Q376&lt;&gt;""),"",J376&amp;"|"&amp;R376)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="377">
+      <x:c r="R377" s="45" t="str">
+        <x:f>IF(OR(J377="",Q377&lt;&gt;""),"",COUNTIF($J$5:J377,J377))</x:f>
+      </x:c>
+      <x:c r="U377" s="45" t="str">
+        <x:f>IF(OR(J377="",Q377&lt;&gt;""),"",J377&amp;"|"&amp;R377)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="378">
+      <x:c r="R378" s="45" t="str">
+        <x:f>IF(OR(J378="",Q378&lt;&gt;""),"",COUNTIF($J$5:J378,J378))</x:f>
+      </x:c>
+      <x:c r="U378" s="45" t="str">
+        <x:f>IF(OR(J378="",Q378&lt;&gt;""),"",J378&amp;"|"&amp;R378)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="379">
+      <x:c r="R379" s="45" t="str">
+        <x:f>IF(OR(J379="",Q379&lt;&gt;""),"",COUNTIF($J$5:J379,J379))</x:f>
+      </x:c>
+      <x:c r="U379" s="45" t="str">
+        <x:f>IF(OR(J379="",Q379&lt;&gt;""),"",J379&amp;"|"&amp;R379)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="380">
+      <x:c r="R380" s="45" t="str">
+        <x:f>IF(OR(J380="",Q380&lt;&gt;""),"",COUNTIF($J$5:J380,J380))</x:f>
+      </x:c>
+      <x:c r="U380" s="45" t="str">
+        <x:f>IF(OR(J380="",Q380&lt;&gt;""),"",J380&amp;"|"&amp;R380)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="381">
+      <x:c r="R381" s="45" t="str">
+        <x:f>IF(OR(J381="",Q381&lt;&gt;""),"",COUNTIF($J$5:J381,J381))</x:f>
+      </x:c>
+      <x:c r="U381" s="45" t="str">
+        <x:f>IF(OR(J381="",Q381&lt;&gt;""),"",J381&amp;"|"&amp;R381)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="382">
+      <x:c r="R382" s="45" t="str">
+        <x:f>IF(OR(J382="",Q382&lt;&gt;""),"",COUNTIF($J$5:J382,J382))</x:f>
+      </x:c>
+      <x:c r="U382" s="45" t="str">
+        <x:f>IF(OR(J382="",Q382&lt;&gt;""),"",J382&amp;"|"&amp;R382)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="383">
+      <x:c r="R383" s="45" t="str">
+        <x:f>IF(OR(J383="",Q383&lt;&gt;""),"",COUNTIF($J$5:J383,J383))</x:f>
+      </x:c>
+      <x:c r="U383" s="45" t="str">
+        <x:f>IF(OR(J383="",Q383&lt;&gt;""),"",J383&amp;"|"&amp;R383)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="384">
+      <x:c r="R384" s="45" t="str">
+        <x:f>IF(OR(J384="",Q384&lt;&gt;""),"",COUNTIF($J$5:J384,J384))</x:f>
+      </x:c>
+      <x:c r="U384" s="45" t="str">
+        <x:f>IF(OR(J384="",Q384&lt;&gt;""),"",J384&amp;"|"&amp;R384)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="385">
+      <x:c r="R385" s="45" t="str">
+        <x:f>IF(OR(J385="",Q385&lt;&gt;""),"",COUNTIF($J$5:J385,J385))</x:f>
+      </x:c>
+      <x:c r="U385" s="45" t="str">
+        <x:f>IF(OR(J385="",Q385&lt;&gt;""),"",J385&amp;"|"&amp;R385)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="386">
+      <x:c r="R386" s="45" t="str">
+        <x:f>IF(OR(J386="",Q386&lt;&gt;""),"",COUNTIF($J$5:J386,J386))</x:f>
+      </x:c>
+      <x:c r="U386" s="45" t="str">
+        <x:f>IF(OR(J386="",Q386&lt;&gt;""),"",J386&amp;"|"&amp;R386)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="387">
+      <x:c r="R387" s="45" t="str">
+        <x:f>IF(OR(J387="",Q387&lt;&gt;""),"",COUNTIF($J$5:J387,J387))</x:f>
+      </x:c>
+      <x:c r="U387" s="45" t="str">
+        <x:f>IF(OR(J387="",Q387&lt;&gt;""),"",J387&amp;"|"&amp;R387)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="388">
+      <x:c r="R388" s="45" t="str">
+        <x:f>IF(OR(J388="",Q388&lt;&gt;""),"",COUNTIF($J$5:J388,J388))</x:f>
+      </x:c>
+      <x:c r="U388" s="45" t="str">
+        <x:f>IF(OR(J388="",Q388&lt;&gt;""),"",J388&amp;"|"&amp;R388)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="389">
+      <x:c r="R389" s="45" t="str">
+        <x:f>IF(OR(J389="",Q389&lt;&gt;""),"",COUNTIF($J$5:J389,J389))</x:f>
+      </x:c>
+      <x:c r="U389" s="45" t="str">
+        <x:f>IF(OR(J389="",Q389&lt;&gt;""),"",J389&amp;"|"&amp;R389)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="390">
+      <x:c r="R390" s="45" t="str">
+        <x:f>IF(OR(J390="",Q390&lt;&gt;""),"",COUNTIF($J$5:J390,J390))</x:f>
+      </x:c>
+      <x:c r="U390" s="45" t="str">
+        <x:f>IF(OR(J390="",Q390&lt;&gt;""),"",J390&amp;"|"&amp;R390)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="391">
+      <x:c r="R391" s="45" t="str">
+        <x:f>IF(OR(J391="",Q391&lt;&gt;""),"",COUNTIF($J$5:J391,J391))</x:f>
+      </x:c>
+      <x:c r="U391" s="45" t="str">
+        <x:f>IF(OR(J391="",Q391&lt;&gt;""),"",J391&amp;"|"&amp;R391)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="392">
+      <x:c r="R392" s="45" t="str">
+        <x:f>IF(OR(J392="",Q392&lt;&gt;""),"",COUNTIF($J$5:J392,J392))</x:f>
+      </x:c>
+      <x:c r="U392" s="45" t="str">
+        <x:f>IF(OR(J392="",Q392&lt;&gt;""),"",J392&amp;"|"&amp;R392)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="393">
+      <x:c r="R393" s="45" t="str">
+        <x:f>IF(OR(J393="",Q393&lt;&gt;""),"",COUNTIF($J$5:J393,J393))</x:f>
+      </x:c>
+      <x:c r="U393" s="45" t="str">
+        <x:f>IF(OR(J393="",Q393&lt;&gt;""),"",J393&amp;"|"&amp;R393)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="394">
+      <x:c r="R394" s="45" t="str">
+        <x:f>IF(OR(J394="",Q394&lt;&gt;""),"",COUNTIF($J$5:J394,J394))</x:f>
+      </x:c>
+      <x:c r="U394" s="45" t="str">
+        <x:f>IF(OR(J394="",Q394&lt;&gt;""),"",J394&amp;"|"&amp;R394)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="395">
+      <x:c r="R395" s="45" t="str">
+        <x:f>IF(OR(J395="",Q395&lt;&gt;""),"",COUNTIF($J$5:J395,J395))</x:f>
+      </x:c>
+      <x:c r="U395" s="45" t="str">
+        <x:f>IF(OR(J395="",Q395&lt;&gt;""),"",J395&amp;"|"&amp;R395)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="396">
+      <x:c r="R396" s="45" t="str">
+        <x:f>IF(OR(J396="",Q396&lt;&gt;""),"",COUNTIF($J$5:J396,J396))</x:f>
+      </x:c>
+      <x:c r="U396" s="45" t="str">
+        <x:f>IF(OR(J396="",Q396&lt;&gt;""),"",J396&amp;"|"&amp;R396)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="397">
+      <x:c r="R397" s="45" t="str">
+        <x:f>IF(OR(J397="",Q397&lt;&gt;""),"",COUNTIF($J$5:J397,J397))</x:f>
+      </x:c>
+      <x:c r="U397" s="45" t="str">
+        <x:f>IF(OR(J397="",Q397&lt;&gt;""),"",J397&amp;"|"&amp;R397)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="398">
+      <x:c r="R398" s="45" t="str">
+        <x:f>IF(OR(J398="",Q398&lt;&gt;""),"",COUNTIF($J$5:J398,J398))</x:f>
+      </x:c>
+      <x:c r="U398" s="45" t="str">
+        <x:f>IF(OR(J398="",Q398&lt;&gt;""),"",J398&amp;"|"&amp;R398)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="399">
+      <x:c r="R399" s="45" t="str">
+        <x:f>IF(OR(J399="",Q399&lt;&gt;""),"",COUNTIF($J$5:J399,J399))</x:f>
+      </x:c>
+      <x:c r="U399" s="45" t="str">
+        <x:f>IF(OR(J399="",Q399&lt;&gt;""),"",J399&amp;"|"&amp;R399)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="400">
+      <x:c r="R400" s="45" t="str">
+        <x:f>IF(OR(J400="",Q400&lt;&gt;""),"",COUNTIF($J$5:J400,J400))</x:f>
+      </x:c>
+      <x:c r="U400" s="45" t="str">
+        <x:f>IF(OR(J400="",Q400&lt;&gt;""),"",J400&amp;"|"&amp;R400)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="401">
+      <x:c r="R401" s="45" t="str">
+        <x:f>IF(OR(J401="",Q401&lt;&gt;""),"",COUNTIF($J$5:J401,J401))</x:f>
+      </x:c>
+      <x:c r="U401" s="45" t="str">
+        <x:f>IF(OR(J401="",Q401&lt;&gt;""),"",J401&amp;"|"&amp;R401)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="402">
+      <x:c r="R402" s="45" t="str">
+        <x:f>IF(OR(J402="",Q402&lt;&gt;""),"",COUNTIF($J$5:J402,J402))</x:f>
+      </x:c>
+      <x:c r="U402" s="45" t="str">
+        <x:f>IF(OR(J402="",Q402&lt;&gt;""),"",J402&amp;"|"&amp;R402)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="403">
+      <x:c r="R403" s="45" t="str">
+        <x:f>IF(OR(J403="",Q403&lt;&gt;""),"",COUNTIF($J$5:J403,J403))</x:f>
+      </x:c>
+      <x:c r="U403" s="45" t="str">
+        <x:f>IF(OR(J403="",Q403&lt;&gt;""),"",J403&amp;"|"&amp;R403)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="404">
+      <x:c r="R404" s="45" t="str">
+        <x:f>IF(OR(J404="",Q404&lt;&gt;""),"",COUNTIF($J$5:J404,J404))</x:f>
+      </x:c>
+      <x:c r="U404" s="45" t="str">
+        <x:f>IF(OR(J404="",Q404&lt;&gt;""),"",J404&amp;"|"&amp;R404)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="405">
+      <x:c r="R405" s="45" t="str">
+        <x:f>IF(OR(J405="",Q405&lt;&gt;""),"",COUNTIF($J$5:J405,J405))</x:f>
+      </x:c>
+      <x:c r="U405" s="45" t="str">
+        <x:f>IF(OR(J405="",Q405&lt;&gt;""),"",J405&amp;"|"&amp;R405)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="406">
+      <x:c r="R406" s="45" t="str">
+        <x:f>IF(OR(J406="",Q406&lt;&gt;""),"",COUNTIF($J$5:J406,J406))</x:f>
+      </x:c>
+      <x:c r="U406" s="45" t="str">
+        <x:f>IF(OR(J406="",Q406&lt;&gt;""),"",J406&amp;"|"&amp;R406)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="407">
+      <x:c r="R407" s="45" t="str">
+        <x:f>IF(OR(J407="",Q407&lt;&gt;""),"",COUNTIF($J$5:J407,J407))</x:f>
+      </x:c>
+      <x:c r="U407" s="45" t="str">
+        <x:f>IF(OR(J407="",Q407&lt;&gt;""),"",J407&amp;"|"&amp;R407)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="408">
+      <x:c r="R408" s="45" t="str">
+        <x:f>IF(OR(J408="",Q408&lt;&gt;""),"",COUNTIF($J$5:J408,J408))</x:f>
+      </x:c>
+      <x:c r="U408" s="45" t="str">
+        <x:f>IF(OR(J408="",Q408&lt;&gt;""),"",J408&amp;"|"&amp;R408)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="409">
+      <x:c r="R409" s="45" t="str">
+        <x:f>IF(OR(J409="",Q409&lt;&gt;""),"",COUNTIF($J$5:J409,J409))</x:f>
+      </x:c>
+      <x:c r="U409" s="45" t="str">
+        <x:f>IF(OR(J409="",Q409&lt;&gt;""),"",J409&amp;"|"&amp;R409)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="410">
+      <x:c r="R410" s="45" t="str">
+        <x:f>IF(OR(J410="",Q410&lt;&gt;""),"",COUNTIF($J$5:J410,J410))</x:f>
+      </x:c>
+      <x:c r="U410" s="45" t="str">
+        <x:f>IF(OR(J410="",Q410&lt;&gt;""),"",J410&amp;"|"&amp;R410)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="411">
+      <x:c r="R411" s="45" t="str">
+        <x:f>IF(OR(J411="",Q411&lt;&gt;""),"",COUNTIF($J$5:J411,J411))</x:f>
+      </x:c>
+      <x:c r="U411" s="45" t="str">
+        <x:f>IF(OR(J411="",Q411&lt;&gt;""),"",J411&amp;"|"&amp;R411)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="412">
+      <x:c r="R412" s="45" t="str">
+        <x:f>IF(OR(J412="",Q412&lt;&gt;""),"",COUNTIF($J$5:J412,J412))</x:f>
+      </x:c>
+      <x:c r="U412" s="45" t="str">
+        <x:f>IF(OR(J412="",Q412&lt;&gt;""),"",J412&amp;"|"&amp;R412)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="413">
+      <x:c r="R413" s="45" t="str">
+        <x:f>IF(OR(J413="",Q413&lt;&gt;""),"",COUNTIF($J$5:J413,J413))</x:f>
+      </x:c>
+      <x:c r="U413" s="45" t="str">
+        <x:f>IF(OR(J413="",Q413&lt;&gt;""),"",J413&amp;"|"&amp;R413)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="414">
+      <x:c r="R414" s="45" t="str">
+        <x:f>IF(OR(J414="",Q414&lt;&gt;""),"",COUNTIF($J$5:J414,J414))</x:f>
+      </x:c>
+      <x:c r="U414" s="45" t="str">
+        <x:f>IF(OR(J414="",Q414&lt;&gt;""),"",J414&amp;"|"&amp;R414)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="415">
+      <x:c r="R415" s="45" t="str">
+        <x:f>IF(OR(J415="",Q415&lt;&gt;""),"",COUNTIF($J$5:J415,J415))</x:f>
+      </x:c>
+      <x:c r="U415" s="45" t="str">
+        <x:f>IF(OR(J415="",Q415&lt;&gt;""),"",J415&amp;"|"&amp;R415)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="416">
+      <x:c r="R416" s="45" t="str">
+        <x:f>IF(OR(J416="",Q416&lt;&gt;""),"",COUNTIF($J$5:J416,J416))</x:f>
+      </x:c>
+      <x:c r="U416" s="45" t="str">
+        <x:f>IF(OR(J416="",Q416&lt;&gt;""),"",J416&amp;"|"&amp;R416)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="417">
+      <x:c r="R417" s="45" t="str">
+        <x:f>IF(OR(J417="",Q417&lt;&gt;""),"",COUNTIF($J$5:J417,J417))</x:f>
+      </x:c>
+      <x:c r="U417" s="45" t="str">
+        <x:f>IF(OR(J417="",Q417&lt;&gt;""),"",J417&amp;"|"&amp;R417)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="418">
+      <x:c r="R418" s="45" t="str">
+        <x:f>IF(OR(J418="",Q418&lt;&gt;""),"",COUNTIF($J$5:J418,J418))</x:f>
+      </x:c>
+      <x:c r="U418" s="45" t="str">
+        <x:f>IF(OR(J418="",Q418&lt;&gt;""),"",J418&amp;"|"&amp;R418)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="419">
+      <x:c r="R419" s="45" t="str">
+        <x:f>IF(OR(J419="",Q419&lt;&gt;""),"",COUNTIF($J$5:J419,J419))</x:f>
+      </x:c>
+      <x:c r="U419" s="45" t="str">
+        <x:f>IF(OR(J419="",Q419&lt;&gt;""),"",J419&amp;"|"&amp;R419)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="420">
+      <x:c r="R420" s="45" t="str">
+        <x:f>IF(OR(J420="",Q420&lt;&gt;""),"",COUNTIF($J$5:J420,J420))</x:f>
+      </x:c>
+      <x:c r="U420" s="45" t="str">
+        <x:f>IF(OR(J420="",Q420&lt;&gt;""),"",J420&amp;"|"&amp;R420)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="421">
+      <x:c r="R421" s="45" t="str">
+        <x:f>IF(OR(J421="",Q421&lt;&gt;""),"",COUNTIF($J$5:J421,J421))</x:f>
+      </x:c>
+      <x:c r="U421" s="45" t="str">
+        <x:f>IF(OR(J421="",Q421&lt;&gt;""),"",J421&amp;"|"&amp;R421)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="422">
+      <x:c r="R422" s="45" t="str">
+        <x:f>IF(OR(J422="",Q422&lt;&gt;""),"",COUNTIF($J$5:J422,J422))</x:f>
+      </x:c>
+      <x:c r="U422" s="45" t="str">
+        <x:f>IF(OR(J422="",Q422&lt;&gt;""),"",J422&amp;"|"&amp;R422)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="423">
+      <x:c r="R423" s="45" t="str">
+        <x:f>IF(OR(J423="",Q423&lt;&gt;""),"",COUNTIF($J$5:J423,J423))</x:f>
+      </x:c>
+      <x:c r="U423" s="45" t="str">
+        <x:f>IF(OR(J423="",Q423&lt;&gt;""),"",J423&amp;"|"&amp;R423)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="424">
+      <x:c r="R424" s="45" t="str">
+        <x:f>IF(OR(J424="",Q424&lt;&gt;""),"",COUNTIF($J$5:J424,J424))</x:f>
+      </x:c>
+      <x:c r="U424" s="45" t="str">
+        <x:f>IF(OR(J424="",Q424&lt;&gt;""),"",J424&amp;"|"&amp;R424)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="425">
+      <x:c r="R425" s="45" t="str">
+        <x:f>IF(OR(J425="",Q425&lt;&gt;""),"",COUNTIF($J$5:J425,J425))</x:f>
+      </x:c>
+      <x:c r="U425" s="45" t="str">
+        <x:f>IF(OR(J425="",Q425&lt;&gt;""),"",J425&amp;"|"&amp;R425)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="426">
+      <x:c r="R426" s="45" t="str">
+        <x:f>IF(OR(J426="",Q426&lt;&gt;""),"",COUNTIF($J$5:J426,J426))</x:f>
+      </x:c>
+      <x:c r="U426" s="45" t="str">
+        <x:f>IF(OR(J426="",Q426&lt;&gt;""),"",J426&amp;"|"&amp;R426)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="427">
+      <x:c r="R427" s="45" t="str">
+        <x:f>IF(OR(J427="",Q427&lt;&gt;""),"",COUNTIF($J$5:J427,J427))</x:f>
+      </x:c>
+      <x:c r="U427" s="45" t="str">
+        <x:f>IF(OR(J427="",Q427&lt;&gt;""),"",J427&amp;"|"&amp;R427)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="428">
+      <x:c r="R428" s="45" t="str">
+        <x:f>IF(OR(J428="",Q428&lt;&gt;""),"",COUNTIF($J$5:J428,J428))</x:f>
+      </x:c>
+      <x:c r="U428" s="45" t="str">
+        <x:f>IF(OR(J428="",Q428&lt;&gt;""),"",J428&amp;"|"&amp;R428)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="429">
+      <x:c r="R429" s="45" t="str">
+        <x:f>IF(OR(J429="",Q429&lt;&gt;""),"",COUNTIF($J$5:J429,J429))</x:f>
+      </x:c>
+      <x:c r="U429" s="45" t="str">
+        <x:f>IF(OR(J429="",Q429&lt;&gt;""),"",J429&amp;"|"&amp;R429)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="430">
+      <x:c r="R430" s="45" t="str">
+        <x:f>IF(OR(J430="",Q430&lt;&gt;""),"",COUNTIF($J$5:J430,J430))</x:f>
+      </x:c>
+      <x:c r="U430" s="45" t="str">
+        <x:f>IF(OR(J430="",Q430&lt;&gt;""),"",J430&amp;"|"&amp;R430)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="431">
+      <x:c r="R431" s="45" t="str">
+        <x:f>IF(OR(J431="",Q431&lt;&gt;""),"",COUNTIF($J$5:J431,J431))</x:f>
+      </x:c>
+      <x:c r="U431" s="45" t="str">
+        <x:f>IF(OR(J431="",Q431&lt;&gt;""),"",J431&amp;"|"&amp;R431)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="432">
+      <x:c r="R432" s="45" t="str">
+        <x:f>IF(OR(J432="",Q432&lt;&gt;""),"",COUNTIF($J$5:J432,J432))</x:f>
+      </x:c>
+      <x:c r="U432" s="45" t="str">
+        <x:f>IF(OR(J432="",Q432&lt;&gt;""),"",J432&amp;"|"&amp;R432)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="433">
+      <x:c r="R433" s="45" t="str">
+        <x:f>IF(OR(J433="",Q433&lt;&gt;""),"",COUNTIF($J$5:J433,J433))</x:f>
+      </x:c>
+      <x:c r="U433" s="45" t="str">
+        <x:f>IF(OR(J433="",Q433&lt;&gt;""),"",J433&amp;"|"&amp;R433)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="434">
+      <x:c r="R434" s="45" t="str">
+        <x:f>IF(OR(J434="",Q434&lt;&gt;""),"",COUNTIF($J$5:J434,J434))</x:f>
+      </x:c>
+      <x:c r="U434" s="45" t="str">
+        <x:f>IF(OR(J434="",Q434&lt;&gt;""),"",J434&amp;"|"&amp;R434)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="435">
+      <x:c r="R435" s="45" t="str">
+        <x:f>IF(OR(J435="",Q435&lt;&gt;""),"",COUNTIF($J$5:J435,J435))</x:f>
+      </x:c>
+      <x:c r="U435" s="45" t="str">
+        <x:f>IF(OR(J435="",Q435&lt;&gt;""),"",J435&amp;"|"&amp;R435)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="436">
+      <x:c r="R436" s="45" t="str">
+        <x:f>IF(OR(J436="",Q436&lt;&gt;""),"",COUNTIF($J$5:J436,J436))</x:f>
+      </x:c>
+      <x:c r="U436" s="45" t="str">
+        <x:f>IF(OR(J436="",Q436&lt;&gt;""),"",J436&amp;"|"&amp;R436)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="437">
+      <x:c r="R437" s="45" t="str">
+        <x:f>IF(OR(J437="",Q437&lt;&gt;""),"",COUNTIF($J$5:J437,J437))</x:f>
+      </x:c>
+      <x:c r="U437" s="45" t="str">
+        <x:f>IF(OR(J437="",Q437&lt;&gt;""),"",J437&amp;"|"&amp;R437)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="438">
+      <x:c r="R438" s="45" t="str">
+        <x:f>IF(OR(J438="",Q438&lt;&gt;""),"",COUNTIF($J$5:J438,J438))</x:f>
+      </x:c>
+      <x:c r="U438" s="45" t="str">
+        <x:f>IF(OR(J438="",Q438&lt;&gt;""),"",J438&amp;"|"&amp;R438)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="439">
+      <x:c r="R439" s="45" t="str">
+        <x:f>IF(OR(J439="",Q439&lt;&gt;""),"",COUNTIF($J$5:J439,J439))</x:f>
+      </x:c>
+      <x:c r="U439" s="45" t="str">
+        <x:f>IF(OR(J439="",Q439&lt;&gt;""),"",J439&amp;"|"&amp;R439)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="440">
+      <x:c r="R440" s="45" t="str">
+        <x:f>IF(OR(J440="",Q440&lt;&gt;""),"",COUNTIF($J$5:J440,J440))</x:f>
+      </x:c>
+      <x:c r="U440" s="45" t="str">
+        <x:f>IF(OR(J440="",Q440&lt;&gt;""),"",J440&amp;"|"&amp;R440)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="441">
+      <x:c r="R441" s="45" t="str">
+        <x:f>IF(OR(J441="",Q441&lt;&gt;""),"",COUNTIF($J$5:J441,J441))</x:f>
+      </x:c>
+      <x:c r="U441" s="45" t="str">
+        <x:f>IF(OR(J441="",Q441&lt;&gt;""),"",J441&amp;"|"&amp;R441)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="442">
+      <x:c r="R442" s="45" t="str">
+        <x:f>IF(OR(J442="",Q442&lt;&gt;""),"",COUNTIF($J$5:J442,J442))</x:f>
+      </x:c>
+      <x:c r="U442" s="45" t="str">
+        <x:f>IF(OR(J442="",Q442&lt;&gt;""),"",J442&amp;"|"&amp;R442)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="443">
+      <x:c r="R443" s="45" t="str">
+        <x:f>IF(OR(J443="",Q443&lt;&gt;""),"",COUNTIF($J$5:J443,J443))</x:f>
+      </x:c>
+      <x:c r="U443" s="45" t="str">
+        <x:f>IF(OR(J443="",Q443&lt;&gt;""),"",J443&amp;"|"&amp;R443)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="444">
+      <x:c r="R444" s="45" t="str">
+        <x:f>IF(OR(J444="",Q444&lt;&gt;""),"",COUNTIF($J$5:J444,J444))</x:f>
+      </x:c>
+      <x:c r="U444" s="45" t="str">
+        <x:f>IF(OR(J444="",Q444&lt;&gt;""),"",J444&amp;"|"&amp;R444)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="445">
+      <x:c r="R445" s="45" t="str">
+        <x:f>IF(OR(J445="",Q445&lt;&gt;""),"",COUNTIF($J$5:J445,J445))</x:f>
+      </x:c>
+      <x:c r="U445" s="45" t="str">
+        <x:f>IF(OR(J445="",Q445&lt;&gt;""),"",J445&amp;"|"&amp;R445)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="446">
+      <x:c r="R446" s="45" t="str">
+        <x:f>IF(OR(J446="",Q446&lt;&gt;""),"",COUNTIF($J$5:J446,J446))</x:f>
+      </x:c>
+      <x:c r="U446" s="45" t="str">
+        <x:f>IF(OR(J446="",Q446&lt;&gt;""),"",J446&amp;"|"&amp;R446)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="447">
+      <x:c r="R447" s="45" t="str">
+        <x:f>IF(OR(J447="",Q447&lt;&gt;""),"",COUNTIF($J$5:J447,J447))</x:f>
+      </x:c>
+      <x:c r="U447" s="45" t="str">
+        <x:f>IF(OR(J447="",Q447&lt;&gt;""),"",J447&amp;"|"&amp;R447)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="448">
+      <x:c r="R448" s="45" t="str">
+        <x:f>IF(OR(J448="",Q448&lt;&gt;""),"",COUNTIF($J$5:J448,J448))</x:f>
+      </x:c>
+      <x:c r="U448" s="45" t="str">
+        <x:f>IF(OR(J448="",Q448&lt;&gt;""),"",J448&amp;"|"&amp;R448)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="449">
+      <x:c r="R449" s="45" t="str">
+        <x:f>IF(OR(J449="",Q449&lt;&gt;""),"",COUNTIF($J$5:J449,J449))</x:f>
+      </x:c>
+      <x:c r="U449" s="45" t="str">
+        <x:f>IF(OR(J449="",Q449&lt;&gt;""),"",J449&amp;"|"&amp;R449)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="450">
+      <x:c r="R450" s="45" t="str">
+        <x:f>IF(OR(J450="",Q450&lt;&gt;""),"",COUNTIF($J$5:J450,J450))</x:f>
+      </x:c>
+      <x:c r="U450" s="45" t="str">
+        <x:f>IF(OR(J450="",Q450&lt;&gt;""),"",J450&amp;"|"&amp;R450)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="451">
+      <x:c r="R451" s="45" t="str">
+        <x:f>IF(OR(J451="",Q451&lt;&gt;""),"",COUNTIF($J$5:J451,J451))</x:f>
+      </x:c>
+      <x:c r="U451" s="45" t="str">
+        <x:f>IF(OR(J451="",Q451&lt;&gt;""),"",J451&amp;"|"&amp;R451)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="452">
+      <x:c r="R452" s="45" t="str">
+        <x:f>IF(OR(J452="",Q452&lt;&gt;""),"",COUNTIF($J$5:J452,J452))</x:f>
+      </x:c>
+      <x:c r="U452" s="45" t="str">
+        <x:f>IF(OR(J452="",Q452&lt;&gt;""),"",J452&amp;"|"&amp;R452)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="453">
+      <x:c r="R453" s="45" t="str">
+        <x:f>IF(OR(J453="",Q453&lt;&gt;""),"",COUNTIF($J$5:J453,J453))</x:f>
+      </x:c>
+      <x:c r="U453" s="45" t="str">
+        <x:f>IF(OR(J453="",Q453&lt;&gt;""),"",J453&amp;"|"&amp;R453)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="454">
+      <x:c r="R454" s="45" t="str">
+        <x:f>IF(OR(J454="",Q454&lt;&gt;""),"",COUNTIF($J$5:J454,J454))</x:f>
+      </x:c>
+      <x:c r="U454" s="45" t="str">
+        <x:f>IF(OR(J454="",Q454&lt;&gt;""),"",J454&amp;"|"&amp;R454)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="455">
+      <x:c r="R455" s="45" t="str">
+        <x:f>IF(OR(J455="",Q455&lt;&gt;""),"",COUNTIF($J$5:J455,J455))</x:f>
+      </x:c>
+      <x:c r="U455" s="45" t="str">
+        <x:f>IF(OR(J455="",Q455&lt;&gt;""),"",J455&amp;"|"&amp;R455)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="456">
+      <x:c r="R456" s="45" t="str">
+        <x:f>IF(OR(J456="",Q456&lt;&gt;""),"",COUNTIF($J$5:J456,J456))</x:f>
+      </x:c>
+      <x:c r="U456" s="45" t="str">
+        <x:f>IF(OR(J456="",Q456&lt;&gt;""),"",J456&amp;"|"&amp;R456)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="457">
+      <x:c r="R457" s="45" t="str">
+        <x:f>IF(OR(J457="",Q457&lt;&gt;""),"",COUNTIF($J$5:J457,J457))</x:f>
+      </x:c>
+      <x:c r="U457" s="45" t="str">
+        <x:f>IF(OR(J457="",Q457&lt;&gt;""),"",J457&amp;"|"&amp;R457)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="458">
+      <x:c r="R458" s="45" t="str">
+        <x:f>IF(OR(J458="",Q458&lt;&gt;""),"",COUNTIF($J$5:J458,J458))</x:f>
+      </x:c>
+      <x:c r="U458" s="45" t="str">
+        <x:f>IF(OR(J458="",Q458&lt;&gt;""),"",J458&amp;"|"&amp;R458)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="459">
+      <x:c r="R459" s="45" t="str">
+        <x:f>IF(OR(J459="",Q459&lt;&gt;""),"",COUNTIF($J$5:J459,J459))</x:f>
+      </x:c>
+      <x:c r="U459" s="45" t="str">
+        <x:f>IF(OR(J459="",Q459&lt;&gt;""),"",J459&amp;"|"&amp;R459)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="460">
+      <x:c r="R460" s="45" t="str">
+        <x:f>IF(OR(J460="",Q460&lt;&gt;""),"",COUNTIF($J$5:J460,J460))</x:f>
+      </x:c>
+      <x:c r="U460" s="45" t="str">
+        <x:f>IF(OR(J460="",Q460&lt;&gt;""),"",J460&amp;"|"&amp;R460)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="461">
+      <x:c r="R461" s="45" t="str">
+        <x:f>IF(OR(J461="",Q461&lt;&gt;""),"",COUNTIF($J$5:J461,J461))</x:f>
+      </x:c>
+      <x:c r="U461" s="45" t="str">
+        <x:f>IF(OR(J461="",Q461&lt;&gt;""),"",J461&amp;"|"&amp;R461)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="462">
+      <x:c r="R462" s="45" t="str">
+        <x:f>IF(OR(J462="",Q462&lt;&gt;""),"",COUNTIF($J$5:J462,J462))</x:f>
+      </x:c>
+      <x:c r="U462" s="45" t="str">
+        <x:f>IF(OR(J462="",Q462&lt;&gt;""),"",J462&amp;"|"&amp;R462)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="463">
+      <x:c r="R463" s="45" t="str">
+        <x:f>IF(OR(J463="",Q463&lt;&gt;""),"",COUNTIF($J$5:J463,J463))</x:f>
+      </x:c>
+      <x:c r="U463" s="45" t="str">
+        <x:f>IF(OR(J463="",Q463&lt;&gt;""),"",J463&amp;"|"&amp;R463)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="464">
+      <x:c r="R464" s="45" t="str">
+        <x:f>IF(OR(J464="",Q464&lt;&gt;""),"",COUNTIF($J$5:J464,J464))</x:f>
+      </x:c>
+      <x:c r="U464" s="45" t="str">
+        <x:f>IF(OR(J464="",Q464&lt;&gt;""),"",J464&amp;"|"&amp;R464)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="465">
+      <x:c r="R465" s="45" t="str">
+        <x:f>IF(OR(J465="",Q465&lt;&gt;""),"",COUNTIF($J$5:J465,J465))</x:f>
+      </x:c>
+      <x:c r="U465" s="45" t="str">
+        <x:f>IF(OR(J465="",Q465&lt;&gt;""),"",J465&amp;"|"&amp;R465)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="466">
+      <x:c r="R466" s="45" t="str">
+        <x:f>IF(OR(J466="",Q466&lt;&gt;""),"",COUNTIF($J$5:J466,J466))</x:f>
+      </x:c>
+      <x:c r="U466" s="45" t="str">
+        <x:f>IF(OR(J466="",Q466&lt;&gt;""),"",J466&amp;"|"&amp;R466)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="467">
+      <x:c r="R467" s="45" t="str">
+        <x:f>IF(OR(J467="",Q467&lt;&gt;""),"",COUNTIF($J$5:J467,J467))</x:f>
+      </x:c>
+      <x:c r="U467" s="45" t="str">
+        <x:f>IF(OR(J467="",Q467&lt;&gt;""),"",J467&amp;"|"&amp;R467)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="468">
+      <x:c r="R468" s="45" t="str">
+        <x:f>IF(OR(J468="",Q468&lt;&gt;""),"",COUNTIF($J$5:J468,J468))</x:f>
+      </x:c>
+      <x:c r="U468" s="45" t="str">
+        <x:f>IF(OR(J468="",Q468&lt;&gt;""),"",J468&amp;"|"&amp;R468)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="469">
+      <x:c r="R469" s="45" t="str">
+        <x:f>IF(OR(J469="",Q469&lt;&gt;""),"",COUNTIF($J$5:J469,J469))</x:f>
+      </x:c>
+      <x:c r="U469" s="45" t="str">
+        <x:f>IF(OR(J469="",Q469&lt;&gt;""),"",J469&amp;"|"&amp;R469)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="470">
+      <x:c r="R470" s="45" t="str">
+        <x:f>IF(OR(J470="",Q470&lt;&gt;""),"",COUNTIF($J$5:J470,J470))</x:f>
+      </x:c>
+      <x:c r="U470" s="45" t="str">
+        <x:f>IF(OR(J470="",Q470&lt;&gt;""),"",J470&amp;"|"&amp;R470)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="471">
+      <x:c r="R471" s="45" t="str">
+        <x:f>IF(OR(J471="",Q471&lt;&gt;""),"",COUNTIF($J$5:J471,J471))</x:f>
+      </x:c>
+      <x:c r="U471" s="45" t="str">
+        <x:f>IF(OR(J471="",Q471&lt;&gt;""),"",J471&amp;"|"&amp;R471)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="472">
+      <x:c r="R472" s="45" t="str">
+        <x:f>IF(OR(J472="",Q472&lt;&gt;""),"",COUNTIF($J$5:J472,J472))</x:f>
+      </x:c>
+      <x:c r="U472" s="45" t="str">
+        <x:f>IF(OR(J472="",Q472&lt;&gt;""),"",J472&amp;"|"&amp;R472)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="473">
+      <x:c r="R473" s="45" t="str">
+        <x:f>IF(OR(J473="",Q473&lt;&gt;""),"",COUNTIF($J$5:J473,J473))</x:f>
+      </x:c>
+      <x:c r="U473" s="45" t="str">
+        <x:f>IF(OR(J473="",Q473&lt;&gt;""),"",J473&amp;"|"&amp;R473)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="474">
+      <x:c r="R474" s="45" t="str">
+        <x:f>IF(OR(J474="",Q474&lt;&gt;""),"",COUNTIF($J$5:J474,J474))</x:f>
+      </x:c>
+      <x:c r="U474" s="45" t="str">
+        <x:f>IF(OR(J474="",Q474&lt;&gt;""),"",J474&amp;"|"&amp;R474)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="475">
+      <x:c r="R475" s="45" t="str">
+        <x:f>IF(OR(J475="",Q475&lt;&gt;""),"",COUNTIF($J$5:J475,J475))</x:f>
+      </x:c>
+      <x:c r="U475" s="45" t="str">
+        <x:f>IF(OR(J475="",Q475&lt;&gt;""),"",J475&amp;"|"&amp;R475)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="476">
+      <x:c r="R476" s="45" t="str">
+        <x:f>IF(OR(J476="",Q476&lt;&gt;""),"",COUNTIF($J$5:J476,J476))</x:f>
+      </x:c>
+      <x:c r="U476" s="45" t="str">
+        <x:f>IF(OR(J476="",Q476&lt;&gt;""),"",J476&amp;"|"&amp;R476)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="477">
+      <x:c r="R477" s="45" t="str">
+        <x:f>IF(OR(J477="",Q477&lt;&gt;""),"",COUNTIF($J$5:J477,J477))</x:f>
+      </x:c>
+      <x:c r="U477" s="45" t="str">
+        <x:f>IF(OR(J477="",Q477&lt;&gt;""),"",J477&amp;"|"&amp;R477)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="478">
+      <x:c r="R478" s="45" t="str">
+        <x:f>IF(OR(J478="",Q478&lt;&gt;""),"",COUNTIF($J$5:J478,J478))</x:f>
+      </x:c>
+      <x:c r="U478" s="45" t="str">
+        <x:f>IF(OR(J478="",Q478&lt;&gt;""),"",J478&amp;"|"&amp;R478)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="479">
+      <x:c r="R479" s="45" t="str">
+        <x:f>IF(OR(J479="",Q479&lt;&gt;""),"",COUNTIF($J$5:J479,J479))</x:f>
+      </x:c>
+      <x:c r="U479" s="45" t="str">
+        <x:f>IF(OR(J479="",Q479&lt;&gt;""),"",J479&amp;"|"&amp;R479)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="480">
+      <x:c r="R480" s="45" t="str">
+        <x:f>IF(OR(J480="",Q480&lt;&gt;""),"",COUNTIF($J$5:J480,J480))</x:f>
+      </x:c>
+      <x:c r="U480" s="45" t="str">
+        <x:f>IF(OR(J480="",Q480&lt;&gt;""),"",J480&amp;"|"&amp;R480)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="481">
+      <x:c r="R481" s="45" t="str">
+        <x:f>IF(OR(J481="",Q481&lt;&gt;""),"",COUNTIF($J$5:J481,J481))</x:f>
+      </x:c>
+      <x:c r="U481" s="45" t="str">
+        <x:f>IF(OR(J481="",Q481&lt;&gt;""),"",J481&amp;"|"&amp;R481)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="482">
+      <x:c r="R482" s="45" t="str">
+        <x:f>IF(OR(J482="",Q482&lt;&gt;""),"",COUNTIF($J$5:J482,J482))</x:f>
+      </x:c>
+      <x:c r="U482" s="45" t="str">
+        <x:f>IF(OR(J482="",Q482&lt;&gt;""),"",J482&amp;"|"&amp;R482)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="483">
+      <x:c r="R483" s="45" t="str">
+        <x:f>IF(OR(J483="",Q483&lt;&gt;""),"",COUNTIF($J$5:J483,J483))</x:f>
+      </x:c>
+      <x:c r="U483" s="45" t="str">
+        <x:f>IF(OR(J483="",Q483&lt;&gt;""),"",J483&amp;"|"&amp;R483)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="484">
+      <x:c r="R484" s="45" t="str">
+        <x:f>IF(OR(J484="",Q484&lt;&gt;""),"",COUNTIF($J$5:J484,J484))</x:f>
+      </x:c>
+      <x:c r="U484" s="45" t="str">
+        <x:f>IF(OR(J484="",Q484&lt;&gt;""),"",J484&amp;"|"&amp;R484)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="485">
+      <x:c r="R485" s="45" t="str">
+        <x:f>IF(OR(J485="",Q485&lt;&gt;""),"",COUNTIF($J$5:J485,J485))</x:f>
+      </x:c>
+      <x:c r="U485" s="45" t="str">
+        <x:f>IF(OR(J485="",Q485&lt;&gt;""),"",J485&amp;"|"&amp;R485)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="486">
+      <x:c r="R486" s="45" t="str">
+        <x:f>IF(OR(J486="",Q486&lt;&gt;""),"",COUNTIF($J$5:J486,J486))</x:f>
+      </x:c>
+      <x:c r="U486" s="45" t="str">
+        <x:f>IF(OR(J486="",Q486&lt;&gt;""),"",J486&amp;"|"&amp;R486)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="487">
+      <x:c r="R487" s="45" t="str">
+        <x:f>IF(OR(J487="",Q487&lt;&gt;""),"",COUNTIF($J$5:J487,J487))</x:f>
+      </x:c>
+      <x:c r="U487" s="45" t="str">
+        <x:f>IF(OR(J487="",Q487&lt;&gt;""),"",J487&amp;"|"&amp;R487)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="488">
+      <x:c r="R488" s="45" t="str">
+        <x:f>IF(OR(J488="",Q488&lt;&gt;""),"",COUNTIF($J$5:J488,J488))</x:f>
+      </x:c>
+      <x:c r="U488" s="45" t="str">
+        <x:f>IF(OR(J488="",Q488&lt;&gt;""),"",J488&amp;"|"&amp;R488)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="489">
+      <x:c r="R489" s="45" t="str">
+        <x:f>IF(OR(J489="",Q489&lt;&gt;""),"",COUNTIF($J$5:J489,J489))</x:f>
+      </x:c>
+      <x:c r="U489" s="45" t="str">
+        <x:f>IF(OR(J489="",Q489&lt;&gt;""),"",J489&amp;"|"&amp;R489)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="490">
+      <x:c r="R490" s="45" t="str">
+        <x:f>IF(OR(J490="",Q490&lt;&gt;""),"",COUNTIF($J$5:J490,J490))</x:f>
+      </x:c>
+      <x:c r="U490" s="45" t="str">
+        <x:f>IF(OR(J490="",Q490&lt;&gt;""),"",J490&amp;"|"&amp;R490)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="491">
+      <x:c r="R491" s="45" t="str">
+        <x:f>IF(OR(J491="",Q491&lt;&gt;""),"",COUNTIF($J$5:J491,J491))</x:f>
+      </x:c>
+      <x:c r="U491" s="45" t="str">
+        <x:f>IF(OR(J491="",Q491&lt;&gt;""),"",J491&amp;"|"&amp;R491)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="492">
+      <x:c r="R492" s="45" t="str">
+        <x:f>IF(OR(J492="",Q492&lt;&gt;""),"",COUNTIF($J$5:J492,J492))</x:f>
+      </x:c>
+      <x:c r="U492" s="45" t="str">
+        <x:f>IF(OR(J492="",Q492&lt;&gt;""),"",J492&amp;"|"&amp;R492)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="493">
+      <x:c r="R493" s="45" t="str">
+        <x:f>IF(OR(J493="",Q493&lt;&gt;""),"",COUNTIF($J$5:J493,J493))</x:f>
+      </x:c>
+      <x:c r="U493" s="45" t="str">
+        <x:f>IF(OR(J493="",Q493&lt;&gt;""),"",J493&amp;"|"&amp;R493)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="494">
+      <x:c r="R494" s="45" t="str">
+        <x:f>IF(OR(J494="",Q494&lt;&gt;""),"",COUNTIF($J$5:J494,J494))</x:f>
+      </x:c>
+      <x:c r="U494" s="45" t="str">
+        <x:f>IF(OR(J494="",Q494&lt;&gt;""),"",J494&amp;"|"&amp;R494)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="495">
+      <x:c r="R495" s="45" t="str">
+        <x:f>IF(OR(J495="",Q495&lt;&gt;""),"",COUNTIF($J$5:J495,J495))</x:f>
+      </x:c>
+      <x:c r="U495" s="45" t="str">
+        <x:f>IF(OR(J495="",Q495&lt;&gt;""),"",J495&amp;"|"&amp;R495)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="496">
+      <x:c r="R496" s="45" t="str">
+        <x:f>IF(OR(J496="",Q496&lt;&gt;""),"",COUNTIF($J$5:J496,J496))</x:f>
+      </x:c>
+      <x:c r="U496" s="45" t="str">
+        <x:f>IF(OR(J496="",Q496&lt;&gt;""),"",J496&amp;"|"&amp;R496)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="497">
+      <x:c r="R497" s="45" t="str">
+        <x:f>IF(OR(J497="",Q497&lt;&gt;""),"",COUNTIF($J$5:J497,J497))</x:f>
+      </x:c>
+      <x:c r="U497" s="45" t="str">
+        <x:f>IF(OR(J497="",Q497&lt;&gt;""),"",J497&amp;"|"&amp;R497)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="498">
+      <x:c r="R498" s="45" t="str">
+        <x:f>IF(OR(J498="",Q498&lt;&gt;""),"",COUNTIF($J$5:J498,J498))</x:f>
+      </x:c>
+      <x:c r="U498" s="45" t="str">
+        <x:f>IF(OR(J498="",Q498&lt;&gt;""),"",J498&amp;"|"&amp;R498)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="499">
+      <x:c r="R499" s="45" t="str">
+        <x:f>IF(OR(J499="",Q499&lt;&gt;""),"",COUNTIF($J$5:J499,J499))</x:f>
+      </x:c>
+      <x:c r="U499" s="45" t="str">
+        <x:f>IF(OR(J499="",Q499&lt;&gt;""),"",J499&amp;"|"&amp;R499)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="500">
+      <x:c r="R500" s="45" t="str">
+        <x:f>IF(OR(J500="",Q500&lt;&gt;""),"",COUNTIF($J$5:J500,J500))</x:f>
+      </x:c>
+      <x:c r="U500" s="45" t="str">
+        <x:f>IF(OR(J500="",Q500&lt;&gt;""),"",J500&amp;"|"&amp;R500)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="501">
+      <x:c r="R501" s="45" t="str">
+        <x:f>IF(OR(J501="",Q501&lt;&gt;""),"",COUNTIF($J$5:J501,J501))</x:f>
+      </x:c>
+      <x:c r="U501" s="45" t="str">
+        <x:f>IF(OR(J501="",Q501&lt;&gt;""),"",J501&amp;"|"&amp;R501)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="502">
+      <x:c r="R502" s="45" t="str">
+        <x:f>IF(OR(J502="",Q502&lt;&gt;""),"",COUNTIF($J$5:J502,J502))</x:f>
+      </x:c>
+      <x:c r="U502" s="45" t="str">
+        <x:f>IF(OR(J502="",Q502&lt;&gt;""),"",J502&amp;"|"&amp;R502)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="503">
+      <x:c r="R503" s="45" t="str">
+        <x:f>IF(OR(J503="",Q503&lt;&gt;""),"",COUNTIF($J$5:J503,J503))</x:f>
+      </x:c>
+      <x:c r="U503" s="45" t="str">
+        <x:f>IF(OR(J503="",Q503&lt;&gt;""),"",J503&amp;"|"&amp;R503)</x:f>
+      </x:c>
+    </x:row>
+    <x:row r="504">
+      <x:c r="R504" s="45" t="str">
+        <x:f>IF(OR(J504="",Q504&lt;&gt;""),"",COUNTIF($J$5:J504,J504))</x:f>
+      </x:c>
+      <x:c r="U504" s="45" t="str">
+        <x:f>IF(OR(J504="",Q504&lt;&gt;""),"",J504&amp;"|"&amp;R504)</x:f>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4303,7 +8266,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70c0dc9ffcfd4754"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36587522f7804b72"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add user guides to Excel and app
</commit_message>
<xml_diff>
--- a/app/template/캘린더(자동).xlsx
+++ b/app/template/캘린더(자동).xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="Recd4d1d50b864195"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26.8" sheetId="1" r:id="R4d8dd71997184a62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="R14a0a9b085c246bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26.8" sheetId="1" r:id="R45b5a2a756664d28"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,7 +157,7 @@
     <x:numFmt numFmtId="201" formatCode="hh:mm"/>
     <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </x:numFmts>
-  <x:fonts count="20">
+  <x:fonts count="24">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -267,8 +267,31 @@
       <x:color rgb="FFC2C8D0"/>
       <x:name val="맑은 고딕"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="맑은 고딕"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF315D8A"/>
+      <x:name val="맑은 고딕"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF3D4A5C"/>
+      <x:name val="맑은 고딕"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFB33D3D"/>
+      <x:name val="맑은 고딕"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -318,6 +341,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF7F9FC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FAFD"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF0F0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF8F8"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -556,7 +594,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="56">
+  <x:cellXfs count="67">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -718,6 +756,39 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -4118,7 +4189,17 @@
         <x:f>IF(OR(J16="",Q16&lt;&gt;""),"",J16&amp;"|"&amp;R16)</x:f>
       </x:c>
     </x:row>
-    <x:row r="17" ht="22" customHeight="1">
+    <x:row r="17" ht="30" customHeight="1">
+      <x:c r="B17" s="57" t="str">
+        <x:v>Cellendar 사용 방법</x:v>
+      </x:c>
+      <x:c r="C17" s="57"/>
+      <x:c r="D17" s="57"/>
+      <x:c r="E17" s="57"/>
+      <x:c r="F17" s="57"/>
+      <x:c r="G17" s="57"/>
+      <x:c r="H17" s="57"/>
+      <x:c r="I17" s="57"/>
       <x:c r="J17" s="37" t="str"/>
       <x:c r="K17" s="33" t="str"/>
       <x:c r="L17" s="33" t="str"/>
@@ -4139,7 +4220,19 @@
         <x:f>IF(OR(J17="",Q17&lt;&gt;""),"",J17&amp;"|"&amp;R17)</x:f>
       </x:c>
     </x:row>
-    <x:row r="18" ht="22" customHeight="1">
+    <x:row r="18" ht="27" customHeight="1">
+      <x:c r="B18" s="58" t="str">
+        <x:v>1. 일정 입력</x:v>
+      </x:c>
+      <x:c r="C18" s="58"/>
+      <x:c r="D18" s="61" t="str">
+        <x:v>오른쪽 노란 표에서 날짜와 색상을 목록으로 선택하고 제목을 입력하세요.</x:v>
+      </x:c>
+      <x:c r="E18" s="61"/>
+      <x:c r="F18" s="61"/>
+      <x:c r="G18" s="61"/>
+      <x:c r="H18" s="61"/>
+      <x:c r="I18" s="61"/>
       <x:c r="J18" s="37" t="str"/>
       <x:c r="K18" s="33" t="str"/>
       <x:c r="L18" s="33" t="str"/>
@@ -4160,7 +4253,19 @@
         <x:f>IF(OR(J18="",Q18&lt;&gt;""),"",J18&amp;"|"&amp;R18)</x:f>
       </x:c>
     </x:row>
-    <x:row r="19" ht="22" customHeight="1">
+    <x:row r="19" ht="27" customHeight="1">
+      <x:c r="B19" s="58" t="str">
+        <x:v>2. 달력 표시</x:v>
+      </x:c>
+      <x:c r="C19" s="58"/>
+      <x:c r="D19" s="61" t="str">
+        <x:v>같은 날짜의 일정은 달력 칸에 줄바꿈으로 최대 5개까지 표시됩니다.</x:v>
+      </x:c>
+      <x:c r="E19" s="61"/>
+      <x:c r="F19" s="61"/>
+      <x:c r="G19" s="61"/>
+      <x:c r="H19" s="61"/>
+      <x:c r="I19" s="61"/>
       <x:c r="J19" s="37" t="str"/>
       <x:c r="K19" s="33" t="str"/>
       <x:c r="L19" s="33" t="str"/>
@@ -4181,7 +4286,19 @@
         <x:f>IF(OR(J19="",Q19&lt;&gt;""),"",J19&amp;"|"&amp;R19)</x:f>
       </x:c>
     </x:row>
-    <x:row r="20" ht="22" customHeight="1">
+    <x:row r="20" ht="27" customHeight="1">
+      <x:c r="B20" s="58" t="str">
+        <x:v>3. 다음 달</x:v>
+      </x:c>
+      <x:c r="C20" s="58"/>
+      <x:c r="D20" s="61" t="str">
+        <x:v>상단의 연도와 월 숫자만 바꾸면 달력과 날짜 선택 목록이 함께 변경됩니다.</x:v>
+      </x:c>
+      <x:c r="E20" s="61"/>
+      <x:c r="F20" s="61"/>
+      <x:c r="G20" s="61"/>
+      <x:c r="H20" s="61"/>
+      <x:c r="I20" s="61"/>
       <x:c r="J20" s="37" t="str"/>
       <x:c r="K20" s="33" t="str"/>
       <x:c r="L20" s="33" t="str"/>
@@ -4202,7 +4319,19 @@
         <x:f>IF(OR(J20="",Q20&lt;&gt;""),"",J20&amp;"|"&amp;R20)</x:f>
       </x:c>
     </x:row>
-    <x:row r="21" ht="22" customHeight="1">
+    <x:row r="21" ht="27" customHeight="1">
+      <x:c r="B21" s="58" t="str">
+        <x:v>4. 비고 사용</x:v>
+      </x:c>
+      <x:c r="C21" s="58"/>
+      <x:c r="D21" s="61" t="str">
+        <x:v>초록색 비고 영역은 동기화와 관계없이 자유롭게 작성할 수 있습니다.</x:v>
+      </x:c>
+      <x:c r="E21" s="61"/>
+      <x:c r="F21" s="61"/>
+      <x:c r="G21" s="61"/>
+      <x:c r="H21" s="61"/>
+      <x:c r="I21" s="61"/>
       <x:c r="J21" s="37" t="str"/>
       <x:c r="K21" s="33" t="str"/>
       <x:c r="L21" s="33" t="str"/>
@@ -4223,7 +4352,19 @@
         <x:f>IF(OR(J21="",Q21&lt;&gt;""),"",J21&amp;"|"&amp;R21)</x:f>
       </x:c>
     </x:row>
-    <x:row r="22" ht="22" customHeight="1">
+    <x:row r="22" ht="27" customHeight="1">
+      <x:c r="B22" s="58" t="str">
+        <x:v>5. 앱 동기화</x:v>
+      </x:c>
+      <x:c r="C22" s="58"/>
+      <x:c r="D22" s="61" t="str">
+        <x:v>엑셀을 OneDrive의 Cellendar 폴더에 저장한 뒤 앱의 동기화 버튼을 누르세요.</x:v>
+      </x:c>
+      <x:c r="E22" s="61"/>
+      <x:c r="F22" s="61"/>
+      <x:c r="G22" s="61"/>
+      <x:c r="H22" s="61"/>
+      <x:c r="I22" s="61"/>
       <x:c r="J22" s="37" t="str"/>
       <x:c r="K22" s="33" t="str"/>
       <x:c r="L22" s="33" t="str"/>
@@ -4244,7 +4385,19 @@
         <x:f>IF(OR(J22="",Q22&lt;&gt;""),"",J22&amp;"|"&amp;R22)</x:f>
       </x:c>
     </x:row>
-    <x:row r="23" ht="22" customHeight="1">
+    <x:row r="23" ht="27" customHeight="1">
+      <x:c r="B23" s="58" t="str">
+        <x:v>6. 수정·삭제</x:v>
+      </x:c>
+      <x:c r="C23" s="58"/>
+      <x:c r="D23" s="61" t="str">
+        <x:v>휴대폰 앱에서 일정을 누르면 수정하거나 삭제할 수 있습니다.</x:v>
+      </x:c>
+      <x:c r="E23" s="61"/>
+      <x:c r="F23" s="61"/>
+      <x:c r="G23" s="61"/>
+      <x:c r="H23" s="61"/>
+      <x:c r="I23" s="61"/>
       <x:c r="J23" s="37" t="str"/>
       <x:c r="K23" s="33" t="str"/>
       <x:c r="L23" s="33" t="str"/>
@@ -4265,7 +4418,19 @@
         <x:f>IF(OR(J23="",Q23&lt;&gt;""),"",J23&amp;"|"&amp;R23)</x:f>
       </x:c>
     </x:row>
-    <x:row r="24" ht="22" customHeight="1">
+    <x:row r="24" ht="27" customHeight="1">
+      <x:c r="B24" s="63" t="str">
+        <x:v>주의</x:v>
+      </x:c>
+      <x:c r="C24" s="63"/>
+      <x:c r="D24" s="66" t="str">
+        <x:v>회색 ID·수정시간·삭제시간 칸과 내부 조회 영역은 수정하지 마세요.</x:v>
+      </x:c>
+      <x:c r="E24" s="66"/>
+      <x:c r="F24" s="66"/>
+      <x:c r="G24" s="66"/>
+      <x:c r="H24" s="66"/>
+      <x:c r="I24" s="66"/>
       <x:c r="J24" s="37" t="str"/>
       <x:c r="K24" s="33" t="str"/>
       <x:c r="L24" s="33" t="str"/>
@@ -8250,6 +8415,21 @@
   <x:mergeCells>
     <x:mergeCell ref="J1:Q1"/>
     <x:mergeCell ref="J2:Q2"/>
+    <x:mergeCell ref="B17:I17"/>
+    <x:mergeCell ref="B18:C18"/>
+    <x:mergeCell ref="D18:I18"/>
+    <x:mergeCell ref="B19:C19"/>
+    <x:mergeCell ref="D19:I19"/>
+    <x:mergeCell ref="B20:C20"/>
+    <x:mergeCell ref="D20:I20"/>
+    <x:mergeCell ref="B21:C21"/>
+    <x:mergeCell ref="D21:I21"/>
+    <x:mergeCell ref="B22:C22"/>
+    <x:mergeCell ref="D22:I22"/>
+    <x:mergeCell ref="B23:C23"/>
+    <x:mergeCell ref="D23:I23"/>
+    <x:mergeCell ref="B24:C24"/>
+    <x:mergeCell ref="D24:I24"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B3:H3 B5:H5 B7:H7 B9:H9 B11:H11 B13:H13">
     <x:cfRule type="expression" dxfId="1" priority="3" stopIfTrue="1">
@@ -8266,7 +8446,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36587522f7804b72"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64ad3c030f8d46f1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Excel alarm time synchronization
</commit_message>
<xml_diff>
--- a/app/template/캘린더(자동).xlsx
+++ b/app/template/캘린더(자동).xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="R14a0a9b085c246bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26.8" sheetId="1" r:id="R45b5a2a756664d28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="Rdad5954c4fc8459d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26.8" sheetId="1" r:id="R51e518b0c7b24cb6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8446,7 +8446,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64ad3c030f8d46f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa43c3f9bf4f4278"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Rename calendar sheet and show holidays
</commit_message>
<xml_diff>
--- a/app/template/캘린더(자동).xlsx
+++ b/app/template/캘린더(자동).xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="Rdad5954c4fc8459d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26.8" sheetId="1" r:id="R51e518b0c7b24cb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="R561ef939a1014ba6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="달력" sheetId="1" r:id="R5b38d99f43344fc6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3576,11 +3576,11 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
-      <x:c r="B3" s="46" t="n">
+      <x:c r="B3" s="46">
         <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1</x:f>
         <x:v>46229</x:v>
       </x:c>
-      <x:c r="C3" s="47" t="n">
+      <x:c r="C3" s="47">
         <x:f t="shared" ref="C3:H3" si="0">B3+1</x:f>
         <x:v>46230</x:v>
       </x:c>
@@ -3615,25 +3615,25 @@
     </x:row>
     <x:row r="4" ht="72" customHeight="1">
       <x:c r="B4" s="49" t="str">
-        <x:f>XLOOKUP(B3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(B3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(B3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(B3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(B3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(B3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="C4" s="50" t="str">
-        <x:f>XLOOKUP(C3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(C3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(C3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(C3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(C3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(C3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="D4" s="51" t="str">
-        <x:f>XLOOKUP(D3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(D3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(D3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(D3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(D3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(D3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="E4" s="50" t="str">
-        <x:f>XLOOKUP(E3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(E3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(E3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(E3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(E3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(E3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="F4" s="50" t="str">
-        <x:f>XLOOKUP(F3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(F3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(F3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(F3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(F3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(F3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="G4" s="50" t="str">
-        <x:f>XLOOKUP(G3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(G3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(G3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(G3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(G3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(G3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="H4" s="52" t="str">
-        <x:f>XLOOKUP(H3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(H3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(H3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(H3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(H3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(H3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="I4" s="1"/>
       <x:c r="J4" s="30" t="str">
@@ -3675,11 +3675,11 @@
       </x:c>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
-      <x:c r="B5" s="46" t="n">
+      <x:c r="B5" s="46">
         <x:f>H3+1</x:f>
         <x:v>46236</x:v>
       </x:c>
-      <x:c r="C5" s="47" t="n">
+      <x:c r="C5" s="47">
         <x:f t="shared" ref="C5:H5" si="1">B5+1</x:f>
         <x:v>46237</x:v>
       </x:c>
@@ -3728,25 +3728,25 @@
     </x:row>
     <x:row r="6" ht="72" customHeight="1">
       <x:c r="B6" s="49" t="str">
-        <x:f>XLOOKUP(B5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(B5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(B5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(B5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(B5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(B5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="C6" s="51" t="str">
-        <x:f>XLOOKUP(C5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(C5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(C5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(C5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(C5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(C5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="D6" s="51" t="str">
-        <x:f>XLOOKUP(D5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(D5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(D5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(D5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(D5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(D5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="E6" s="51" t="str">
-        <x:f>XLOOKUP(E5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(E5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(E5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(E5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(E5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(E5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="F6" s="51" t="str">
-        <x:f>XLOOKUP(F5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(F5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(F5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(F5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(F5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(F5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="G6" s="51" t="str">
-        <x:f>XLOOKUP(G5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(G5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(G5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(G5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(G5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(G5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="H6" s="52" t="str">
-        <x:f>XLOOKUP(H5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(H5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(H5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(H5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(H5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(H5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="I6" s="1"/>
       <x:c r="J6" s="37" t="str"/>
@@ -3772,11 +3772,11 @@
       </x:c>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
-      <x:c r="B7" s="46" t="n">
+      <x:c r="B7" s="46">
         <x:f>H5+1</x:f>
         <x:v>46243</x:v>
       </x:c>
-      <x:c r="C7" s="47" t="n">
+      <x:c r="C7" s="47">
         <x:f t="shared" ref="C7:H7" si="2">B7+1</x:f>
         <x:v>46244</x:v>
       </x:c>
@@ -3825,25 +3825,26 @@
     </x:row>
     <x:row r="8" ht="72" customHeight="1">
       <x:c r="B8" s="49" t="str">
-        <x:f>XLOOKUP(B7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(B7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(B7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(B7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(B7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(B7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="C8" s="51" t="str">
-        <x:f>XLOOKUP(C7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(C7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(C7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(C7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(C7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(C7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="D8" s="51" t="str">
-        <x:f>XLOOKUP(D7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(D7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(D7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(D7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(D7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(D7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="E8" s="51" t="str">
-        <x:f>XLOOKUP(E7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(E7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(E7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(E7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(E7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(E7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="F8" s="51" t="str">
-        <x:f>XLOOKUP(F7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(F7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(F7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(F7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(F7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(F7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="G8" s="51" t="str">
-        <x:f>XLOOKUP(G7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(G7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(G7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(G7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(G7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(G7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="H8" s="52" t="str">
-        <x:f>XLOOKUP(H7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(H7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(H7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(H7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(H7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(H7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:v>◆ 광복절</x:v>
       </x:c>
       <x:c r="I8" s="1"/>
       <x:c r="J8" s="37" t="str"/>
@@ -3869,11 +3870,11 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
-      <x:c r="B9" s="46" t="n">
+      <x:c r="B9" s="46">
         <x:f>H7+1</x:f>
         <x:v>46250</x:v>
       </x:c>
-      <x:c r="C9" s="47" t="n">
+      <x:c r="C9" s="47">
         <x:f t="shared" ref="C9:H9" si="3">B9+1</x:f>
         <x:v>46251</x:v>
       </x:c>
@@ -3920,25 +3921,26 @@
     </x:row>
     <x:row r="10" ht="72" customHeight="1">
       <x:c r="B10" s="49" t="str">
-        <x:f>XLOOKUP(B9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(B9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(B9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(B9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(B9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(B9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="C10" s="51" t="str">
-        <x:f>XLOOKUP(C9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(C9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(C9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(C9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(C9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(C9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:v>◆ 광복절 대체 휴일</x:v>
       </x:c>
       <x:c r="D10" s="51" t="str">
-        <x:f>XLOOKUP(D9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(D9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(D9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(D9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(D9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(D9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="E10" s="51" t="str">
-        <x:f>XLOOKUP(E9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(E9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(E9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(E9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(E9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(E9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="F10" s="51" t="str">
-        <x:f>XLOOKUP(F9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(F9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(F9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(F9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(F9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(F9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="G10" s="51" t="str">
-        <x:f>XLOOKUP(G9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(G9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(G9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(G9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(G9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(G9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="H10" s="52" t="str">
-        <x:f>XLOOKUP(H9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(H9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(H9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(H9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(H9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(H9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="I10" s="1"/>
       <x:c r="J10" s="37" t="str"/>
@@ -3962,11 +3964,11 @@
       </x:c>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
-      <x:c r="B11" s="46" t="n">
+      <x:c r="B11" s="46">
         <x:f>H9+1</x:f>
         <x:v>46257</x:v>
       </x:c>
-      <x:c r="C11" s="47" t="n">
+      <x:c r="C11" s="47">
         <x:f t="shared" ref="C11:H11" si="4">B11+1</x:f>
         <x:v>46258</x:v>
       </x:c>
@@ -4013,25 +4015,25 @@
     </x:row>
     <x:row r="12" ht="72" customHeight="1">
       <x:c r="B12" s="49" t="str">
-        <x:f>XLOOKUP(B11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(B11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(B11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(B11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(B11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(B11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="C12" s="51" t="str">
-        <x:f>XLOOKUP(C11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(C11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(C11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(C11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(C11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(C11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="D12" s="51" t="str">
-        <x:f>XLOOKUP(D11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(D11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(D11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(D11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(D11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(D11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="E12" s="51" t="str">
-        <x:f>XLOOKUP(E11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(E11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(E11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(E11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(E11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(E11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="F12" s="51" t="str">
-        <x:f>XLOOKUP(F11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(F11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(F11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(F11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(F11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(F11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="G12" s="51" t="str">
-        <x:f>XLOOKUP(G11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(G11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(G11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(G11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(G11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(G11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="H12" s="52" t="str">
-        <x:f>XLOOKUP(H11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(H11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(H11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(H11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(H11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(H11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="I12" s="1"/>
       <x:c r="J12" s="37" t="str"/>
@@ -4055,11 +4057,11 @@
       </x:c>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
-      <x:c r="B13" s="46" t="n">
+      <x:c r="B13" s="46">
         <x:f>H11+1</x:f>
         <x:v>46264</x:v>
       </x:c>
-      <x:c r="C13" s="47" t="n">
+      <x:c r="C13" s="47">
         <x:f t="shared" ref="C13:H13" si="5">B13+1</x:f>
         <x:v>46265</x:v>
       </x:c>
@@ -4106,25 +4108,25 @@
     </x:row>
     <x:row r="14" ht="72" customHeight="1">
       <x:c r="B14" s="53" t="str">
-        <x:f>XLOOKUP(B13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(B13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(B13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(B13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(B13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(B13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="C14" s="54" t="str">
-        <x:f>XLOOKUP(C13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(C13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(C13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(C13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(C13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(C13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="D14" s="54" t="str">
-        <x:f>XLOOKUP(D13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(D13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(D13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(D13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(D13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(D13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="E14" s="54" t="str">
-        <x:f>XLOOKUP(E13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(E13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(E13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(E13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(E13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(E13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="F14" s="54" t="str">
-        <x:f>XLOOKUP(F13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(F13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(F13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(F13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(F13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(F13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="G14" s="54" t="str">
-        <x:f>XLOOKUP(G13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(G13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(G13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(G13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(G13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(G13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="H14" s="55" t="str">
-        <x:f>XLOOKUP(H13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+        <x:f>IF(XLOOKUP(H13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(H13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(H13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(H13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(H13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="I14" s="2"/>
       <x:c r="J14" s="37" t="str"/>
@@ -8446,7 +8448,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa43c3f9bf4f4278"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10b5e5e780824c58"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Move holidays beside dates and clear deleted rows
</commit_message>
<xml_diff>
--- a/app/template/캘린더(자동).xlsx
+++ b/app/template/캘린더(자동).xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="R561ef939a1014ba6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="달력" sheetId="1" r:id="R5b38d99f43344fc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="Rcf4bb265a46e43cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="달력" sheetId="1" r:id="Ra69ac5ca36bf4fa3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -594,7 +594,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="67">
+  <x:cellXfs count="68">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -727,14 +727,17 @@
     <x:xf numFmtId="0" fontId="19" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="19" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="176" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="176" fontId="7" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="176" fontId="12" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
@@ -794,7 +797,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="표준" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="2">
+  <x:dxfs count="44">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -804,6 +807,258 @@
     <x:dxf>
       <x:font>
         <x:color rgb="FF808080"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFE85858"/>
       </x:font>
     </x:dxf>
   </x:dxfs>
@@ -3496,6 +3751,8 @@
     <x:col min="20" max="20" width="11" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="9" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="14" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="4" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="4" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
@@ -3531,6 +3788,12 @@
       <x:c r="T1" s="43" t="str">
         <x:v>색상 목록</x:v>
       </x:c>
+      <x:c r="V1" s="45" t="str">
+        <x:v>달력 실제 날짜</x:v>
+      </x:c>
+      <x:c r="W1" s="45" t="str">
+        <x:v>공휴일명</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
       <x:c r="B2" s="4" t="s">
@@ -3574,35 +3837,42 @@
       <x:c r="T2" s="43" t="str">
         <x:v>파랑</x:v>
       </x:c>
+      <x:c r="V2" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+0</x:f>
+        <x:v>46229</x:v>
+      </x:c>
+      <x:c r="W2" s="45" t="str">
+        <x:f>XLOOKUP(V2,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
-      <x:c r="B3" s="46">
-        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1</x:f>
-        <x:v>46229</x:v>
-      </x:c>
-      <x:c r="C3" s="47">
-        <x:f t="shared" ref="C3:H3" si="0">B3+1</x:f>
-        <x:v>46230</x:v>
-      </x:c>
-      <x:c r="D3" s="47">
-        <x:f t="shared" si="0"/>
-        <x:v>46231</x:v>
-      </x:c>
-      <x:c r="E3" s="47">
-        <x:f t="shared" si="0"/>
-        <x:v>46232</x:v>
-      </x:c>
-      <x:c r="F3" s="47">
-        <x:f t="shared" si="0"/>
-        <x:v>46233</x:v>
-      </x:c>
-      <x:c r="G3" s="47">
-        <x:f t="shared" si="0"/>
-        <x:v>46234</x:v>
-      </x:c>
-      <x:c r="H3" s="48">
-        <x:f t="shared" si="0"/>
-        <x:v>46235</x:v>
+      <x:c r="B3" s="47" t="str">
+        <x:f>IF($W$2&lt;&gt;"",$W$2&amp;REPT(" ",MAX(2,18-LEN($W$2)))&amp;DAY($V$2),REPT(" ",16-LEN(DAY($V$2)))&amp;DAY($V$2))</x:f>
+        <x:v>              26</x:v>
+      </x:c>
+      <x:c r="C3" s="48" t="str">
+        <x:f t="shared" ref="C3:H3" si="0">IF($W$3&lt;&gt;"",$W$3&amp;REPT(" ",MAX(2,18-LEN($W$3)))&amp;DAY($V$3),REPT(" ",16-LEN(DAY($V$3)))&amp;DAY($V$3))</x:f>
+        <x:v>              27</x:v>
+      </x:c>
+      <x:c r="D3" s="48" t="str">
+        <x:f t="shared" si="0">IF($W$4&lt;&gt;"",$W$4&amp;REPT(" ",MAX(2,18-LEN($W$4)))&amp;DAY($V$4),REPT(" ",16-LEN(DAY($V$4)))&amp;DAY($V$4))</x:f>
+        <x:v>              28</x:v>
+      </x:c>
+      <x:c r="E3" s="48" t="str">
+        <x:f t="shared" si="0">IF($W$5&lt;&gt;"",$W$5&amp;REPT(" ",MAX(2,18-LEN($W$5)))&amp;DAY($V$5),REPT(" ",16-LEN(DAY($V$5)))&amp;DAY($V$5))</x:f>
+        <x:v>              29</x:v>
+      </x:c>
+      <x:c r="F3" s="48" t="str">
+        <x:f t="shared" si="0">IF($W$6&lt;&gt;"",$W$6&amp;REPT(" ",MAX(2,18-LEN($W$6)))&amp;DAY($V$6),REPT(" ",16-LEN(DAY($V$6)))&amp;DAY($V$6))</x:f>
+        <x:v>              30</x:v>
+      </x:c>
+      <x:c r="G3" s="48" t="str">
+        <x:f t="shared" si="0">IF($W$7&lt;&gt;"",$W$7&amp;REPT(" ",MAX(2,18-LEN($W$7)))&amp;DAY($V$7),REPT(" ",16-LEN(DAY($V$7)))&amp;DAY($V$7))</x:f>
+        <x:v>              31</x:v>
+      </x:c>
+      <x:c r="H3" s="49" t="str">
+        <x:f t="shared" si="0">IF($W$8&lt;&gt;"",$W$8&amp;REPT(" ",MAX(2,18-LEN($W$8)))&amp;DAY($V$8),REPT(" ",16-LEN(DAY($V$8)))&amp;DAY($V$8))</x:f>
+        <x:v>               1</x:v>
       </x:c>
       <x:c r="I3" s="1"/>
       <x:c r="S3" s="44" t="n">
@@ -3612,28 +3882,35 @@
       <x:c r="T3" s="43" t="str">
         <x:v>빨강</x:v>
       </x:c>
+      <x:c r="V3" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+1</x:f>
+        <x:v>46230</x:v>
+      </x:c>
+      <x:c r="W3" s="45" t="str">
+        <x:f>XLOOKUP(V3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="4" ht="72" customHeight="1">
-      <x:c r="B4" s="49" t="str">
-        <x:f>IF(XLOOKUP(B3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(B3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(B3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(B3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(B3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="C4" s="50" t="str">
-        <x:f>IF(XLOOKUP(C3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(C3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(C3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(C3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(C3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="D4" s="51" t="str">
-        <x:f>IF(XLOOKUP(D3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(D3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(D3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(D3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(D3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="E4" s="50" t="str">
-        <x:f>IF(XLOOKUP(E3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(E3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(E3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(E3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(E3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="F4" s="50" t="str">
-        <x:f>IF(XLOOKUP(F3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(F3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(F3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(F3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(F3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="G4" s="50" t="str">
-        <x:f>IF(XLOOKUP(G3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(G3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(G3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(G3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(G3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="H4" s="52" t="str">
-        <x:f>IF(XLOOKUP(H3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(H3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(H3,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(H3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(H3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      <x:c r="B4" s="50" t="str">
+        <x:f>XLOOKUP($V$2&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$2&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$2&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$2&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$2&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$2&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$2&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$2&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$2&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="C4" s="51" t="str">
+        <x:f>XLOOKUP($V$3&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$3&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$3&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$3&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$3&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="D4" s="52" t="str">
+        <x:f>XLOOKUP($V$4&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$4&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$4&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$4&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$4&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$4&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$4&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$4&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$4&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="E4" s="51" t="str">
+        <x:f>XLOOKUP($V$5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="F4" s="51" t="str">
+        <x:f>XLOOKUP($V$6&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$6&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$6&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$6&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$6&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$6&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$6&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$6&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$6&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="G4" s="51" t="str">
+        <x:f>XLOOKUP($V$7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="H4" s="53" t="str">
+        <x:f>XLOOKUP($V$8&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$8&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$8&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$8&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$8&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$8&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$8&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$8&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$8&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="I4" s="1"/>
       <x:c r="J4" s="30" t="str">
@@ -3673,35 +3950,42 @@
       <x:c r="U4" s="45" t="str">
         <x:v>내부 조회 키</x:v>
       </x:c>
+      <x:c r="V4" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+2</x:f>
+        <x:v>46231</x:v>
+      </x:c>
+      <x:c r="W4" s="45" t="str">
+        <x:f>XLOOKUP(V4,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
-      <x:c r="B5" s="46">
-        <x:f>H3+1</x:f>
-        <x:v>46236</x:v>
-      </x:c>
-      <x:c r="C5" s="47">
-        <x:f t="shared" ref="C5:H5" si="1">B5+1</x:f>
-        <x:v>46237</x:v>
-      </x:c>
-      <x:c r="D5" s="47">
-        <x:f t="shared" si="1"/>
-        <x:v>46238</x:v>
-      </x:c>
-      <x:c r="E5" s="47">
-        <x:f t="shared" si="1"/>
-        <x:v>46239</x:v>
-      </x:c>
-      <x:c r="F5" s="47">
-        <x:f t="shared" si="1"/>
-        <x:v>46240</x:v>
-      </x:c>
-      <x:c r="G5" s="47">
-        <x:f t="shared" si="1"/>
-        <x:v>46241</x:v>
-      </x:c>
-      <x:c r="H5" s="48">
-        <x:f t="shared" si="1"/>
-        <x:v>46242</x:v>
+      <x:c r="B5" s="47" t="str">
+        <x:f>IF($W$9&lt;&gt;"",$W$9&amp;REPT(" ",MAX(2,18-LEN($W$9)))&amp;DAY($V$9),REPT(" ",16-LEN(DAY($V$9)))&amp;DAY($V$9))</x:f>
+        <x:v>               2</x:v>
+      </x:c>
+      <x:c r="C5" s="48" t="str">
+        <x:f t="shared" ref="C5:H5" si="1">IF($W$10&lt;&gt;"",$W$10&amp;REPT(" ",MAX(2,18-LEN($W$10)))&amp;DAY($V$10),REPT(" ",16-LEN(DAY($V$10)))&amp;DAY($V$10))</x:f>
+        <x:v>               3</x:v>
+      </x:c>
+      <x:c r="D5" s="48" t="str">
+        <x:f t="shared" si="1">IF($W$11&lt;&gt;"",$W$11&amp;REPT(" ",MAX(2,18-LEN($W$11)))&amp;DAY($V$11),REPT(" ",16-LEN(DAY($V$11)))&amp;DAY($V$11))</x:f>
+        <x:v>               4</x:v>
+      </x:c>
+      <x:c r="E5" s="48" t="str">
+        <x:f t="shared" si="1">IF($W$12&lt;&gt;"",$W$12&amp;REPT(" ",MAX(2,18-LEN($W$12)))&amp;DAY($V$12),REPT(" ",16-LEN(DAY($V$12)))&amp;DAY($V$12))</x:f>
+        <x:v>               5</x:v>
+      </x:c>
+      <x:c r="F5" s="48" t="str">
+        <x:f t="shared" si="1">IF($W$13&lt;&gt;"",$W$13&amp;REPT(" ",MAX(2,18-LEN($W$13)))&amp;DAY($V$13),REPT(" ",16-LEN(DAY($V$13)))&amp;DAY($V$13))</x:f>
+        <x:v>               6</x:v>
+      </x:c>
+      <x:c r="G5" s="48" t="str">
+        <x:f t="shared" si="1">IF($W$14&lt;&gt;"",$W$14&amp;REPT(" ",MAX(2,18-LEN($W$14)))&amp;DAY($V$14),REPT(" ",16-LEN(DAY($V$14)))&amp;DAY($V$14))</x:f>
+        <x:v>               7</x:v>
+      </x:c>
+      <x:c r="H5" s="49" t="str">
+        <x:f t="shared" si="1">IF($W$15&lt;&gt;"",$W$15&amp;REPT(" ",MAX(2,18-LEN($W$15)))&amp;DAY($V$15),REPT(" ",16-LEN(DAY($V$15)))&amp;DAY($V$15))</x:f>
+        <x:v>               8</x:v>
       </x:c>
       <x:c r="I5" s="1"/>
       <x:c r="J5" s="37" t="str"/>
@@ -3725,28 +4009,35 @@
       <x:c r="U5" s="45" t="str">
         <x:f>IF(OR(J5="",Q5&lt;&gt;""),"",J5&amp;"|"&amp;R5)</x:f>
       </x:c>
+      <x:c r="V5" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+3</x:f>
+        <x:v>46232</x:v>
+      </x:c>
+      <x:c r="W5" s="45" t="str">
+        <x:f>XLOOKUP(V5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="6" ht="72" customHeight="1">
-      <x:c r="B6" s="49" t="str">
-        <x:f>IF(XLOOKUP(B5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(B5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(B5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(B5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(B5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="C6" s="51" t="str">
-        <x:f>IF(XLOOKUP(C5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(C5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(C5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(C5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(C5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="D6" s="51" t="str">
-        <x:f>IF(XLOOKUP(D5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(D5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(D5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(D5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(D5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="E6" s="51" t="str">
-        <x:f>IF(XLOOKUP(E5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(E5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(E5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(E5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(E5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="F6" s="51" t="str">
-        <x:f>IF(XLOOKUP(F5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(F5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(F5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(F5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(F5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="G6" s="51" t="str">
-        <x:f>IF(XLOOKUP(G5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(G5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(G5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(G5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(G5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="H6" s="52" t="str">
-        <x:f>IF(XLOOKUP(H5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(H5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(H5,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(H5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(H5&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H5&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H5&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H5&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H5&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      <x:c r="B6" s="50" t="str">
+        <x:f>XLOOKUP($V$9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="C6" s="52" t="str">
+        <x:f>XLOOKUP($V$10&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$10&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$10&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$10&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$10&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$10&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$10&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$10&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$10&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="D6" s="52" t="str">
+        <x:f>XLOOKUP($V$11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="E6" s="52" t="str">
+        <x:f>XLOOKUP($V$12&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$12&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$12&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$12&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$12&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$12&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$12&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$12&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$12&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="F6" s="52" t="str">
+        <x:f>XLOOKUP($V$13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="G6" s="52" t="str">
+        <x:f>XLOOKUP($V$14&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$14&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$14&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$14&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$14&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$14&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$14&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$14&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$14&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="H6" s="53" t="str">
+        <x:f>XLOOKUP($V$15&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$15&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$15&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$15&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$15&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$15&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$15&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$15&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$15&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="I6" s="1"/>
       <x:c r="J6" s="37" t="str"/>
@@ -3770,35 +4061,42 @@
       <x:c r="U6" s="45" t="str">
         <x:f>IF(OR(J6="",Q6&lt;&gt;""),"",J6&amp;"|"&amp;R6)</x:f>
       </x:c>
+      <x:c r="V6" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+4</x:f>
+        <x:v>46233</x:v>
+      </x:c>
+      <x:c r="W6" s="45" t="str">
+        <x:f>XLOOKUP(V6,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
-      <x:c r="B7" s="46">
-        <x:f>H5+1</x:f>
-        <x:v>46243</x:v>
-      </x:c>
-      <x:c r="C7" s="47">
-        <x:f t="shared" ref="C7:H7" si="2">B7+1</x:f>
-        <x:v>46244</x:v>
-      </x:c>
-      <x:c r="D7" s="47">
-        <x:f t="shared" si="2"/>
-        <x:v>46245</x:v>
-      </x:c>
-      <x:c r="E7" s="47">
-        <x:f t="shared" si="2"/>
-        <x:v>46246</x:v>
-      </x:c>
-      <x:c r="F7" s="47">
-        <x:f t="shared" si="2"/>
-        <x:v>46247</x:v>
-      </x:c>
-      <x:c r="G7" s="47">
-        <x:f t="shared" si="2"/>
-        <x:v>46248</x:v>
-      </x:c>
-      <x:c r="H7" s="48">
-        <x:f t="shared" si="2"/>
-        <x:v>46249</x:v>
+      <x:c r="B7" s="47" t="str">
+        <x:f>IF($W$16&lt;&gt;"",$W$16&amp;REPT(" ",MAX(2,18-LEN($W$16)))&amp;DAY($V$16),REPT(" ",16-LEN(DAY($V$16)))&amp;DAY($V$16))</x:f>
+        <x:v>               9</x:v>
+      </x:c>
+      <x:c r="C7" s="48" t="str">
+        <x:f t="shared" ref="C7:H7" si="2">IF($W$17&lt;&gt;"",$W$17&amp;REPT(" ",MAX(2,18-LEN($W$17)))&amp;DAY($V$17),REPT(" ",16-LEN(DAY($V$17)))&amp;DAY($V$17))</x:f>
+        <x:v>              10</x:v>
+      </x:c>
+      <x:c r="D7" s="48" t="str">
+        <x:f t="shared" si="2">IF($W$18&lt;&gt;"",$W$18&amp;REPT(" ",MAX(2,18-LEN($W$18)))&amp;DAY($V$18),REPT(" ",16-LEN(DAY($V$18)))&amp;DAY($V$18))</x:f>
+        <x:v>              11</x:v>
+      </x:c>
+      <x:c r="E7" s="48" t="str">
+        <x:f t="shared" si="2">IF($W$19&lt;&gt;"",$W$19&amp;REPT(" ",MAX(2,18-LEN($W$19)))&amp;DAY($V$19),REPT(" ",16-LEN(DAY($V$19)))&amp;DAY($V$19))</x:f>
+        <x:v>              12</x:v>
+      </x:c>
+      <x:c r="F7" s="48" t="str">
+        <x:f t="shared" si="2">IF($W$20&lt;&gt;"",$W$20&amp;REPT(" ",MAX(2,18-LEN($W$20)))&amp;DAY($V$20),REPT(" ",16-LEN(DAY($V$20)))&amp;DAY($V$20))</x:f>
+        <x:v>              13</x:v>
+      </x:c>
+      <x:c r="G7" s="48" t="str">
+        <x:f t="shared" si="2">IF($W$21&lt;&gt;"",$W$21&amp;REPT(" ",MAX(2,18-LEN($W$21)))&amp;DAY($V$21),REPT(" ",16-LEN(DAY($V$21)))&amp;DAY($V$21))</x:f>
+        <x:v>              14</x:v>
+      </x:c>
+      <x:c r="H7" s="49" t="str">
+        <x:f t="shared" si="2">IF($W$22&lt;&gt;"",$W$22&amp;REPT(" ",MAX(2,18-LEN($W$22)))&amp;DAY($V$22),REPT(" ",16-LEN(DAY($V$22)))&amp;DAY($V$22))</x:f>
+        <x:v>광복절               15</x:v>
       </x:c>
       <x:c r="I7" s="1"/>
       <x:c r="J7" s="37" t="str"/>
@@ -3822,29 +4120,35 @@
       <x:c r="U7" s="45" t="str">
         <x:f>IF(OR(J7="",Q7&lt;&gt;""),"",J7&amp;"|"&amp;R7)</x:f>
       </x:c>
+      <x:c r="V7" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+5</x:f>
+        <x:v>46234</x:v>
+      </x:c>
+      <x:c r="W7" s="45" t="str">
+        <x:f>XLOOKUP(V7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="8" ht="72" customHeight="1">
-      <x:c r="B8" s="49" t="str">
-        <x:f>IF(XLOOKUP(B7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(B7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(B7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(B7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(B7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="C8" s="51" t="str">
-        <x:f>IF(XLOOKUP(C7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(C7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(C7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(C7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(C7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="D8" s="51" t="str">
-        <x:f>IF(XLOOKUP(D7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(D7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(D7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(D7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(D7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="E8" s="51" t="str">
-        <x:f>IF(XLOOKUP(E7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(E7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(E7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(E7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(E7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="F8" s="51" t="str">
-        <x:f>IF(XLOOKUP(F7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(F7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(F7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(F7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(F7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="G8" s="51" t="str">
-        <x:f>IF(XLOOKUP(G7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(G7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(G7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(G7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(G7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="H8" s="52" t="str">
-        <x:f>IF(XLOOKUP(H7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(H7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(H7,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(H7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(H7&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H7&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H7&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H7&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H7&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-        <x:v>◆ 광복절</x:v>
+      <x:c r="B8" s="50" t="str">
+        <x:f>XLOOKUP($V$16&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$16&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$16&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$16&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$16&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$16&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$16&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$16&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$16&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="C8" s="52" t="str">
+        <x:f>XLOOKUP($V$17&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$17&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$17&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$17&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$17&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$17&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$17&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$17&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$17&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="D8" s="52" t="str">
+        <x:f>XLOOKUP($V$18&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$18&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$18&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$18&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$18&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$18&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$18&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$18&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$18&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="E8" s="52" t="str">
+        <x:f>XLOOKUP($V$19&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$19&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$19&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$19&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$19&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$19&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$19&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$19&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$19&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="F8" s="52" t="str">
+        <x:f>XLOOKUP($V$20&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$20&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$20&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$20&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$20&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$20&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$20&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$20&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$20&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="G8" s="52" t="str">
+        <x:f>XLOOKUP($V$21&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$21&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$21&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$21&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$21&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$21&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$21&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$21&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$21&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="H8" s="53" t="str">
+        <x:f>XLOOKUP($V$22&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$22&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$22&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$22&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$22&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$22&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$22&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$22&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$22&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="I8" s="1"/>
       <x:c r="J8" s="37" t="str"/>
@@ -3868,35 +4172,42 @@
       <x:c r="U8" s="45" t="str">
         <x:f>IF(OR(J8="",Q8&lt;&gt;""),"",J8&amp;"|"&amp;R8)</x:f>
       </x:c>
+      <x:c r="V8" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+6</x:f>
+        <x:v>46235</x:v>
+      </x:c>
+      <x:c r="W8" s="45" t="str">
+        <x:f>XLOOKUP(V8,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
-      <x:c r="B9" s="46">
-        <x:f>H7+1</x:f>
-        <x:v>46250</x:v>
-      </x:c>
-      <x:c r="C9" s="47">
-        <x:f t="shared" ref="C9:H9" si="3">B9+1</x:f>
-        <x:v>46251</x:v>
-      </x:c>
-      <x:c r="D9" s="47">
-        <x:f t="shared" si="3"/>
-        <x:v>46252</x:v>
-      </x:c>
-      <x:c r="E9" s="47">
-        <x:f t="shared" si="3"/>
-        <x:v>46253</x:v>
-      </x:c>
-      <x:c r="F9" s="47">
-        <x:f t="shared" si="3"/>
-        <x:v>46254</x:v>
-      </x:c>
-      <x:c r="G9" s="47">
-        <x:f t="shared" si="3"/>
-        <x:v>46255</x:v>
-      </x:c>
-      <x:c r="H9" s="48">
-        <x:f t="shared" si="3"/>
-        <x:v>46256</x:v>
+      <x:c r="B9" s="47" t="str">
+        <x:f>IF($W$23&lt;&gt;"",$W$23&amp;REPT(" ",MAX(2,18-LEN($W$23)))&amp;DAY($V$23),REPT(" ",16-LEN(DAY($V$23)))&amp;DAY($V$23))</x:f>
+        <x:v>              16</x:v>
+      </x:c>
+      <x:c r="C9" s="48" t="str">
+        <x:f t="shared" ref="C9:H9" si="3">IF($W$24&lt;&gt;"",$W$24&amp;REPT(" ",MAX(2,18-LEN($W$24)))&amp;DAY($V$24),REPT(" ",16-LEN(DAY($V$24)))&amp;DAY($V$24))</x:f>
+        <x:v>광복절 대체 휴일         17</x:v>
+      </x:c>
+      <x:c r="D9" s="48" t="str">
+        <x:f t="shared" si="3">IF($W$25&lt;&gt;"",$W$25&amp;REPT(" ",MAX(2,18-LEN($W$25)))&amp;DAY($V$25),REPT(" ",16-LEN(DAY($V$25)))&amp;DAY($V$25))</x:f>
+        <x:v>              18</x:v>
+      </x:c>
+      <x:c r="E9" s="48" t="str">
+        <x:f t="shared" si="3">IF($W$26&lt;&gt;"",$W$26&amp;REPT(" ",MAX(2,18-LEN($W$26)))&amp;DAY($V$26),REPT(" ",16-LEN(DAY($V$26)))&amp;DAY($V$26))</x:f>
+        <x:v>              19</x:v>
+      </x:c>
+      <x:c r="F9" s="48" t="str">
+        <x:f t="shared" si="3">IF($W$27&lt;&gt;"",$W$27&amp;REPT(" ",MAX(2,18-LEN($W$27)))&amp;DAY($V$27),REPT(" ",16-LEN(DAY($V$27)))&amp;DAY($V$27))</x:f>
+        <x:v>              20</x:v>
+      </x:c>
+      <x:c r="G9" s="48" t="str">
+        <x:f t="shared" si="3">IF($W$28&lt;&gt;"",$W$28&amp;REPT(" ",MAX(2,18-LEN($W$28)))&amp;DAY($V$28),REPT(" ",16-LEN(DAY($V$28)))&amp;DAY($V$28))</x:f>
+        <x:v>              21</x:v>
+      </x:c>
+      <x:c r="H9" s="49" t="str">
+        <x:f t="shared" si="3">IF($W$29&lt;&gt;"",$W$29&amp;REPT(" ",MAX(2,18-LEN($W$29)))&amp;DAY($V$29),REPT(" ",16-LEN(DAY($V$29)))&amp;DAY($V$29))</x:f>
+        <x:v>              22</x:v>
       </x:c>
       <x:c r="I9" s="1"/>
       <x:c r="J9" s="37" t="str"/>
@@ -3918,29 +4229,35 @@
       <x:c r="U9" s="45" t="str">
         <x:f>IF(OR(J9="",Q9&lt;&gt;""),"",J9&amp;"|"&amp;R9)</x:f>
       </x:c>
+      <x:c r="V9" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+7</x:f>
+        <x:v>46236</x:v>
+      </x:c>
+      <x:c r="W9" s="45" t="str">
+        <x:f>XLOOKUP(V9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="10" ht="72" customHeight="1">
-      <x:c r="B10" s="49" t="str">
-        <x:f>IF(XLOOKUP(B9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(B9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(B9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(B9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(B9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="C10" s="51" t="str">
-        <x:f>IF(XLOOKUP(C9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(C9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(C9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(C9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(C9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-        <x:v>◆ 광복절 대체 휴일</x:v>
-      </x:c>
-      <x:c r="D10" s="51" t="str">
-        <x:f>IF(XLOOKUP(D9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(D9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(D9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(D9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(D9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="E10" s="51" t="str">
-        <x:f>IF(XLOOKUP(E9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(E9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(E9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(E9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(E9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="F10" s="51" t="str">
-        <x:f>IF(XLOOKUP(F9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(F9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(F9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(F9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(F9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="G10" s="51" t="str">
-        <x:f>IF(XLOOKUP(G9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(G9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(G9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(G9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(G9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="H10" s="52" t="str">
-        <x:f>IF(XLOOKUP(H9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(H9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(H9,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(H9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(H9&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H9&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H9&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H9&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H9&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      <x:c r="B10" s="50" t="str">
+        <x:f>XLOOKUP($V$23&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$23&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$23&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$23&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$23&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$23&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$23&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$23&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$23&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="C10" s="52" t="str">
+        <x:f>XLOOKUP($V$24&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$24&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$24&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$24&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$24&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$24&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$24&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$24&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$24&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="D10" s="52" t="str">
+        <x:f>XLOOKUP($V$25&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$25&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$25&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$25&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$25&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$25&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$25&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$25&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$25&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="E10" s="52" t="str">
+        <x:f>XLOOKUP($V$26&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$26&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$26&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$26&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$26&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$26&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$26&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$26&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$26&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="F10" s="52" t="str">
+        <x:f>XLOOKUP($V$27&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$27&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$27&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$27&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$27&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$27&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$27&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$27&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$27&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="G10" s="52" t="str">
+        <x:f>XLOOKUP($V$28&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$28&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$28&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$28&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$28&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$28&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$28&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$28&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$28&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="H10" s="53" t="str">
+        <x:f>XLOOKUP($V$29&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$29&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$29&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$29&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$29&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$29&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$29&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$29&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$29&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="I10" s="1"/>
       <x:c r="J10" s="37" t="str"/>
@@ -3962,35 +4279,42 @@
       <x:c r="U10" s="45" t="str">
         <x:f>IF(OR(J10="",Q10&lt;&gt;""),"",J10&amp;"|"&amp;R10)</x:f>
       </x:c>
+      <x:c r="V10" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+8</x:f>
+        <x:v>46237</x:v>
+      </x:c>
+      <x:c r="W10" s="45" t="str">
+        <x:f>XLOOKUP(V10,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
-      <x:c r="B11" s="46">
-        <x:f>H9+1</x:f>
-        <x:v>46257</x:v>
-      </x:c>
-      <x:c r="C11" s="47">
-        <x:f t="shared" ref="C11:H11" si="4">B11+1</x:f>
-        <x:v>46258</x:v>
-      </x:c>
-      <x:c r="D11" s="47">
-        <x:f t="shared" si="4"/>
-        <x:v>46259</x:v>
-      </x:c>
-      <x:c r="E11" s="47">
-        <x:f t="shared" si="4"/>
-        <x:v>46260</x:v>
-      </x:c>
-      <x:c r="F11" s="47">
-        <x:f t="shared" si="4"/>
-        <x:v>46261</x:v>
-      </x:c>
-      <x:c r="G11" s="47">
-        <x:f t="shared" si="4"/>
-        <x:v>46262</x:v>
-      </x:c>
-      <x:c r="H11" s="48">
-        <x:f t="shared" si="4"/>
-        <x:v>46263</x:v>
+      <x:c r="B11" s="47" t="str">
+        <x:f>IF($W$30&lt;&gt;"",$W$30&amp;REPT(" ",MAX(2,18-LEN($W$30)))&amp;DAY($V$30),REPT(" ",16-LEN(DAY($V$30)))&amp;DAY($V$30))</x:f>
+        <x:v>              23</x:v>
+      </x:c>
+      <x:c r="C11" s="48" t="str">
+        <x:f t="shared" ref="C11:H11" si="4">IF($W$31&lt;&gt;"",$W$31&amp;REPT(" ",MAX(2,18-LEN($W$31)))&amp;DAY($V$31),REPT(" ",16-LEN(DAY($V$31)))&amp;DAY($V$31))</x:f>
+        <x:v>              24</x:v>
+      </x:c>
+      <x:c r="D11" s="48" t="str">
+        <x:f t="shared" si="4">IF($W$32&lt;&gt;"",$W$32&amp;REPT(" ",MAX(2,18-LEN($W$32)))&amp;DAY($V$32),REPT(" ",16-LEN(DAY($V$32)))&amp;DAY($V$32))</x:f>
+        <x:v>              25</x:v>
+      </x:c>
+      <x:c r="E11" s="48" t="str">
+        <x:f t="shared" si="4">IF($W$33&lt;&gt;"",$W$33&amp;REPT(" ",MAX(2,18-LEN($W$33)))&amp;DAY($V$33),REPT(" ",16-LEN(DAY($V$33)))&amp;DAY($V$33))</x:f>
+        <x:v>              26</x:v>
+      </x:c>
+      <x:c r="F11" s="48" t="str">
+        <x:f t="shared" si="4">IF($W$34&lt;&gt;"",$W$34&amp;REPT(" ",MAX(2,18-LEN($W$34)))&amp;DAY($V$34),REPT(" ",16-LEN(DAY($V$34)))&amp;DAY($V$34))</x:f>
+        <x:v>              27</x:v>
+      </x:c>
+      <x:c r="G11" s="48" t="str">
+        <x:f t="shared" si="4">IF($W$35&lt;&gt;"",$W$35&amp;REPT(" ",MAX(2,18-LEN($W$35)))&amp;DAY($V$35),REPT(" ",16-LEN(DAY($V$35)))&amp;DAY($V$35))</x:f>
+        <x:v>              28</x:v>
+      </x:c>
+      <x:c r="H11" s="49" t="str">
+        <x:f t="shared" si="4">IF($W$36&lt;&gt;"",$W$36&amp;REPT(" ",MAX(2,18-LEN($W$36)))&amp;DAY($V$36),REPT(" ",16-LEN(DAY($V$36)))&amp;DAY($V$36))</x:f>
+        <x:v>              29</x:v>
       </x:c>
       <x:c r="I11" s="1"/>
       <x:c r="J11" s="37" t="str"/>
@@ -4012,28 +4336,35 @@
       <x:c r="U11" s="45" t="str">
         <x:f>IF(OR(J11="",Q11&lt;&gt;""),"",J11&amp;"|"&amp;R11)</x:f>
       </x:c>
+      <x:c r="V11" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+9</x:f>
+        <x:v>46238</x:v>
+      </x:c>
+      <x:c r="W11" s="45" t="str">
+        <x:f>XLOOKUP(V11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="12" ht="72" customHeight="1">
-      <x:c r="B12" s="49" t="str">
-        <x:f>IF(XLOOKUP(B11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(B11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(B11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(B11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(B11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="C12" s="51" t="str">
-        <x:f>IF(XLOOKUP(C11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(C11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(C11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(C11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(C11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="D12" s="51" t="str">
-        <x:f>IF(XLOOKUP(D11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(D11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(D11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(D11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(D11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="E12" s="51" t="str">
-        <x:f>IF(XLOOKUP(E11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(E11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(E11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(E11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(E11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="F12" s="51" t="str">
-        <x:f>IF(XLOOKUP(F11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(F11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(F11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(F11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(F11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="G12" s="51" t="str">
-        <x:f>IF(XLOOKUP(G11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(G11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(G11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(G11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(G11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="H12" s="52" t="str">
-        <x:f>IF(XLOOKUP(H11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(H11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(H11,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(H11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(H11&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H11&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H11&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H11&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H11&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      <x:c r="B12" s="50" t="str">
+        <x:f>XLOOKUP($V$30&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$30&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$30&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$30&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$30&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$30&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$30&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$30&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$30&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="C12" s="52" t="str">
+        <x:f>XLOOKUP($V$31&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$31&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$31&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$31&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$31&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$31&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$31&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$31&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$31&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="D12" s="52" t="str">
+        <x:f>XLOOKUP($V$32&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$32&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$32&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$32&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$32&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$32&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$32&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$32&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$32&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="E12" s="52" t="str">
+        <x:f>XLOOKUP($V$33&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$33&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$33&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$33&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$33&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$33&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$33&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$33&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$33&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="F12" s="52" t="str">
+        <x:f>XLOOKUP($V$34&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$34&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$34&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$34&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$34&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$34&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$34&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$34&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$34&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="G12" s="52" t="str">
+        <x:f>XLOOKUP($V$35&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$35&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$35&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$35&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$35&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$35&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$35&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$35&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$35&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="H12" s="53" t="str">
+        <x:f>XLOOKUP($V$36&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$36&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$36&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$36&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$36&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$36&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$36&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$36&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$36&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="I12" s="1"/>
       <x:c r="J12" s="37" t="str"/>
@@ -4055,35 +4386,42 @@
       <x:c r="U12" s="45" t="str">
         <x:f>IF(OR(J12="",Q12&lt;&gt;""),"",J12&amp;"|"&amp;R12)</x:f>
       </x:c>
+      <x:c r="V12" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+10</x:f>
+        <x:v>46239</x:v>
+      </x:c>
+      <x:c r="W12" s="45" t="str">
+        <x:f>XLOOKUP(V12,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
-      <x:c r="B13" s="46">
-        <x:f>H11+1</x:f>
-        <x:v>46264</x:v>
-      </x:c>
-      <x:c r="C13" s="47">
-        <x:f t="shared" ref="C13:H13" si="5">B13+1</x:f>
-        <x:v>46265</x:v>
-      </x:c>
-      <x:c r="D13" s="47">
-        <x:f t="shared" si="5"/>
-        <x:v>46266</x:v>
-      </x:c>
-      <x:c r="E13" s="47">
-        <x:f t="shared" si="5"/>
-        <x:v>46267</x:v>
-      </x:c>
-      <x:c r="F13" s="47">
-        <x:f t="shared" si="5"/>
-        <x:v>46268</x:v>
-      </x:c>
-      <x:c r="G13" s="47">
-        <x:f t="shared" si="5"/>
-        <x:v>46269</x:v>
-      </x:c>
-      <x:c r="H13" s="48">
-        <x:f t="shared" si="5"/>
-        <x:v>46270</x:v>
+      <x:c r="B13" s="47" t="str">
+        <x:f>IF($W$37&lt;&gt;"",$W$37&amp;REPT(" ",MAX(2,18-LEN($W$37)))&amp;DAY($V$37),REPT(" ",16-LEN(DAY($V$37)))&amp;DAY($V$37))</x:f>
+        <x:v>              30</x:v>
+      </x:c>
+      <x:c r="C13" s="48" t="str">
+        <x:f t="shared" ref="C13:H13" si="5">IF($W$38&lt;&gt;"",$W$38&amp;REPT(" ",MAX(2,18-LEN($W$38)))&amp;DAY($V$38),REPT(" ",16-LEN(DAY($V$38)))&amp;DAY($V$38))</x:f>
+        <x:v>              31</x:v>
+      </x:c>
+      <x:c r="D13" s="48" t="str">
+        <x:f t="shared" si="5">IF($W$39&lt;&gt;"",$W$39&amp;REPT(" ",MAX(2,18-LEN($W$39)))&amp;DAY($V$39),REPT(" ",16-LEN(DAY($V$39)))&amp;DAY($V$39))</x:f>
+        <x:v>               1</x:v>
+      </x:c>
+      <x:c r="E13" s="48" t="str">
+        <x:f t="shared" si="5">IF($W$40&lt;&gt;"",$W$40&amp;REPT(" ",MAX(2,18-LEN($W$40)))&amp;DAY($V$40),REPT(" ",16-LEN(DAY($V$40)))&amp;DAY($V$40))</x:f>
+        <x:v>               2</x:v>
+      </x:c>
+      <x:c r="F13" s="48" t="str">
+        <x:f t="shared" si="5">IF($W$41&lt;&gt;"",$W$41&amp;REPT(" ",MAX(2,18-LEN($W$41)))&amp;DAY($V$41),REPT(" ",16-LEN(DAY($V$41)))&amp;DAY($V$41))</x:f>
+        <x:v>               3</x:v>
+      </x:c>
+      <x:c r="G13" s="48" t="str">
+        <x:f t="shared" si="5">IF($W$42&lt;&gt;"",$W$42&amp;REPT(" ",MAX(2,18-LEN($W$42)))&amp;DAY($V$42),REPT(" ",16-LEN(DAY($V$42)))&amp;DAY($V$42))</x:f>
+        <x:v>               4</x:v>
+      </x:c>
+      <x:c r="H13" s="49" t="str">
+        <x:f t="shared" si="5">IF($W$43&lt;&gt;"",$W$43&amp;REPT(" ",MAX(2,18-LEN($W$43)))&amp;DAY($V$43),REPT(" ",16-LEN(DAY($V$43)))&amp;DAY($V$43))</x:f>
+        <x:v>               5</x:v>
       </x:c>
       <x:c r="I13" s="1"/>
       <x:c r="J13" s="37" t="str"/>
@@ -4105,28 +4443,35 @@
       <x:c r="U13" s="45" t="str">
         <x:f>IF(OR(J13="",Q13&lt;&gt;""),"",J13&amp;"|"&amp;R13)</x:f>
       </x:c>
+      <x:c r="V13" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+11</x:f>
+        <x:v>46240</x:v>
+      </x:c>
+      <x:c r="W13" s="45" t="str">
+        <x:f>XLOOKUP(V13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="14" ht="72" customHeight="1">
-      <x:c r="B14" s="53" t="str">
-        <x:f>IF(XLOOKUP(B13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(B13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(B13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(B13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(B13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(B13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(B13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(B13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="C14" s="54" t="str">
-        <x:f>IF(XLOOKUP(C13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(C13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(C13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(C13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(C13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(C13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(C13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(C13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="D14" s="54" t="str">
-        <x:f>IF(XLOOKUP(D13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(D13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(D13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(D13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(D13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(D13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(D13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(D13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="E14" s="54" t="str">
-        <x:f>IF(XLOOKUP(E13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(E13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(E13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(E13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(E13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(E13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(E13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(E13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="F14" s="54" t="str">
-        <x:f>IF(XLOOKUP(F13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(F13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(F13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(F13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(F13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(F13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(F13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(F13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="G14" s="54" t="str">
-        <x:f>IF(XLOOKUP(G13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(G13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(G13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(G13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(G13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(G13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(G13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(G13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
-      </x:c>
-      <x:c r="H14" s="55" t="str">
-        <x:f>IF(XLOOKUP(H13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")="","","◆ "&amp;XLOOKUP(H13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,""))&amp;IF(AND(XLOOKUP(H13,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")&lt;&gt;"",XLOOKUP(H13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&lt;&gt;""),CHAR(10),"")&amp;XLOOKUP(H13&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP(H13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H13&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H13&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H13&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP(H13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP(H13&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      <x:c r="B14" s="54" t="str">
+        <x:f>XLOOKUP($V$37&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$37&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$37&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$37&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$37&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$37&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$37&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$37&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$37&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="C14" s="55" t="str">
+        <x:f>XLOOKUP($V$38&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$38&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$38&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$38&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$38&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$38&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$38&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$38&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$38&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="D14" s="55" t="str">
+        <x:f>XLOOKUP($V$39&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$39&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$39&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$39&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$39&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$39&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$39&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$39&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$39&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="E14" s="55" t="str">
+        <x:f>XLOOKUP($V$40&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$40&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$40&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$40&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$40&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$40&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$40&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$40&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$40&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="F14" s="55" t="str">
+        <x:f>XLOOKUP($V$41&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$41&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$41&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$41&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$41&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$41&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$41&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$41&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$41&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="G14" s="55" t="str">
+        <x:f>XLOOKUP($V$42&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$42&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$42&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$42&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$42&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$42&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$42&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$42&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$42&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
+      </x:c>
+      <x:c r="H14" s="56" t="str">
+        <x:f>XLOOKUP($V$43&amp;"|"&amp;1,$U$5:$U$504,$K$5:$K$504,"")&amp;IF(XLOOKUP($V$43&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$43&amp;"|"&amp;2,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$43&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$43&amp;"|"&amp;3,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$43&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$43&amp;"|"&amp;4,$U$5:$U$504,$K$5:$K$504,""))&amp;IF(XLOOKUP($V$43&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,"")="","",CHAR(10)&amp;XLOOKUP($V$43&amp;"|"&amp;5,$U$5:$U$504,$K$5:$K$504,""))</x:f>
       </x:c>
       <x:c r="I14" s="2"/>
       <x:c r="J14" s="37" t="str"/>
@@ -4148,6 +4493,13 @@
       <x:c r="U14" s="45" t="str">
         <x:f>IF(OR(J14="",Q14&lt;&gt;""),"",J14&amp;"|"&amp;R14)</x:f>
       </x:c>
+      <x:c r="V14" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+12</x:f>
+        <x:v>46241</x:v>
+      </x:c>
+      <x:c r="W14" s="45" t="str">
+        <x:f>XLOOKUP(V14,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
       <x:c r="J15" s="37" t="str"/>
@@ -4169,6 +4521,13 @@
       <x:c r="U15" s="45" t="str">
         <x:f>IF(OR(J15="",Q15&lt;&gt;""),"",J15&amp;"|"&amp;R15)</x:f>
       </x:c>
+      <x:c r="V15" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+13</x:f>
+        <x:v>46242</x:v>
+      </x:c>
+      <x:c r="W15" s="45" t="str">
+        <x:f>XLOOKUP(V15,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="16" ht="22" customHeight="1">
       <x:c r="J16" s="37" t="str"/>
@@ -4190,18 +4549,25 @@
       <x:c r="U16" s="45" t="str">
         <x:f>IF(OR(J16="",Q16&lt;&gt;""),"",J16&amp;"|"&amp;R16)</x:f>
       </x:c>
+      <x:c r="V16" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+14</x:f>
+        <x:v>46243</x:v>
+      </x:c>
+      <x:c r="W16" s="45" t="str">
+        <x:f>XLOOKUP(V16,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
-      <x:c r="B17" s="57" t="str">
+      <x:c r="B17" s="58" t="str">
         <x:v>Cellendar 사용 방법</x:v>
       </x:c>
-      <x:c r="C17" s="57"/>
-      <x:c r="D17" s="57"/>
-      <x:c r="E17" s="57"/>
-      <x:c r="F17" s="57"/>
-      <x:c r="G17" s="57"/>
-      <x:c r="H17" s="57"/>
-      <x:c r="I17" s="57"/>
+      <x:c r="C17" s="58"/>
+      <x:c r="D17" s="58"/>
+      <x:c r="E17" s="58"/>
+      <x:c r="F17" s="58"/>
+      <x:c r="G17" s="58"/>
+      <x:c r="H17" s="58"/>
+      <x:c r="I17" s="58"/>
       <x:c r="J17" s="37" t="str"/>
       <x:c r="K17" s="33" t="str"/>
       <x:c r="L17" s="33" t="str"/>
@@ -4221,20 +4587,27 @@
       <x:c r="U17" s="45" t="str">
         <x:f>IF(OR(J17="",Q17&lt;&gt;""),"",J17&amp;"|"&amp;R17)</x:f>
       </x:c>
+      <x:c r="V17" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+15</x:f>
+        <x:v>46244</x:v>
+      </x:c>
+      <x:c r="W17" s="45" t="str">
+        <x:f>XLOOKUP(V17,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="18" ht="27" customHeight="1">
-      <x:c r="B18" s="58" t="str">
+      <x:c r="B18" s="59" t="str">
         <x:v>1. 일정 입력</x:v>
       </x:c>
-      <x:c r="C18" s="58"/>
-      <x:c r="D18" s="61" t="str">
+      <x:c r="C18" s="59"/>
+      <x:c r="D18" s="62" t="str">
         <x:v>오른쪽 노란 표에서 날짜와 색상을 목록으로 선택하고 제목을 입력하세요.</x:v>
       </x:c>
-      <x:c r="E18" s="61"/>
-      <x:c r="F18" s="61"/>
-      <x:c r="G18" s="61"/>
-      <x:c r="H18" s="61"/>
-      <x:c r="I18" s="61"/>
+      <x:c r="E18" s="62"/>
+      <x:c r="F18" s="62"/>
+      <x:c r="G18" s="62"/>
+      <x:c r="H18" s="62"/>
+      <x:c r="I18" s="62"/>
       <x:c r="J18" s="37" t="str"/>
       <x:c r="K18" s="33" t="str"/>
       <x:c r="L18" s="33" t="str"/>
@@ -4254,20 +4627,27 @@
       <x:c r="U18" s="45" t="str">
         <x:f>IF(OR(J18="",Q18&lt;&gt;""),"",J18&amp;"|"&amp;R18)</x:f>
       </x:c>
+      <x:c r="V18" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+16</x:f>
+        <x:v>46245</x:v>
+      </x:c>
+      <x:c r="W18" s="45" t="str">
+        <x:f>XLOOKUP(V18,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="19" ht="27" customHeight="1">
-      <x:c r="B19" s="58" t="str">
+      <x:c r="B19" s="59" t="str">
         <x:v>2. 달력 표시</x:v>
       </x:c>
-      <x:c r="C19" s="58"/>
-      <x:c r="D19" s="61" t="str">
+      <x:c r="C19" s="59"/>
+      <x:c r="D19" s="62" t="str">
         <x:v>같은 날짜의 일정은 달력 칸에 줄바꿈으로 최대 5개까지 표시됩니다.</x:v>
       </x:c>
-      <x:c r="E19" s="61"/>
-      <x:c r="F19" s="61"/>
-      <x:c r="G19" s="61"/>
-      <x:c r="H19" s="61"/>
-      <x:c r="I19" s="61"/>
+      <x:c r="E19" s="62"/>
+      <x:c r="F19" s="62"/>
+      <x:c r="G19" s="62"/>
+      <x:c r="H19" s="62"/>
+      <x:c r="I19" s="62"/>
       <x:c r="J19" s="37" t="str"/>
       <x:c r="K19" s="33" t="str"/>
       <x:c r="L19" s="33" t="str"/>
@@ -4287,20 +4667,27 @@
       <x:c r="U19" s="45" t="str">
         <x:f>IF(OR(J19="",Q19&lt;&gt;""),"",J19&amp;"|"&amp;R19)</x:f>
       </x:c>
+      <x:c r="V19" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+17</x:f>
+        <x:v>46246</x:v>
+      </x:c>
+      <x:c r="W19" s="45" t="str">
+        <x:f>XLOOKUP(V19,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="20" ht="27" customHeight="1">
-      <x:c r="B20" s="58" t="str">
-        <x:v>3. 다음 달</x:v>
-      </x:c>
-      <x:c r="C20" s="58"/>
-      <x:c r="D20" s="61" t="str">
-        <x:v>상단의 연도와 월 숫자만 바꾸면 달력과 날짜 선택 목록이 함께 변경됩니다.</x:v>
-      </x:c>
-      <x:c r="E20" s="61"/>
-      <x:c r="F20" s="61"/>
-      <x:c r="G20" s="61"/>
-      <x:c r="H20" s="61"/>
-      <x:c r="I20" s="61"/>
+      <x:c r="B20" s="59" t="str">
+        <x:v>공휴일</x:v>
+      </x:c>
+      <x:c r="C20" s="59"/>
+      <x:c r="D20" s="62" t="str">
+        <x:v>공휴일 시트의 휴일명은 날짜 숫자 왼쪽에 표시되고 날짜와 함께 빨간색으로 표시됩니다.</x:v>
+      </x:c>
+      <x:c r="E20" s="62"/>
+      <x:c r="F20" s="62"/>
+      <x:c r="G20" s="62"/>
+      <x:c r="H20" s="62"/>
+      <x:c r="I20" s="62"/>
       <x:c r="J20" s="37" t="str"/>
       <x:c r="K20" s="33" t="str"/>
       <x:c r="L20" s="33" t="str"/>
@@ -4320,20 +4707,27 @@
       <x:c r="U20" s="45" t="str">
         <x:f>IF(OR(J20="",Q20&lt;&gt;""),"",J20&amp;"|"&amp;R20)</x:f>
       </x:c>
+      <x:c r="V20" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+18</x:f>
+        <x:v>46247</x:v>
+      </x:c>
+      <x:c r="W20" s="45" t="str">
+        <x:f>XLOOKUP(V20,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="21" ht="27" customHeight="1">
-      <x:c r="B21" s="58" t="str">
-        <x:v>4. 비고 사용</x:v>
-      </x:c>
-      <x:c r="C21" s="58"/>
-      <x:c r="D21" s="61" t="str">
-        <x:v>초록색 비고 영역은 동기화와 관계없이 자유롭게 작성할 수 있습니다.</x:v>
-      </x:c>
-      <x:c r="E21" s="61"/>
-      <x:c r="F21" s="61"/>
-      <x:c r="G21" s="61"/>
-      <x:c r="H21" s="61"/>
-      <x:c r="I21" s="61"/>
+      <x:c r="B21" s="59" t="str">
+        <x:v>3. 다음 달</x:v>
+      </x:c>
+      <x:c r="C21" s="59"/>
+      <x:c r="D21" s="62" t="str">
+        <x:v>상단의 연도와 월 숫자만 바꾸면 달력과 날짜 선택 목록이 함께 변경됩니다.</x:v>
+      </x:c>
+      <x:c r="E21" s="62"/>
+      <x:c r="F21" s="62"/>
+      <x:c r="G21" s="62"/>
+      <x:c r="H21" s="62"/>
+      <x:c r="I21" s="62"/>
       <x:c r="J21" s="37" t="str"/>
       <x:c r="K21" s="33" t="str"/>
       <x:c r="L21" s="33" t="str"/>
@@ -4353,20 +4747,27 @@
       <x:c r="U21" s="45" t="str">
         <x:f>IF(OR(J21="",Q21&lt;&gt;""),"",J21&amp;"|"&amp;R21)</x:f>
       </x:c>
+      <x:c r="V21" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+19</x:f>
+        <x:v>46248</x:v>
+      </x:c>
+      <x:c r="W21" s="45" t="str">
+        <x:f>XLOOKUP(V21,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="22" ht="27" customHeight="1">
-      <x:c r="B22" s="58" t="str">
-        <x:v>5. 앱 동기화</x:v>
-      </x:c>
-      <x:c r="C22" s="58"/>
-      <x:c r="D22" s="61" t="str">
-        <x:v>엑셀을 OneDrive의 Cellendar 폴더에 저장한 뒤 앱의 동기화 버튼을 누르세요.</x:v>
-      </x:c>
-      <x:c r="E22" s="61"/>
-      <x:c r="F22" s="61"/>
-      <x:c r="G22" s="61"/>
-      <x:c r="H22" s="61"/>
-      <x:c r="I22" s="61"/>
+      <x:c r="B22" s="59" t="str">
+        <x:v>4. 비고 사용</x:v>
+      </x:c>
+      <x:c r="C22" s="59"/>
+      <x:c r="D22" s="62" t="str">
+        <x:v>초록색 비고 영역은 동기화와 관계없이 자유롭게 작성할 수 있습니다.</x:v>
+      </x:c>
+      <x:c r="E22" s="62"/>
+      <x:c r="F22" s="62"/>
+      <x:c r="G22" s="62"/>
+      <x:c r="H22" s="62"/>
+      <x:c r="I22" s="62"/>
       <x:c r="J22" s="37" t="str"/>
       <x:c r="K22" s="33" t="str"/>
       <x:c r="L22" s="33" t="str"/>
@@ -4386,20 +4787,28 @@
       <x:c r="U22" s="45" t="str">
         <x:f>IF(OR(J22="",Q22&lt;&gt;""),"",J22&amp;"|"&amp;R22)</x:f>
       </x:c>
+      <x:c r="V22" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+20</x:f>
+        <x:v>46249</x:v>
+      </x:c>
+      <x:c r="W22" s="45" t="str">
+        <x:f>XLOOKUP(V22,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+        <x:v>광복절</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="27" customHeight="1">
-      <x:c r="B23" s="58" t="str">
-        <x:v>6. 수정·삭제</x:v>
-      </x:c>
-      <x:c r="C23" s="58"/>
-      <x:c r="D23" s="61" t="str">
-        <x:v>휴대폰 앱에서 일정을 누르면 수정하거나 삭제할 수 있습니다.</x:v>
-      </x:c>
-      <x:c r="E23" s="61"/>
-      <x:c r="F23" s="61"/>
-      <x:c r="G23" s="61"/>
-      <x:c r="H23" s="61"/>
-      <x:c r="I23" s="61"/>
+      <x:c r="B23" s="59" t="str">
+        <x:v>5. 앱 동기화</x:v>
+      </x:c>
+      <x:c r="C23" s="59"/>
+      <x:c r="D23" s="62" t="str">
+        <x:v>엑셀을 OneDrive의 Cellendar 폴더에 저장한 뒤 앱의 동기화 버튼을 누르세요.</x:v>
+      </x:c>
+      <x:c r="E23" s="62"/>
+      <x:c r="F23" s="62"/>
+      <x:c r="G23" s="62"/>
+      <x:c r="H23" s="62"/>
+      <x:c r="I23" s="62"/>
       <x:c r="J23" s="37" t="str"/>
       <x:c r="K23" s="33" t="str"/>
       <x:c r="L23" s="33" t="str"/>
@@ -4419,20 +4828,27 @@
       <x:c r="U23" s="45" t="str">
         <x:f>IF(OR(J23="",Q23&lt;&gt;""),"",J23&amp;"|"&amp;R23)</x:f>
       </x:c>
+      <x:c r="V23" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+21</x:f>
+        <x:v>46250</x:v>
+      </x:c>
+      <x:c r="W23" s="45" t="str">
+        <x:f>XLOOKUP(V23,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="24" ht="27" customHeight="1">
-      <x:c r="B24" s="63" t="str">
-        <x:v>주의</x:v>
-      </x:c>
-      <x:c r="C24" s="63"/>
-      <x:c r="D24" s="66" t="str">
-        <x:v>회색 ID·수정시간·삭제시간 칸과 내부 조회 영역은 수정하지 마세요.</x:v>
-      </x:c>
-      <x:c r="E24" s="66"/>
-      <x:c r="F24" s="66"/>
-      <x:c r="G24" s="66"/>
-      <x:c r="H24" s="66"/>
-      <x:c r="I24" s="66"/>
+      <x:c r="B24" s="59" t="str">
+        <x:v>6. 수정·삭제</x:v>
+      </x:c>
+      <x:c r="C24" s="59"/>
+      <x:c r="D24" s="62" t="str">
+        <x:v>휴대폰 앱에서 일정을 누르면 수정하거나 삭제할 수 있습니다.</x:v>
+      </x:c>
+      <x:c r="E24" s="62"/>
+      <x:c r="F24" s="62"/>
+      <x:c r="G24" s="62"/>
+      <x:c r="H24" s="62"/>
+      <x:c r="I24" s="62"/>
       <x:c r="J24" s="37" t="str"/>
       <x:c r="K24" s="33" t="str"/>
       <x:c r="L24" s="33" t="str"/>
@@ -4452,8 +4868,28 @@
       <x:c r="U24" s="45" t="str">
         <x:f>IF(OR(J24="",Q24&lt;&gt;""),"",J24&amp;"|"&amp;R24)</x:f>
       </x:c>
-    </x:row>
-    <x:row r="25" ht="22" customHeight="1">
+      <x:c r="V24" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+22</x:f>
+        <x:v>46251</x:v>
+      </x:c>
+      <x:c r="W24" s="45" t="str">
+        <x:f>XLOOKUP(V24,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+        <x:v>광복절 대체 휴일</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="27" customHeight="1">
+      <x:c r="B25" s="64" t="str">
+        <x:v>주의</x:v>
+      </x:c>
+      <x:c r="C25" s="64"/>
+      <x:c r="D25" s="67" t="str">
+        <x:v>회색 ID·수정시간·삭제시간 칸과 내부 조회 영역은 수정하지 마세요.</x:v>
+      </x:c>
+      <x:c r="E25" s="67"/>
+      <x:c r="F25" s="67"/>
+      <x:c r="G25" s="67"/>
+      <x:c r="H25" s="67"/>
+      <x:c r="I25" s="67"/>
       <x:c r="J25" s="37" t="str"/>
       <x:c r="K25" s="33" t="str"/>
       <x:c r="L25" s="33" t="str"/>
@@ -4472,6 +4908,13 @@
       <x:c r="T25" s="43"/>
       <x:c r="U25" s="45" t="str">
         <x:f>IF(OR(J25="",Q25&lt;&gt;""),"",J25&amp;"|"&amp;R25)</x:f>
+      </x:c>
+      <x:c r="V25" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+23</x:f>
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="W25" s="45" t="str">
+        <x:f>XLOOKUP(V25,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
       </x:c>
     </x:row>
     <x:row r="26" ht="22" customHeight="1">
@@ -4494,6 +4937,13 @@
       <x:c r="U26" s="45" t="str">
         <x:f>IF(OR(J26="",Q26&lt;&gt;""),"",J26&amp;"|"&amp;R26)</x:f>
       </x:c>
+      <x:c r="V26" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+24</x:f>
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="W26" s="45" t="str">
+        <x:f>XLOOKUP(V26,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="27" ht="22" customHeight="1">
       <x:c r="J27" s="37" t="str"/>
@@ -4515,6 +4965,13 @@
       <x:c r="U27" s="45" t="str">
         <x:f>IF(OR(J27="",Q27&lt;&gt;""),"",J27&amp;"|"&amp;R27)</x:f>
       </x:c>
+      <x:c r="V27" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+25</x:f>
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="W27" s="45" t="str">
+        <x:f>XLOOKUP(V27,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="28" ht="22" customHeight="1">
       <x:c r="J28" s="37" t="str"/>
@@ -4536,6 +4993,13 @@
       <x:c r="U28" s="45" t="str">
         <x:f>IF(OR(J28="",Q28&lt;&gt;""),"",J28&amp;"|"&amp;R28)</x:f>
       </x:c>
+      <x:c r="V28" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+26</x:f>
+        <x:v>46255</x:v>
+      </x:c>
+      <x:c r="W28" s="45" t="str">
+        <x:f>XLOOKUP(V28,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="29" ht="22" customHeight="1">
       <x:c r="J29" s="37" t="str"/>
@@ -4557,6 +5021,13 @@
       <x:c r="U29" s="45" t="str">
         <x:f>IF(OR(J29="",Q29&lt;&gt;""),"",J29&amp;"|"&amp;R29)</x:f>
       </x:c>
+      <x:c r="V29" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+27</x:f>
+        <x:v>46256</x:v>
+      </x:c>
+      <x:c r="W29" s="45" t="str">
+        <x:f>XLOOKUP(V29,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="30" ht="22" customHeight="1">
       <x:c r="J30" s="37" t="str"/>
@@ -4578,6 +5049,13 @@
       <x:c r="U30" s="45" t="str">
         <x:f>IF(OR(J30="",Q30&lt;&gt;""),"",J30&amp;"|"&amp;R30)</x:f>
       </x:c>
+      <x:c r="V30" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+28</x:f>
+        <x:v>46257</x:v>
+      </x:c>
+      <x:c r="W30" s="45" t="str">
+        <x:f>XLOOKUP(V30,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="31" ht="22" customHeight="1">
       <x:c r="J31" s="37" t="str"/>
@@ -4599,6 +5077,13 @@
       <x:c r="U31" s="45" t="str">
         <x:f>IF(OR(J31="",Q31&lt;&gt;""),"",J31&amp;"|"&amp;R31)</x:f>
       </x:c>
+      <x:c r="V31" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+29</x:f>
+        <x:v>46258</x:v>
+      </x:c>
+      <x:c r="W31" s="45" t="str">
+        <x:f>XLOOKUP(V31,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="32" ht="22" customHeight="1">
       <x:c r="J32" s="37" t="str"/>
@@ -4620,6 +5105,13 @@
       <x:c r="U32" s="45" t="str">
         <x:f>IF(OR(J32="",Q32&lt;&gt;""),"",J32&amp;"|"&amp;R32)</x:f>
       </x:c>
+      <x:c r="V32" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+30</x:f>
+        <x:v>46259</x:v>
+      </x:c>
+      <x:c r="W32" s="45" t="str">
+        <x:f>XLOOKUP(V32,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="33" ht="22" customHeight="1">
       <x:c r="J33" s="37" t="str"/>
@@ -4636,6 +5128,13 @@
       <x:c r="U33" s="45" t="str">
         <x:f>IF(OR(J33="",Q33&lt;&gt;""),"",J33&amp;"|"&amp;R33)</x:f>
       </x:c>
+      <x:c r="V33" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+31</x:f>
+        <x:v>46260</x:v>
+      </x:c>
+      <x:c r="W33" s="45" t="str">
+        <x:f>XLOOKUP(V33,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="34" ht="22" customHeight="1">
       <x:c r="J34" s="37" t="str"/>
@@ -4652,6 +5151,13 @@
       <x:c r="U34" s="45" t="str">
         <x:f>IF(OR(J34="",Q34&lt;&gt;""),"",J34&amp;"|"&amp;R34)</x:f>
       </x:c>
+      <x:c r="V34" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+32</x:f>
+        <x:v>46261</x:v>
+      </x:c>
+      <x:c r="W34" s="45" t="str">
+        <x:f>XLOOKUP(V34,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="R35" s="45" t="str">
@@ -4660,6 +5166,13 @@
       <x:c r="U35" s="45" t="str">
         <x:f>IF(OR(J35="",Q35&lt;&gt;""),"",J35&amp;"|"&amp;R35)</x:f>
       </x:c>
+      <x:c r="V35" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+33</x:f>
+        <x:v>46262</x:v>
+      </x:c>
+      <x:c r="W35" s="45" t="str">
+        <x:f>XLOOKUP(V35,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="R36" s="45" t="str">
@@ -4668,6 +5181,13 @@
       <x:c r="U36" s="45" t="str">
         <x:f>IF(OR(J36="",Q36&lt;&gt;""),"",J36&amp;"|"&amp;R36)</x:f>
       </x:c>
+      <x:c r="V36" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+34</x:f>
+        <x:v>46263</x:v>
+      </x:c>
+      <x:c r="W36" s="45" t="str">
+        <x:f>XLOOKUP(V36,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="R37" s="45" t="str">
@@ -4676,6 +5196,13 @@
       <x:c r="U37" s="45" t="str">
         <x:f>IF(OR(J37="",Q37&lt;&gt;""),"",J37&amp;"|"&amp;R37)</x:f>
       </x:c>
+      <x:c r="V37" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+35</x:f>
+        <x:v>46264</x:v>
+      </x:c>
+      <x:c r="W37" s="45" t="str">
+        <x:f>XLOOKUP(V37,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="R38" s="45" t="str">
@@ -4684,6 +5211,13 @@
       <x:c r="U38" s="45" t="str">
         <x:f>IF(OR(J38="",Q38&lt;&gt;""),"",J38&amp;"|"&amp;R38)</x:f>
       </x:c>
+      <x:c r="V38" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+36</x:f>
+        <x:v>46265</x:v>
+      </x:c>
+      <x:c r="W38" s="45" t="str">
+        <x:f>XLOOKUP(V38,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="R39" s="45" t="str">
@@ -4692,6 +5226,13 @@
       <x:c r="U39" s="45" t="str">
         <x:f>IF(OR(J39="",Q39&lt;&gt;""),"",J39&amp;"|"&amp;R39)</x:f>
       </x:c>
+      <x:c r="V39" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+37</x:f>
+        <x:v>46266</x:v>
+      </x:c>
+      <x:c r="W39" s="45" t="str">
+        <x:f>XLOOKUP(V39,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="40">
       <x:c r="R40" s="45" t="str">
@@ -4700,6 +5241,13 @@
       <x:c r="U40" s="45" t="str">
         <x:f>IF(OR(J40="",Q40&lt;&gt;""),"",J40&amp;"|"&amp;R40)</x:f>
       </x:c>
+      <x:c r="V40" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+38</x:f>
+        <x:v>46267</x:v>
+      </x:c>
+      <x:c r="W40" s="45" t="str">
+        <x:f>XLOOKUP(V40,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="41">
       <x:c r="R41" s="45" t="str">
@@ -4708,6 +5256,13 @@
       <x:c r="U41" s="45" t="str">
         <x:f>IF(OR(J41="",Q41&lt;&gt;""),"",J41&amp;"|"&amp;R41)</x:f>
       </x:c>
+      <x:c r="V41" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+39</x:f>
+        <x:v>46268</x:v>
+      </x:c>
+      <x:c r="W41" s="45" t="str">
+        <x:f>XLOOKUP(V41,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="42">
       <x:c r="R42" s="45" t="str">
@@ -4716,6 +5271,13 @@
       <x:c r="U42" s="45" t="str">
         <x:f>IF(OR(J42="",Q42&lt;&gt;""),"",J42&amp;"|"&amp;R42)</x:f>
       </x:c>
+      <x:c r="V42" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+40</x:f>
+        <x:v>46269</x:v>
+      </x:c>
+      <x:c r="W42" s="45" t="str">
+        <x:f>XLOOKUP(V42,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
+      </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="R43" s="45" t="str">
@@ -4723,6 +5285,13 @@
       </x:c>
       <x:c r="U43" s="45" t="str">
         <x:f>IF(OR(J43="",Q43&lt;&gt;""),"",J43&amp;"|"&amp;R43)</x:f>
+      </x:c>
+      <x:c r="V43" s="46" t="n">
+        <x:f>DATE($G$1,$H$1,1)-WEEKDAY(DATE($G$1,$H$1,1),1)+1+41</x:f>
+        <x:v>46270</x:v>
+      </x:c>
+      <x:c r="W43" s="45" t="str">
+        <x:f>XLOOKUP(V43,'공휴일'!$A$2:$A$306,'공휴일'!$B$2:$B$306,"")</x:f>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -8432,10 +9001,222 @@
     <x:mergeCell ref="D23:I23"/>
     <x:mergeCell ref="B24:C24"/>
     <x:mergeCell ref="D24:I24"/>
+    <x:mergeCell ref="B25:C25"/>
+    <x:mergeCell ref="D25:I25"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B3:H3 B5:H5 B7:H7 B9:H9 B11:H11 B13:H13">
     <x:cfRule type="expression" dxfId="1" priority="3" stopIfTrue="1">
       <x:formula>MONTH(B3)&lt;&gt;$H$1</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="B3:B3">
+    <x:cfRule type="expression" dxfId="2" priority="4">
+      <x:formula>$W$2&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C3:C3">
+    <x:cfRule type="expression" dxfId="3" priority="5">
+      <x:formula>$W$3&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="D3:D3">
+    <x:cfRule type="expression" dxfId="4" priority="6">
+      <x:formula>$W$4&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="E3:E3">
+    <x:cfRule type="expression" dxfId="5" priority="7">
+      <x:formula>$W$5&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="F3:F3">
+    <x:cfRule type="expression" dxfId="6" priority="8">
+      <x:formula>$W$6&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G3:G3">
+    <x:cfRule type="expression" dxfId="7" priority="9">
+      <x:formula>$W$7&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="H3:H3">
+    <x:cfRule type="expression" dxfId="8" priority="10">
+      <x:formula>$W$8&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="B5:B5">
+    <x:cfRule type="expression" dxfId="9" priority="11">
+      <x:formula>$W$9&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C5:C5">
+    <x:cfRule type="expression" dxfId="10" priority="12">
+      <x:formula>$W$10&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="D5:D5">
+    <x:cfRule type="expression" dxfId="11" priority="13">
+      <x:formula>$W$11&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="E5:E5">
+    <x:cfRule type="expression" dxfId="12" priority="14">
+      <x:formula>$W$12&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="F5:F5">
+    <x:cfRule type="expression" dxfId="13" priority="15">
+      <x:formula>$W$13&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G5:G5">
+    <x:cfRule type="expression" dxfId="14" priority="16">
+      <x:formula>$W$14&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="H5:H5">
+    <x:cfRule type="expression" dxfId="15" priority="17">
+      <x:formula>$W$15&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="B7:B7">
+    <x:cfRule type="expression" dxfId="16" priority="18">
+      <x:formula>$W$16&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C7:C7">
+    <x:cfRule type="expression" dxfId="17" priority="19">
+      <x:formula>$W$17&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="D7:D7">
+    <x:cfRule type="expression" dxfId="18" priority="20">
+      <x:formula>$W$18&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="E7:E7">
+    <x:cfRule type="expression" dxfId="19" priority="21">
+      <x:formula>$W$19&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="F7:F7">
+    <x:cfRule type="expression" dxfId="20" priority="22">
+      <x:formula>$W$20&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G7:G7">
+    <x:cfRule type="expression" dxfId="21" priority="23">
+      <x:formula>$W$21&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="H7:H7">
+    <x:cfRule type="expression" dxfId="22" priority="24">
+      <x:formula>$W$22&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="B9:B9">
+    <x:cfRule type="expression" dxfId="23" priority="25">
+      <x:formula>$W$23&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C9:C9">
+    <x:cfRule type="expression" dxfId="24" priority="26">
+      <x:formula>$W$24&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="D9:D9">
+    <x:cfRule type="expression" dxfId="25" priority="27">
+      <x:formula>$W$25&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="E9:E9">
+    <x:cfRule type="expression" dxfId="26" priority="28">
+      <x:formula>$W$26&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="F9:F9">
+    <x:cfRule type="expression" dxfId="27" priority="29">
+      <x:formula>$W$27&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G9:G9">
+    <x:cfRule type="expression" dxfId="28" priority="30">
+      <x:formula>$W$28&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="H9:H9">
+    <x:cfRule type="expression" dxfId="29" priority="31">
+      <x:formula>$W$29&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="B11:B11">
+    <x:cfRule type="expression" dxfId="30" priority="32">
+      <x:formula>$W$30&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C11:C11">
+    <x:cfRule type="expression" dxfId="31" priority="33">
+      <x:formula>$W$31&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="D11:D11">
+    <x:cfRule type="expression" dxfId="32" priority="34">
+      <x:formula>$W$32&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="E11:E11">
+    <x:cfRule type="expression" dxfId="33" priority="35">
+      <x:formula>$W$33&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="F11:F11">
+    <x:cfRule type="expression" dxfId="34" priority="36">
+      <x:formula>$W$34&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G11:G11">
+    <x:cfRule type="expression" dxfId="35" priority="37">
+      <x:formula>$W$35&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="H11:H11">
+    <x:cfRule type="expression" dxfId="36" priority="38">
+      <x:formula>$W$36&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="B13:B13">
+    <x:cfRule type="expression" dxfId="37" priority="39">
+      <x:formula>$W$37&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="C13:C13">
+    <x:cfRule type="expression" dxfId="38" priority="40">
+      <x:formula>$W$38&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="D13:D13">
+    <x:cfRule type="expression" dxfId="39" priority="41">
+      <x:formula>$W$39&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="E13:E13">
+    <x:cfRule type="expression" dxfId="40" priority="42">
+      <x:formula>$W$40&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="F13:F13">
+    <x:cfRule type="expression" dxfId="41" priority="43">
+      <x:formula>$W$41&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="G13:G13">
+    <x:cfRule type="expression" dxfId="42" priority="44">
+      <x:formula>$W$42&lt;&gt;""</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="H13:H13">
+    <x:cfRule type="expression" dxfId="43" priority="45">
+      <x:formula>$W$43&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
@@ -8448,7 +9229,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10b5e5e780824c58"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9aebcb94d6f4e44"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix repeated dates in older Excel
</commit_message>
<xml_diff>
--- a/app/template/캘린더(자동).xlsx
+++ b/app/template/캘린더(자동).xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="Rd522d779f81a4e80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="달력" sheetId="1" r:id="Rb1b539de605f4134"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공휴일" sheetId="2" r:id="R1fa1aa669f03435d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="달력" sheetId="1" r:id="R32fef00f85024245"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3847,31 +3847,31 @@
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="B3" s="47" t="str">
-        <x:f>IF($W$2&lt;&gt;"",$W$2&amp;REPT(" ",MAX(2,18-LEN($W$2)))&amp;DAY($V$2),REPT(" ",16-LEN(DAY($V$2)))&amp;DAY($V$2))</x:f>
+        <x:f>IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              26</x:v>
       </x:c>
       <x:c r="C3" s="48" t="str">
-        <x:f t="shared" ref="C3:H3" si="0">IF($W$3&lt;&gt;"",$W$3&amp;REPT(" ",MAX(2,18-LEN($W$3)))&amp;DAY($V$3),REPT(" ",16-LEN(DAY($V$3)))&amp;DAY($V$3))</x:f>
+        <x:f t="shared" ref="C3:H3" si="0">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              27</x:v>
       </x:c>
       <x:c r="D3" s="48" t="str">
-        <x:f t="shared" si="0">IF($W$4&lt;&gt;"",$W$4&amp;REPT(" ",MAX(2,18-LEN($W$4)))&amp;DAY($V$4),REPT(" ",16-LEN(DAY($V$4)))&amp;DAY($V$4))</x:f>
+        <x:f t="shared" si="0">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              28</x:v>
       </x:c>
       <x:c r="E3" s="48" t="str">
-        <x:f t="shared" si="0">IF($W$5&lt;&gt;"",$W$5&amp;REPT(" ",MAX(2,18-LEN($W$5)))&amp;DAY($V$5),REPT(" ",16-LEN(DAY($V$5)))&amp;DAY($V$5))</x:f>
+        <x:f t="shared" si="0">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              29</x:v>
       </x:c>
       <x:c r="F3" s="48" t="str">
-        <x:f t="shared" si="0">IF($W$6&lt;&gt;"",$W$6&amp;REPT(" ",MAX(2,18-LEN($W$6)))&amp;DAY($V$6),REPT(" ",16-LEN(DAY($V$6)))&amp;DAY($V$6))</x:f>
+        <x:f t="shared" si="0">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              30</x:v>
       </x:c>
       <x:c r="G3" s="48" t="str">
-        <x:f t="shared" si="0">IF($W$7&lt;&gt;"",$W$7&amp;REPT(" ",MAX(2,18-LEN($W$7)))&amp;DAY($V$7),REPT(" ",16-LEN(DAY($V$7)))&amp;DAY($V$7))</x:f>
+        <x:f t="shared" si="0">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              31</x:v>
       </x:c>
       <x:c r="H3" s="49" t="str">
-        <x:f t="shared" si="0">IF($W$8&lt;&gt;"",$W$8&amp;REPT(" ",MAX(2,18-LEN($W$8)))&amp;DAY($V$8),REPT(" ",16-LEN(DAY($V$8)))&amp;DAY($V$8))</x:f>
+        <x:f t="shared" si="0">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>               1</x:v>
       </x:c>
       <x:c r="I3" s="1"/>
@@ -3960,31 +3960,31 @@
     </x:row>
     <x:row r="5" ht="22" customHeight="1">
       <x:c r="B5" s="47" t="str">
-        <x:f>IF($W$9&lt;&gt;"",$W$9&amp;REPT(" ",MAX(2,18-LEN($W$9)))&amp;DAY($V$9),REPT(" ",16-LEN(DAY($V$9)))&amp;DAY($V$9))</x:f>
+        <x:f>IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>               2</x:v>
       </x:c>
       <x:c r="C5" s="48" t="str">
-        <x:f t="shared" ref="C5:H5" si="1">IF($W$10&lt;&gt;"",$W$10&amp;REPT(" ",MAX(2,18-LEN($W$10)))&amp;DAY($V$10),REPT(" ",16-LEN(DAY($V$10)))&amp;DAY($V$10))</x:f>
+        <x:f t="shared" ref="C5:H5" si="1">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>               3</x:v>
       </x:c>
       <x:c r="D5" s="48" t="str">
-        <x:f t="shared" si="1">IF($W$11&lt;&gt;"",$W$11&amp;REPT(" ",MAX(2,18-LEN($W$11)))&amp;DAY($V$11),REPT(" ",16-LEN(DAY($V$11)))&amp;DAY($V$11))</x:f>
+        <x:f t="shared" si="1">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>               4</x:v>
       </x:c>
       <x:c r="E5" s="48" t="str">
-        <x:f t="shared" si="1">IF($W$12&lt;&gt;"",$W$12&amp;REPT(" ",MAX(2,18-LEN($W$12)))&amp;DAY($V$12),REPT(" ",16-LEN(DAY($V$12)))&amp;DAY($V$12))</x:f>
+        <x:f t="shared" si="1">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>               5</x:v>
       </x:c>
       <x:c r="F5" s="48" t="str">
-        <x:f t="shared" si="1">IF($W$13&lt;&gt;"",$W$13&amp;REPT(" ",MAX(2,18-LEN($W$13)))&amp;DAY($V$13),REPT(" ",16-LEN(DAY($V$13)))&amp;DAY($V$13))</x:f>
+        <x:f t="shared" si="1">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>               6</x:v>
       </x:c>
       <x:c r="G5" s="48" t="str">
-        <x:f t="shared" si="1">IF($W$14&lt;&gt;"",$W$14&amp;REPT(" ",MAX(2,18-LEN($W$14)))&amp;DAY($V$14),REPT(" ",16-LEN(DAY($V$14)))&amp;DAY($V$14))</x:f>
+        <x:f t="shared" si="1">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>               7</x:v>
       </x:c>
       <x:c r="H5" s="49" t="str">
-        <x:f t="shared" si="1">IF($W$15&lt;&gt;"",$W$15&amp;REPT(" ",MAX(2,18-LEN($W$15)))&amp;DAY($V$15),REPT(" ",16-LEN(DAY($V$15)))&amp;DAY($V$15))</x:f>
+        <x:f t="shared" si="1">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>               8</x:v>
       </x:c>
       <x:c r="I5" s="1"/>
@@ -4071,31 +4071,31 @@
     </x:row>
     <x:row r="7" ht="22" customHeight="1">
       <x:c r="B7" s="47" t="str">
-        <x:f>IF($W$16&lt;&gt;"",$W$16&amp;REPT(" ",MAX(2,18-LEN($W$16)))&amp;DAY($V$16),REPT(" ",16-LEN(DAY($V$16)))&amp;DAY($V$16))</x:f>
+        <x:f>IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>               9</x:v>
       </x:c>
       <x:c r="C7" s="48" t="str">
-        <x:f t="shared" ref="C7:H7" si="2">IF($W$17&lt;&gt;"",$W$17&amp;REPT(" ",MAX(2,18-LEN($W$17)))&amp;DAY($V$17),REPT(" ",16-LEN(DAY($V$17)))&amp;DAY($V$17))</x:f>
+        <x:f t="shared" ref="C7:H7" si="2">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              10</x:v>
       </x:c>
       <x:c r="D7" s="48" t="str">
-        <x:f t="shared" si="2">IF($W$18&lt;&gt;"",$W$18&amp;REPT(" ",MAX(2,18-LEN($W$18)))&amp;DAY($V$18),REPT(" ",16-LEN(DAY($V$18)))&amp;DAY($V$18))</x:f>
+        <x:f t="shared" si="2">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              11</x:v>
       </x:c>
       <x:c r="E7" s="48" t="str">
-        <x:f t="shared" si="2">IF($W$19&lt;&gt;"",$W$19&amp;REPT(" ",MAX(2,18-LEN($W$19)))&amp;DAY($V$19),REPT(" ",16-LEN(DAY($V$19)))&amp;DAY($V$19))</x:f>
+        <x:f t="shared" si="2">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              12</x:v>
       </x:c>
       <x:c r="F7" s="48" t="str">
-        <x:f t="shared" si="2">IF($W$20&lt;&gt;"",$W$20&amp;REPT(" ",MAX(2,18-LEN($W$20)))&amp;DAY($V$20),REPT(" ",16-LEN(DAY($V$20)))&amp;DAY($V$20))</x:f>
+        <x:f t="shared" si="2">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              13</x:v>
       </x:c>
       <x:c r="G7" s="48" t="str">
-        <x:f t="shared" si="2">IF($W$21&lt;&gt;"",$W$21&amp;REPT(" ",MAX(2,18-LEN($W$21)))&amp;DAY($V$21),REPT(" ",16-LEN(DAY($V$21)))&amp;DAY($V$21))</x:f>
+        <x:f t="shared" si="2">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              14</x:v>
       </x:c>
       <x:c r="H7" s="49" t="str">
-        <x:f t="shared" si="2">IF($W$22&lt;&gt;"",$W$22&amp;REPT(" ",MAX(2,18-LEN($W$22)))&amp;DAY($V$22),REPT(" ",16-LEN(DAY($V$22)))&amp;DAY($V$22))</x:f>
+        <x:f t="shared" si="2">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>광복절               15</x:v>
       </x:c>
       <x:c r="I7" s="1"/>
@@ -4182,31 +4182,31 @@
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
       <x:c r="B9" s="47" t="str">
-        <x:f>IF($W$23&lt;&gt;"",$W$23&amp;REPT(" ",MAX(2,18-LEN($W$23)))&amp;DAY($V$23),REPT(" ",16-LEN(DAY($V$23)))&amp;DAY($V$23))</x:f>
+        <x:f>IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              16</x:v>
       </x:c>
       <x:c r="C9" s="48" t="str">
-        <x:f t="shared" ref="C9:H9" si="3">IF($W$24&lt;&gt;"",$W$24&amp;REPT(" ",MAX(2,18-LEN($W$24)))&amp;DAY($V$24),REPT(" ",16-LEN(DAY($V$24)))&amp;DAY($V$24))</x:f>
+        <x:f t="shared" ref="C9:H9" si="3">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>광복절 대체 휴일         17</x:v>
       </x:c>
       <x:c r="D9" s="48" t="str">
-        <x:f t="shared" si="3">IF($W$25&lt;&gt;"",$W$25&amp;REPT(" ",MAX(2,18-LEN($W$25)))&amp;DAY($V$25),REPT(" ",16-LEN(DAY($V$25)))&amp;DAY($V$25))</x:f>
+        <x:f t="shared" si="3">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              18</x:v>
       </x:c>
       <x:c r="E9" s="48" t="str">
-        <x:f t="shared" si="3">IF($W$26&lt;&gt;"",$W$26&amp;REPT(" ",MAX(2,18-LEN($W$26)))&amp;DAY($V$26),REPT(" ",16-LEN(DAY($V$26)))&amp;DAY($V$26))</x:f>
+        <x:f t="shared" si="3">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              19</x:v>
       </x:c>
       <x:c r="F9" s="48" t="str">
-        <x:f t="shared" si="3">IF($W$27&lt;&gt;"",$W$27&amp;REPT(" ",MAX(2,18-LEN($W$27)))&amp;DAY($V$27),REPT(" ",16-LEN(DAY($V$27)))&amp;DAY($V$27))</x:f>
+        <x:f t="shared" si="3">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              20</x:v>
       </x:c>
       <x:c r="G9" s="48" t="str">
-        <x:f t="shared" si="3">IF($W$28&lt;&gt;"",$W$28&amp;REPT(" ",MAX(2,18-LEN($W$28)))&amp;DAY($V$28),REPT(" ",16-LEN(DAY($V$28)))&amp;DAY($V$28))</x:f>
+        <x:f t="shared" si="3">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              21</x:v>
       </x:c>
       <x:c r="H9" s="49" t="str">
-        <x:f t="shared" si="3">IF($W$29&lt;&gt;"",$W$29&amp;REPT(" ",MAX(2,18-LEN($W$29)))&amp;DAY($V$29),REPT(" ",16-LEN(DAY($V$29)))&amp;DAY($V$29))</x:f>
+        <x:f t="shared" si="3">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              22</x:v>
       </x:c>
       <x:c r="I9" s="1"/>
@@ -4289,31 +4289,31 @@
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
       <x:c r="B11" s="47" t="str">
-        <x:f>IF($W$30&lt;&gt;"",$W$30&amp;REPT(" ",MAX(2,18-LEN($W$30)))&amp;DAY($V$30),REPT(" ",16-LEN(DAY($V$30)))&amp;DAY($V$30))</x:f>
+        <x:f>IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              23</x:v>
       </x:c>
       <x:c r="C11" s="48" t="str">
-        <x:f t="shared" ref="C11:H11" si="4">IF($W$31&lt;&gt;"",$W$31&amp;REPT(" ",MAX(2,18-LEN($W$31)))&amp;DAY($V$31),REPT(" ",16-LEN(DAY($V$31)))&amp;DAY($V$31))</x:f>
+        <x:f t="shared" ref="C11:H11" si="4">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              24</x:v>
       </x:c>
       <x:c r="D11" s="48" t="str">
-        <x:f t="shared" si="4">IF($W$32&lt;&gt;"",$W$32&amp;REPT(" ",MAX(2,18-LEN($W$32)))&amp;DAY($V$32),REPT(" ",16-LEN(DAY($V$32)))&amp;DAY($V$32))</x:f>
+        <x:f t="shared" si="4">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              25</x:v>
       </x:c>
       <x:c r="E11" s="48" t="str">
-        <x:f t="shared" si="4">IF($W$33&lt;&gt;"",$W$33&amp;REPT(" ",MAX(2,18-LEN($W$33)))&amp;DAY($V$33),REPT(" ",16-LEN(DAY($V$33)))&amp;DAY($V$33))</x:f>
+        <x:f t="shared" si="4">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              26</x:v>
       </x:c>
       <x:c r="F11" s="48" t="str">
-        <x:f t="shared" si="4">IF($W$34&lt;&gt;"",$W$34&amp;REPT(" ",MAX(2,18-LEN($W$34)))&amp;DAY($V$34),REPT(" ",16-LEN(DAY($V$34)))&amp;DAY($V$34))</x:f>
+        <x:f t="shared" si="4">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              27</x:v>
       </x:c>
       <x:c r="G11" s="48" t="str">
-        <x:f t="shared" si="4">IF($W$35&lt;&gt;"",$W$35&amp;REPT(" ",MAX(2,18-LEN($W$35)))&amp;DAY($V$35),REPT(" ",16-LEN(DAY($V$35)))&amp;DAY($V$35))</x:f>
+        <x:f t="shared" si="4">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              28</x:v>
       </x:c>
       <x:c r="H11" s="49" t="str">
-        <x:f t="shared" si="4">IF($W$36&lt;&gt;"",$W$36&amp;REPT(" ",MAX(2,18-LEN($W$36)))&amp;DAY($V$36),REPT(" ",16-LEN(DAY($V$36)))&amp;DAY($V$36))</x:f>
+        <x:f t="shared" si="4">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              29</x:v>
       </x:c>
       <x:c r="I11" s="1"/>
@@ -4396,31 +4396,31 @@
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
       <x:c r="B13" s="47" t="str">
-        <x:f>IF($W$37&lt;&gt;"",$W$37&amp;REPT(" ",MAX(2,18-LEN($W$37)))&amp;DAY($V$37),REPT(" ",16-LEN(DAY($V$37)))&amp;DAY($V$37))</x:f>
+        <x:f>IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              30</x:v>
       </x:c>
       <x:c r="C13" s="48" t="str">
-        <x:f t="shared" ref="C13:H13" si="5">IF($W$38&lt;&gt;"",$W$38&amp;REPT(" ",MAX(2,18-LEN($W$38)))&amp;DAY($V$38),REPT(" ",16-LEN(DAY($V$38)))&amp;DAY($V$38))</x:f>
+        <x:f t="shared" ref="C13:H13" si="5">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>              31</x:v>
       </x:c>
       <x:c r="D13" s="48" t="str">
-        <x:f t="shared" si="5">IF($W$39&lt;&gt;"",$W$39&amp;REPT(" ",MAX(2,18-LEN($W$39)))&amp;DAY($V$39),REPT(" ",16-LEN(DAY($V$39)))&amp;DAY($V$39))</x:f>
+        <x:f t="shared" si="5">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>               1</x:v>
       </x:c>
       <x:c r="E13" s="48" t="str">
-        <x:f t="shared" si="5">IF($W$40&lt;&gt;"",$W$40&amp;REPT(" ",MAX(2,18-LEN($W$40)))&amp;DAY($V$40),REPT(" ",16-LEN(DAY($V$40)))&amp;DAY($V$40))</x:f>
+        <x:f t="shared" si="5">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>               2</x:v>
       </x:c>
       <x:c r="F13" s="48" t="str">
-        <x:f t="shared" si="5">IF($W$41&lt;&gt;"",$W$41&amp;REPT(" ",MAX(2,18-LEN($W$41)))&amp;DAY($V$41),REPT(" ",16-LEN(DAY($V$41)))&amp;DAY($V$41))</x:f>
+        <x:f t="shared" si="5">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>               3</x:v>
       </x:c>
       <x:c r="G13" s="48" t="str">
-        <x:f t="shared" si="5">IF($W$42&lt;&gt;"",$W$42&amp;REPT(" ",MAX(2,18-LEN($W$42)))&amp;DAY($V$42),REPT(" ",16-LEN(DAY($V$42)))&amp;DAY($V$42))</x:f>
+        <x:f t="shared" si="5">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>               4</x:v>
       </x:c>
       <x:c r="H13" s="49" t="str">
-        <x:f t="shared" si="5">IF($W$43&lt;&gt;"",$W$43&amp;REPT(" ",MAX(2,18-LEN($W$43)))&amp;DAY($V$43),REPT(" ",16-LEN(DAY($V$43)))&amp;DAY($V$43))</x:f>
+        <x:f t="shared" si="5">IF(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;"",INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&amp;REPT(" ",MAX(2,18-LEN(INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)),REPT(" ",16-LEN(DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1))))&amp;DAY(INDEX($V$2:$V$43,(ROW()-3)/2*7+COLUMN()-1)))</x:f>
         <x:v>               5</x:v>
       </x:c>
       <x:c r="I13" s="1"/>
@@ -9011,212 +9011,212 @@
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="B3:B3">
     <x:cfRule type="expression" dxfId="2" priority="4">
-      <x:formula>$W$2&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="C3:C3">
     <x:cfRule type="expression" dxfId="3" priority="5">
-      <x:formula>$W$3&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="D3:D3">
     <x:cfRule type="expression" dxfId="4" priority="6">
-      <x:formula>$W$4&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="E3:E3">
     <x:cfRule type="expression" dxfId="5" priority="7">
-      <x:formula>$W$5&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="F3:F3">
     <x:cfRule type="expression" dxfId="6" priority="8">
-      <x:formula>$W$6&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="G3:G3">
     <x:cfRule type="expression" dxfId="7" priority="9">
-      <x:formula>$W$7&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="H3:H3">
     <x:cfRule type="expression" dxfId="8" priority="10">
-      <x:formula>$W$8&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="B5:B5">
     <x:cfRule type="expression" dxfId="9" priority="11">
-      <x:formula>$W$9&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="C5:C5">
     <x:cfRule type="expression" dxfId="10" priority="12">
-      <x:formula>$W$10&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="D5:D5">
     <x:cfRule type="expression" dxfId="11" priority="13">
-      <x:formula>$W$11&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="E5:E5">
     <x:cfRule type="expression" dxfId="12" priority="14">
-      <x:formula>$W$12&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="F5:F5">
     <x:cfRule type="expression" dxfId="13" priority="15">
-      <x:formula>$W$13&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="G5:G5">
     <x:cfRule type="expression" dxfId="14" priority="16">
-      <x:formula>$W$14&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="H5:H5">
     <x:cfRule type="expression" dxfId="15" priority="17">
-      <x:formula>$W$15&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="B7:B7">
     <x:cfRule type="expression" dxfId="16" priority="18">
-      <x:formula>$W$16&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="C7:C7">
     <x:cfRule type="expression" dxfId="17" priority="19">
-      <x:formula>$W$17&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="D7:D7">
     <x:cfRule type="expression" dxfId="18" priority="20">
-      <x:formula>$W$18&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="E7:E7">
     <x:cfRule type="expression" dxfId="19" priority="21">
-      <x:formula>$W$19&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="F7:F7">
     <x:cfRule type="expression" dxfId="20" priority="22">
-      <x:formula>$W$20&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="G7:G7">
     <x:cfRule type="expression" dxfId="21" priority="23">
-      <x:formula>$W$21&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="H7:H7">
     <x:cfRule type="expression" dxfId="22" priority="24">
-      <x:formula>$W$22&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="B9:B9">
     <x:cfRule type="expression" dxfId="23" priority="25">
-      <x:formula>$W$23&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="C9:C9">
     <x:cfRule type="expression" dxfId="24" priority="26">
-      <x:formula>$W$24&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="D9:D9">
     <x:cfRule type="expression" dxfId="25" priority="27">
-      <x:formula>$W$25&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="E9:E9">
     <x:cfRule type="expression" dxfId="26" priority="28">
-      <x:formula>$W$26&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="F9:F9">
     <x:cfRule type="expression" dxfId="27" priority="29">
-      <x:formula>$W$27&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="G9:G9">
     <x:cfRule type="expression" dxfId="28" priority="30">
-      <x:formula>$W$28&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="H9:H9">
     <x:cfRule type="expression" dxfId="29" priority="31">
-      <x:formula>$W$29&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="B11:B11">
     <x:cfRule type="expression" dxfId="30" priority="32">
-      <x:formula>$W$30&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="C11:C11">
     <x:cfRule type="expression" dxfId="31" priority="33">
-      <x:formula>$W$31&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="D11:D11">
     <x:cfRule type="expression" dxfId="32" priority="34">
-      <x:formula>$W$32&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="E11:E11">
     <x:cfRule type="expression" dxfId="33" priority="35">
-      <x:formula>$W$33&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="F11:F11">
     <x:cfRule type="expression" dxfId="34" priority="36">
-      <x:formula>$W$34&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="G11:G11">
     <x:cfRule type="expression" dxfId="35" priority="37">
-      <x:formula>$W$35&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="H11:H11">
     <x:cfRule type="expression" dxfId="36" priority="38">
-      <x:formula>$W$36&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="B13:B13">
     <x:cfRule type="expression" dxfId="37" priority="39">
-      <x:formula>$W$37&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="C13:C13">
     <x:cfRule type="expression" dxfId="38" priority="40">
-      <x:formula>$W$38&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="D13:D13">
     <x:cfRule type="expression" dxfId="39" priority="41">
-      <x:formula>$W$39&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="E13:E13">
     <x:cfRule type="expression" dxfId="40" priority="42">
-      <x:formula>$W$40&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="F13:F13">
     <x:cfRule type="expression" dxfId="41" priority="43">
-      <x:formula>$W$41&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="G13:G13">
     <x:cfRule type="expression" dxfId="42" priority="44">
-      <x:formula>$W$42&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="H13:H13">
     <x:cfRule type="expression" dxfId="43" priority="45">
-      <x:formula>$W$43&lt;&gt;""</x:formula>
+      <x:formula>INDEX($W$2:$W$43,(ROW()-3)/2*7+COLUMN()-1)&lt;&gt;""</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:dataValidations count="2">
@@ -9229,7 +9229,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f31163ba21d4fce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d5a24897e864535"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>